<commit_message>
rag: changed ingest method for new cases
</commit_message>
<xml_diff>
--- a/data/Goldstandard_anonymisiert.xlsx
+++ b/data/Goldstandard_anonymisiert.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>[{"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}]</t>
+          <t>[{"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "110", "text": "Zugsteuerung erkennt das zweite Drehgestell nicht. Fehlerhafter Crimp am Stecker X75 unterflur. Leitungen haben Wackelkontakt. Montage-Team muss Crimpung erneuern.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Fehlerhafter Crimp am Stecker X75 unterflur. [...] Montage-Team muss Crimpung erneuern."}, "cot_begruendung": "Ein fehlerhafter Crimp durch das Montage-Team führt zu einem Wackelkontakt, was einen Ausführungsfehler (Montage) im Werk darstellt. Da die Zugsteuerung das Drehgestell nicht erkennt, ist keine Fahrtübersicht gegeben, was eine Inbetriebnahme blockiert (Blocker)."}, {"fall_id": "193", "text": "Palette mit den Seitenscheiben für Wagen 6 war 2 Tage verschwunden. Ein Staplerfahrer hat sie im falschen Hallenschiff bei den Rohbauteilen abgestellt statt an der Linie. Verzögerung im Fensterbau.", "zielvariablen": {"ursache": "Logistik", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Ein Staplerfahrer hat sie im falschen Hallenschiff bei den Rohbauteilen abgestellt statt an der Linie."}, "cot_begruendung": "Das Abstellen einer Palette am falschen Ort durch internes Logistik-Personal ist ein intralogistischer Fehler (Logistik/Logistik). Da die Teile gefunden wurden und verbaut werden können, handelt es sich um eine zeitliche Nacharbeit."}]</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>[{"fall_id": "79", "text": "Sitzbezüge im gesamten Wagen reißen an der Naht ein. Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge müssen getauscht werden.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge"}, "cot_begruendung": "Die mangelhafte Stoffqualität eines externen Lieferanten ist ein Materialfehler. Die Bemerkungen 'gesamter Wagen' und 'neuen Serie' verweisen auf einen Serienfehler. Das Austauschen der Bezüge ist Nacharbeit, aber kein Blocker für Inbetriebsetzungen."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}]</t>
+          <t>[{"fall_id": "148", "text": "Sitzgestell wackelt.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Sitzgestell wackelt."}, "cot_begruendung": "Nur das Symptom 'wackelt' ist gegeben. Ob der Werker Schrauben vergessen hat, die Bohrungen falsch gesetzt sind oder das Gestell vom Lieferanten verzogen ist, ist nicht ersichtlich. Causal Faithfulness verlangt hier die Abstention (Unbekannt)."}, {"fall_id": "79", "text": "Sitzbezüge im gesamten Wagen reißen an der Naht ein. Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge müssen getauscht werden.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge"}, "cot_begruendung": "Die mangelhafte Stoffqualität eines externen Lieferanten ist ein Materialfehler. Die Bemerkungen 'gesamter Wagen' und 'neuen Serie' verweisen auf einen Serienfehler. Das Austauschen der Bezüge ist Nacharbeit, aber kein Blocker für Inbetriebsetzungen."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>[{"fall_id": "100", "text": "Schraube M8x20 an Haltestange im FGR WE2 rundgedreht. Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden."}, "cot_begruendung": "Das Runddrehen einer Schraube durch Nutzung eines falschen Bits durch den Werker ist ein Montagefehler im Werk. Das Ausbohren der defekten Schraube ist zeitintensiv, aber eine klassische Nacharbeit, die den Fertigungsablauf nicht komplett stoppt."}, {"fall_id": "14", "text": "Notbremsschleife falsch gepinnt an Stecker X12 im Fahrerpult. Pin 3 und Pin 5 vertauscht, Funktion nicht gegeben. Fehler bei Verkabelung durch Schicht 2.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Fehler bei Verkabelung durch Schicht 2"}, "cot_begruendung": "Die falsch gepinnte Notbremsschleife wurde explizit durch eine interne Schicht ('Verkabelung durch Schicht 2') verursacht, was Montage/Werk als Ursprung festlegt. Da die Notbremse eine sicherheitskritische Funktion ist und nicht funktioniert, handelt es sich um einen Blocker."}, {"fall_id": "4", "text": "Erdungsband am Triebdrehgestell WE1 links vergessen anzuschrauben. Schraube liegt lose auf dem Rahmen.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "vergessen anzuschrauben"}, "cot_begruendung": "Das vergessene Anschrauben ('Schraube liegt lose auf dem Rahmen') ist ein eindeutiger Montage- und Ausführungsfehler im Werk. Da eine fehlende Erdung am Triebdrehgestell ein massives Sicherheitsrisiko darstellt und die Inbetriebnahme verhindert, ist dies ein Blocker."}]</t>
+          <t>[{"fall_id": "100", "text": "Schraube M8x20 an Haltestange im FGR WE2 rundgedreht. Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden."}, "cot_begruendung": "Das Runddrehen einer Schraube durch Nutzung eines falschen Bits durch den Werker ist ein Montagefehler im Werk. Das Ausbohren der defekten Schraube ist zeitintensiv, aber eine klassische Nacharbeit, die den Fertigungsablauf nicht komplett stoppt."}, {"fall_id": "14", "text": "Notbremsschleife falsch gepinnt an Stecker X12 im Fahrerpult. Pin 3 und Pin 5 vertauscht, Funktion nicht gegeben. Fehler bei Verkabelung durch Schicht 2.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Fehler bei Verkabelung durch Schicht 2"}, "cot_begruendung": "Die falsch gepinnte Notbremsschleife wurde explizit durch eine interne Schicht ('Verkabelung durch Schicht 2') verursacht, was Montage/Werk als Ursprung festlegt. Da die Notbremse eine sicherheitskritische Funktion ist und nicht funktioniert, handelt es sich um einen Blocker."}, {"fall_id": "4", "text": "Erdungsband am Triebdrehgestell WE1 links vergessen anzuschrauben. Schraube liegt lose auf dem Rahmen.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "vergessen anzuschrauben"}, "cot_begruendung": "Das vergessene Anschrauben ('Schraube liegt lose auf dem Rahmen') ist ein eindeutiger Montage- und Ausführungsfehler im Werk. Da eine fehlende Erdung am Triebdrehgestell ein massives Sicherheitsrisiko darstellt und die Inbetriebnahme verhindert, ist dies ein Blocker."}]</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>[{"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
+          <t>[{"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}, {"fall_id": "162", "text": "Graue Flecken auf dem neuen Fußbodenbelag im FGR. Reinigungskraft hat den Spezialreiniger nicht richtig verdünnt, wodurch Rückstände beim Trocknen entstanden sind. Einmal feucht nachwischen behebt das Problem.", "zielvariablen": {"ursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Reinigungskraft hat den Spezialreiniger nicht richtig verdünnt"}, "cot_begruendung": "Falsche Dosierung des Reinigungsmittels durch die Reinigungskraft ist ein klassischer Fehler der internen Reinigung (Werk). Da sich der Mangel durch simples Nachwischen beheben lässt, wird er als 'Info' oder sehr leichte Nacharbeit deklariert."}]</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>[{"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}, {"fall_id": "65", "text": "Tür geht nicht.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Tür geht nicht."}, "cot_begruendung": "Der Text 'Tür geht nicht' ist maximal unspezifisch. Es fehlen jegliche Hinweise auf mechanische, elektrische, softwareseitige oder prozessuale Ursachen. Gemäß Abstention-Vorgabe muss Unbekannt ausgegeben werden."}]</t>
+          <t>[{"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}, {"fall_id": "101", "text": "Klemmschutz an Fahrgasttür 3 LWS löst viel zu früh aus. Schließvorgang bricht bei leichtem Windstoß ab. Sensorik-Parameter in der neuen Türsoftware (V1.4) von Fa. [Platzhalter] sind zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte angefordert.", "zielvariablen": {"ursache": "Software", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Sensorik-Parameter in der neuen Türsoftware [...] zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte"}, "cot_begruendung": "Der Text beschreibt ein funktionales Problem der Fahrgasttür aufgrund zu empfindlicher Parameter in der 'neuen Türsoftware', welche von einem externen Lieferanten stammt. Da die 'gesamte Flotte' ein Update benötigt, handelt es sich um einen Serienfehler. Ein fehlerhafter Klemmschutz betrifft die Sicherheit und Zuverlässigkeit der Türen, was die Inbetriebnahme blockiert."}]</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>[{"fall_id": "20", "text": "Typenschild für Klimakompressor im SAP mit falscher Seriennummer hinterlegt. Scan am Arbeitsplatz schlägt fehl.", "zielvariablen": {"grundursache": "Software", "ursprung": "Logistik", "kritikalitaet": "Info", "serie": false, "text_snippet": "im SAP mit falscher Seriennummer hinterlegt"}, "cot_begruendung": "Ein Datenfehler in der SAP-Datenbank ist eine logistische oder softwareseitige Grundursache. Da das Bauteil physisch in Ordnung ist und nur im System korrigiert werden muss, ist dies kein Fertigungsblocker, sondern eine 'Info' für das Datenmanagement."}, {"fall_id": "37", "text": "Kaffeemaschine im Zugbegleiterabteil mit großer Delle angeliefert. Karton außen war komplett intakt, also vermutlich schon beim Lieferanten vor Verpackung passiert.", "zielvariablen": {"grundursache": "Handhabung", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Karton außen war komplett intakt, also vermutlich schon beim Lieferanten vor Verpackung passiert."}, "cot_begruendung": "Die Logik des QA-Mitarbeiters folgert aus dem intakten Karton, dass der Schaden (Handhabung) bereits 'beim Lieferanten vor Verpackung' entstanden ist. Eine verbeulte Kaffeemaschine bedingt einen Austausch (Nacharbeit), stoppt aber die Fahrzeugfertigung nicht."}, {"fall_id": "5", "text": "Monitore FGR zeigen falsche Haltestellen an. Softwarestand V2.1 fehlerhaft. Update auf V2.2 durch Fa. [Platzhalter] für den gesamten Zug 15 nötig.", "zielvariablen": {"grundursache": "Software", "ursprung": "Lieferant", "kritikalitaet": "Info", "serie": true, "text_snippet": "Softwarestand V2.1 fehlerhaft [...] für den gesamten Zug 15 nötig"}, "cot_begruendung": "Der Text benennt explizit einen 'Softwarestand V2.1 fehlerhaft', der von einer externen Firma (Lieferant) behoben werden muss. Der Vermerk 'gesamten Zug 15' klassifiziert den Fehler als Serie. Ein Software-Update bei Monitoren hindert den Zugbau nicht physisch, daher als 'Info' oder leichte Nacharbeit eingestuft."}]</t>
+          <t>[{"fall_id": "20", "text": "Typenschild für Klimakompressor im SAP mit falscher Seriennummer hinterlegt. Scan am Arbeitsplatz schlägt fehl.", "zielvariablen": {"ursache": "Software", "ursprung": "Logistik", "kritikalitaet": "Info", "serie": false, "text_snippet": "im SAP mit falscher Seriennummer hinterlegt"}, "cot_begruendung": "Ein Datenfehler in der SAP-Datenbank ist eine logistische oder softwareseitige Grundursache. Da das Bauteil physisch in Ordnung ist und nur im System korrigiert werden muss, ist dies kein Fertigungsblocker, sondern eine 'Info' für das Datenmanagement."}, {"fall_id": "37", "text": "Kaffeemaschine im Zugbegleiterabteil mit großer Delle angeliefert. Karton außen war komplett intakt, also vermutlich schon beim Lieferanten vor Verpackung passiert.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Karton außen war komplett intakt, also vermutlich schon beim Lieferanten vor Verpackung passiert."}, "cot_begruendung": "Die Logik des QA-Mitarbeiters folgert aus dem intakten Karton, dass der Schaden (Handhabung) bereits 'beim Lieferanten vor Verpackung' entstanden ist. Eine verbeulte Kaffeemaschine bedingt einen Austausch (Nacharbeit), stoppt aber die Fahrzeugfertigung nicht."}, {"fall_id": "5", "text": "Monitore FGR zeigen falsche Haltestellen an. Softwarestand V2.1 fehlerhaft. Update auf V2.2 durch Fa. [Platzhalter] für den gesamten Zug 15 nötig.", "zielvariablen": {"ursache": "Software", "ursprung": "Lieferant", "kritikalitaet": "Info", "serie": true, "text_snippet": "Softwarestand V2.1 fehlerhaft [...] für den gesamten Zug 15 nötig"}, "cot_begruendung": "Der Text benennt explizit einen 'Softwarestand V2.1 fehlerhaft', der von einer externen Firma (Lieferant) behoben werden muss. Der Vermerk 'gesamten Zug 15' klassifiziert den Fehler als Serie. Ein Software-Update bei Monitoren hindert den Zugbau nicht physisch, daher als 'Info' oder leichte Nacharbeit eingestuft."}]</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>[{"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "76", "text": "Türen LWS öffnen sich, wenn Taster für RWS gedrückt wird. Software-Mapping in der DCU vom Engineering komplett vertauscht. Gefahr für Leib und Leben, IBS abgebrochen.", "zielvariablen": {"grundursache": "Software", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Software-Mapping in der DCU vom Engineering komplett vertauscht. Gefahr für Leib und Leben, IBS abgebrochen."}, "cot_begruendung": "Vertauschtes Software-Mapping durch das Engineering ist ein Software/Konstruktions-Fehler. Ein sicherheitskritisches Türproblem mit Abbruch der IBS ist der Inbegriff eines harten Blockers."}]</t>
+          <t>[{"fall_id": "101", "text": "Klemmschutz an Fahrgasttür 3 LWS löst viel zu früh aus. Schließvorgang bricht bei leichtem Windstoß ab. Sensorik-Parameter in der neuen Türsoftware (V1.4) von Fa. [Platzhalter] sind zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte angefordert.", "zielvariablen": {"ursache": "Software", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Sensorik-Parameter in der neuen Türsoftware [...] zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte"}, "cot_begruendung": "Der Text beschreibt ein funktionales Problem der Fahrgasttür aufgrund zu empfindlicher Parameter in der 'neuen Türsoftware', welche von einem externen Lieferanten stammt. Da die 'gesamte Flotte' ein Update benötigt, handelt es sich um einen Serienfehler. Ein fehlerhafter Klemmschutz betrifft die Sicherheit und Zuverlässigkeit der Türen, was die Inbetriebnahme blockiert."}, {"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}]</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>[{"fall_id": "40", "text": "PMA-Schlauch am Unterflur WE1 links kollidiert leicht mit der Achse. Kabelbinder wurde vom Werker zu locker gezogen.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Kabelbinder wurde vom Werker zu locker gezogen."}, "cot_begruendung": "Ein zu locker gezogener Kabelbinder durch den Werker ist ein klassischer Montagefehler im Werk. Die leichte Kollision des Schlauchs muss durch Setzen eines neuen Kabelbinders nachgearbeitet werden, hält die Produktion aber nicht an."}, {"fall_id": "87", "text": "Riss in der Bremsscheibe WE2 Achse 1. Metallurgische Prüfung zeigt Lunker im Guss. Alle Scheiben der Charge von Fa. [Platzhalter] betroffen. Keine Streckenfreigabe.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Lunker im Guss. Alle Scheiben der Charge von Fa. [Platzhalter] betroffen. Keine Streckenfreigabe."}, "cot_begruendung": "Lunker im Guss bei Lieferung durch eine externe Firma sind ein massiver Materialfehler des Lieferanten. Das Wort 'Charge' kennzeichnet es als Serienfehler. Da sicherheitsrelevante Bremsen betroffen sind und die Streckenfreigabe verweigert wird, ist dies ein absoluter Blocker."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}]</t>
+          <t>[{"fall_id": "40", "text": "PMA-Schlauch am Unterflur WE1 links kollidiert leicht mit der Achse. Kabelbinder wurde vom Werker zu locker gezogen.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Kabelbinder wurde vom Werker zu locker gezogen."}, "cot_begruendung": "Ein zu locker gezogener Kabelbinder durch den Werker ist ein klassischer Montagefehler im Werk. Die leichte Kollision des Schlauchs muss durch Setzen eines neuen Kabelbinders nachgearbeitet werden, hält die Produktion aber nicht an."}, {"fall_id": "104", "text": "Wischwasserbehälter WE1 undicht. Schweißnaht am Kunststoffgehäuse hat Haarrisse. Offenbar Produktionsfehler vom Hersteller. Tropft auf die darunterliegende Elektrik. Sofortiger Tausch nötig.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Schweißnaht am Kunststoffgehäuse hat Haarrisse. Offenbar Produktionsfehler vom Hersteller."}, "cot_begruendung": "Ein undichter Behälter aufgrund von Haarrissen in der Schweißnaht ab Werk ist ein Materialfehler, der vom Hersteller (Lieferant) verursacht wurde. Da das Wasser auf die Elektrik tropft und ein sofortiger Tausch gefordert wird, liegt eine hohe Kritikalität (Blocker) vor."}, {"fall_id": "87", "text": "Riss in der Bremsscheibe WE2 Achse 1. Metallurgische Prüfung zeigt Lunker im Guss. Alle Scheiben der Charge von Fa. [Platzhalter] betroffen. Keine Streckenfreigabe.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Lunker im Guss. Alle Scheiben der Charge von Fa. [Platzhalter] betroffen. Keine Streckenfreigabe."}, "cot_begruendung": "Lunker im Guss bei Lieferung durch eine externe Firma sind ein massiver Materialfehler des Lieferanten. Das Wort 'Charge' kennzeichnet es als Serienfehler. Da sicherheitsrelevante Bremsen betroffen sind und die Streckenfreigabe verweigert wird, ist dies ein absoluter Blocker."}]</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>[{"fall_id": "22", "text": "Fahrgasttür RWS öffnet nicht bei Tasterbetätigung. DCU gibt keinen Befehl raus. Ersatzteil aus Lager geholt, Tür funktioniert wieder. Defekte DCU geht an Lieferant retour.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "DCU gibt keinen Befehl raus. [...] Defekte DCU geht an Lieferant retour"}, "cot_begruendung": "Die Door Control Unit (DCU) ist intern defekt, was auf einen Materialfehler des Lieferanten schließen lässt. Da das Ersatzteil sofort aus dem Lager verfügbar war und die Produktion nicht gestoppt wurde, bleibt es bei einer Nacharbeit."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}, {"fall_id": "67", "text": "Versteifungsrippe RWS im Unterflur nicht verschweißt, nur geheftet. Schweißer hat die finale Naht komplett vergessen. Fahrzeug darf so nicht aufgebockt werden.", "zielvariablen": {"grundursache": "Fertigung", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Schweißer hat die finale Naht komplett vergessen. Fahrzeug darf so nicht aufgebockt werden."}, "cot_begruendung": "Das Vergessen der finalen Schweißnaht durch den Schweißer ist ein schwerer Fertigungsfehler im Rohbau (Werk). Da die Statik gefährdet ist ('Fahrzeug darf so nicht aufgebockt werden'), liegt ein kritischer Blocker vor."}]</t>
+          <t>[{"fall_id": "175", "text": "Schwarze Abdeckkappe an der Haltestange RWS beim Einstieg vergessen. Werker hat die Beilagen-Kiste beim Aufräumen übersehen.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat die Beilagen-Kiste beim Aufräumen übersehen."}, "cot_begruendung": "Das Übersehen von Bauteilen durch den Werker ist ein klassischer Montagefehler im Werk. Das Aufklipsen der Abdeckkappe ist in wenigen Sekunden erledigt (Nacharbeit)."}, {"fall_id": "22", "text": "Fahrgasttür RWS öffnet nicht bei Tasterbetätigung. DCU gibt keinen Befehl raus. Ersatzteil aus Lager geholt, Tür funktioniert wieder. Defekte DCU geht an Lieferant retour.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "DCU gibt keinen Befehl raus. [...] Defekte DCU geht an Lieferant retour"}, "cot_begruendung": "Die Door Control Unit (DCU) ist intern defekt, was auf einen Materialfehler des Lieferanten schließen lässt. Da das Ersatzteil sofort aus dem Lager verfügbar war und die Produktion nicht gestoppt wurde, bleibt es bei einer Nacharbeit."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}]</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>[{"fall_id": "58", "text": "Lack zerkratzt.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Lack zerkratzt."}, "cot_begruendung": "Der Text beschreibt lediglich das Symptom 'Lack zerkratzt', liefert jedoch keinen Kontext zur Entstehung (z. B. Transport, unachtsamer Werker, Reinigung). Zur Vermeidung von Halluzinationen muss die Abstention-Logik angewandt und 'Unbekannt' ausgegeben werden."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "67", "text": "Versteifungsrippe RWS im Unterflur nicht verschweißt, nur geheftet. Schweißer hat die finale Naht komplett vergessen. Fahrzeug darf so nicht aufgebockt werden.", "zielvariablen": {"grundursache": "Fertigung", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Schweißer hat die finale Naht komplett vergessen. Fahrzeug darf so nicht aufgebockt werden."}, "cot_begruendung": "Das Vergessen der finalen Schweißnaht durch den Schweißer ist ein schwerer Fertigungsfehler im Rohbau (Werk). Da die Statik gefährdet ist ('Fahrzeug darf so nicht aufgebockt werden'), liegt ein kritischer Blocker vor."}]</t>
+          <t>[{"fall_id": "58", "text": "Lack zerkratzt.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Lack zerkratzt."}, "cot_begruendung": "Der Text beschreibt lediglich das Symptom 'Lack zerkratzt', liefert jedoch keinen Kontext zur Entstehung (z. B. Transport, unachtsamer Werker, Reinigung). Zur Vermeidung von Halluzinationen muss die Abstention-Logik angewandt und 'Unbekannt' ausgegeben werden."}, {"fall_id": "152", "text": "Abdeckbleche für die Heizkanäle LWS aus unserer eigenen Stanzerei sind an der Kante um 10 Grad zu wenig abgekantet. Betrifft alle 40 Bleche von heute. Können so nicht montiert werden, Kante steht ab.", "zielvariablen": {"ursache": "Fertigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "aus unserer eigenen Stanzerei sind an der Kante um 10 Grad zu wenig abgekantet. Betrifft alle 40 Bleche"}, "cot_begruendung": "Ein Biegefehler aus der 'eigenen Stanzerei' ist ein interner Fertigungsfehler (Werk). Da 'alle 40 Bleche von heute' betroffen sind, liegt ein Serienfehler vor. Die Bleche müssen nachgebogen werden (Nacharbeit), stoppen aber nicht den kompletten Wagenausbau."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}]</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>[{"fall_id": "67", "text": "Versteifungsrippe RWS im Unterflur nicht verschweißt, nur geheftet. Schweißer hat die finale Naht komplett vergessen. Fahrzeug darf so nicht aufgebockt werden.", "zielvariablen": {"grundursache": "Fertigung", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Schweißer hat die finale Naht komplett vergessen. Fahrzeug darf so nicht aufgebockt werden."}, "cot_begruendung": "Das Vergessen der finalen Schweißnaht durch den Schweißer ist ein schwerer Fertigungsfehler im Rohbau (Werk). Da die Statik gefährdet ist ('Fahrzeug darf so nicht aufgebockt werden'), liegt ein kritischer Blocker vor."}, {"fall_id": "1", "text": "Wasser tropft aus Klimaanlage im FGR bei Wagenübergang WE2. Ablaufschlauch hat Riss ab Werk. Tausch erforderlich.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Ablaufschlauch hat Riss ab Werk"}, "cot_begruendung": "Der Text beschreibt eine Undichtigkeit aufgrund eines gerissenen Ablaufschlauchs 'ab Werk'. Da das Teil bereits defekt angeliefert wurde, ist die Ursache ein Materialfehler und der Ursprung der Lieferant. Eine undichte Klimaanlage über dem Fahrgastraum verhindert den Fahrzeugeinsatz, daher Kritikalität Blocker. Keine Hinweise auf eine Wiederholung."}, {"fall_id": "81", "text": "Druckluftrohr kollidiert mit dem Drehgestellrahmen WE1 beim Ausdrehen in Kurven. Routing der Rohre im 3D-Modell berücksichtigt den Ausdrehwinkel nicht. Engineering muss Routing sofort ändern, keine Freigabe für Dynamik-Tests.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Routing der Rohre im 3D-Modell berücksichtigt den Ausdrehwinkel nicht. Engineering muss Routing sofort ändern, keine Freigabe für Dynamik-Tests."}, "cot_begruendung": "Ein fehlender Ausdrehwinkel im 3D-Modell ist ein Konstruktionsfehler des Engineerings. Da keine Freigabe für Tests erteilt wird ('keine Freigabe für Dynamik-Tests'), liegt ein Blocker vor."}]</t>
+          <t>[{"fall_id": "104", "text": "Wischwasserbehälter WE1 undicht. Schweißnaht am Kunststoffgehäuse hat Haarrisse. Offenbar Produktionsfehler vom Hersteller. Tropft auf die darunterliegende Elektrik. Sofortiger Tausch nötig.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Schweißnaht am Kunststoffgehäuse hat Haarrisse. Offenbar Produktionsfehler vom Hersteller."}, "cot_begruendung": "Ein undichter Behälter aufgrund von Haarrissen in der Schweißnaht ab Werk ist ein Materialfehler, der vom Hersteller (Lieferant) verursacht wurde. Da das Wasser auf die Elektrik tropft und ein sofortiger Tausch gefordert wird, liegt eine hohe Kritikalität (Blocker) vor."}, {"fall_id": "110", "text": "Zugsteuerung erkennt das zweite Drehgestell nicht. Fehlerhafter Crimp am Stecker X75 unterflur. Leitungen haben Wackelkontakt. Montage-Team muss Crimpung erneuern.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Fehlerhafter Crimp am Stecker X75 unterflur. [...] Montage-Team muss Crimpung erneuern."}, "cot_begruendung": "Ein fehlerhafter Crimp durch das Montage-Team führt zu einem Wackelkontakt, was einen Ausführungsfehler (Montage) im Werk darstellt. Da die Zugsteuerung das Drehgestell nicht erkennt, ist keine Fahrtübersicht gegeben, was eine Inbetriebnahme blockiert (Blocker)."}, {"fall_id": "141", "text": "Erdungsband am Hochspannungsschrank WE1 nicht verschraubt, hängt lose herab. Werker hat es vergessen anzuschließen. Lebensgefahr beim Einschalten der Fahrleitungsspannung!", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker hat es vergessen anzuschließen. Lebensgefahr beim Einschalten"}, "cot_begruendung": "Das Vergessen des Erdungsbandes durch den Werker ist ein klassischer Montagefehler im eigenen Werk. Da eine lose Erdung an einem Hochspannungsschrank absolute Lebensgefahr bedeutet und die IBS verhindert, ist es ein kritischer Blocker."}]</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>[{"fall_id": "75", "text": "Großer Spiegel in der Nasszelle komplett zersplittert. Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang.", "zielvariablen": {"grundursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang."}, "cot_begruendung": "Der durchstoßene Karton im Wareneingang durch einen Gabelstapler ist ein eindeutiger Transportschaden (Logistik). Ein kaputter Spiegel muss bestellt und nachgearbeitet werden, hält den Zugbau aber nicht auf."}, {"fall_id": "30", "text": "Gummiprofil an Einstiegstür WE1 rissig. Betrifft Lieferung von ABC-Gummi der KW12 komplett. Material ist spröde.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Betrifft Lieferung von ABC-Gummi der KW12 komplett. Material ist spröde."}, "cot_begruendung": "Das spröde Gummiprofil ist auf eine fehlerhafte Materiallieferung von 'ABC-Gummi' zurückzuführen (Material/Lieferant). Der Hinweis 'Lieferung [...] komplett' markiert dies eindeutig als Serienfehler. Ein rissiges Gummi muss getauscht werden (Nacharbeit)."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}]</t>
+          <t>[{"fall_id": "75", "text": "Großer Spiegel in der Nasszelle komplett zersplittert. Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang.", "zielvariablen": {"ursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang."}, "cot_begruendung": "Der durchstoßene Karton im Wareneingang durch einen Gabelstapler ist ein eindeutiger Transportschaden (Logistik). Ein kaputter Spiegel muss bestellt und nachgearbeitet werden, hält den Zugbau aber nicht auf."}, {"fall_id": "104", "text": "Wischwasserbehälter WE1 undicht. Schweißnaht am Kunststoffgehäuse hat Haarrisse. Offenbar Produktionsfehler vom Hersteller. Tropft auf die darunterliegende Elektrik. Sofortiger Tausch nötig.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Schweißnaht am Kunststoffgehäuse hat Haarrisse. Offenbar Produktionsfehler vom Hersteller."}, "cot_begruendung": "Ein undichter Behälter aufgrund von Haarrissen in der Schweißnaht ab Werk ist ein Materialfehler, der vom Hersteller (Lieferant) verursacht wurde. Da das Wasser auf die Elektrik tropft und ein sofortiger Tausch gefordert wird, liegt eine hohe Kritikalität (Blocker) vor."}, {"fall_id": "162", "text": "Graue Flecken auf dem neuen Fußbodenbelag im FGR. Reinigungskraft hat den Spezialreiniger nicht richtig verdünnt, wodurch Rückstände beim Trocknen entstanden sind. Einmal feucht nachwischen behebt das Problem.", "zielvariablen": {"ursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Reinigungskraft hat den Spezialreiniger nicht richtig verdünnt"}, "cot_begruendung": "Falsche Dosierung des Reinigungsmittels durch die Reinigungskraft ist ein klassischer Fehler der internen Reinigung (Werk). Da sich der Mangel durch simples Nachwischen beheben lässt, wird er als 'Info' oder sehr leichte Nacharbeit deklariert."}]</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>[{"fall_id": "87", "text": "Riss in der Bremsscheibe WE2 Achse 1. Metallurgische Prüfung zeigt Lunker im Guss. Alle Scheiben der Charge von Fa. [Platzhalter] betroffen. Keine Streckenfreigabe.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Lunker im Guss. Alle Scheiben der Charge von Fa. [Platzhalter] betroffen. Keine Streckenfreigabe."}, "cot_begruendung": "Lunker im Guss bei Lieferung durch eine externe Firma sind ein massiver Materialfehler des Lieferanten. Das Wort 'Charge' kennzeichnet es als Serienfehler. Da sicherheitsrelevante Bremsen betroffen sind und die Streckenfreigabe verweigert wird, ist dies ein absoluter Blocker."}, {"fall_id": "69", "text": "HVAC-Einheit für WE2 mit tiefen Kratzern und verbogenen Lamellen angeliefert worden. Verpackung war aufgerissen. Eindeutiger Handhabungsschaden durch Zulieferer Fa. [Platzhalter] vor Versand.", "zielvariablen": {"grundursache": "Handhabung", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Eindeutiger Handhabungsschaden durch Zulieferer Fa. [Platzhalter] vor Versand."}, "cot_begruendung": "Der Schaden wird explizit als Handhabungsfehler durch den externen Zulieferer vor dem Versand identifiziert (Handhabung/Lieferant). Verborgene Lamellen erfordern eine Nacharbeit, stoppen aber die generelle Produktion des Wagens meist nicht sofort."}, {"fall_id": "26", "text": "Hauptkabelstrang HKS-3 unterflur am Drehgestell WE2 durchtrennt. Staplerfahrer hat beim Abladen der Palette reingestochen. Kabelbaum muss komplett neu.", "zielvariablen": {"grundursache": "Handhabung", "ursprung": "Logistik", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Staplerfahrer hat beim Abladen der Palette reingestochen"}, "cot_begruendung": "Der Text beschreibt eindeutig eine mechanische Beschädigung durch einen Staplerfahrer beim Abladen. Dies ist ein Handhabungsfehler, der der Logistik zuzuordnen ist. Da der Hauptkabelstrang komplett neu muss, kann das Fahrzeug elektrisch nicht in Betrieb genommen werden (Blocker)."}]</t>
+          <t>[{"fall_id": "87", "text": "Riss in der Bremsscheibe WE2 Achse 1. Metallurgische Prüfung zeigt Lunker im Guss. Alle Scheiben der Charge von Fa. [Platzhalter] betroffen. Keine Streckenfreigabe.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Lunker im Guss. Alle Scheiben der Charge von Fa. [Platzhalter] betroffen. Keine Streckenfreigabe."}, "cot_begruendung": "Lunker im Guss bei Lieferung durch eine externe Firma sind ein massiver Materialfehler des Lieferanten. Das Wort 'Charge' kennzeichnet es als Serienfehler. Da sicherheitsrelevante Bremsen betroffen sind und die Streckenfreigabe verweigert wird, ist dies ein absoluter Blocker."}, {"fall_id": "130", "text": "Ultraschallprüfung der Achswelle WE1 zeigt Haarriss im Material. Vermutlich fehlerhafter Schmiedeprozess beim Hersteller XYZ. Achse darf nicht verbaut werden.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Haarriss im Material. Vermutlich fehlerhafter Schmiedeprozess beim Hersteller XYZ. Achse darf nicht verbaut werden."}, "cot_begruendung": "Ein Haarriss im Schmiedestahl, der auf den Hersteller zurückzuführen ist, ist ein Materialfehler beim Lieferanten. Eine defekte Achswelle ist ein hochsicherheitsrelevantes Bauteil; ein Einbauverbot bedeutet Blocker-Status."}, {"fall_id": "69", "text": "HVAC-Einheit für WE2 mit tiefen Kratzern und verbogenen Lamellen angeliefert worden. Verpackung war aufgerissen. Eindeutiger Handhabungsschaden durch Zulieferer Fa. [Platzhalter] vor Versand.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Eindeutiger Handhabungsschaden durch Zulieferer Fa. [Platzhalter] vor Versand."}, "cot_begruendung": "Der Schaden wird explizit als Handhabungsfehler durch den externen Zulieferer vor dem Versand identifiziert (Handhabung/Lieferant). Verborgene Lamellen erfordern eine Nacharbeit, stoppen aber die generelle Produktion des Wagens meist nicht sofort."}]</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>[{"fall_id": "8", "text": "Frontmaske hat matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend. Muss poliert/nachlackiert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend"}, "cot_begruendung": "Fehler beim Auftragen des Lacks ('Klarlack teilweise nicht deckend') weisen auf einen Verarbeitungs- bzw. Prozessfehler direkt in der Werksfertigung hin. Dies erfordert eine optische Nacharbeit, stellt aber keine funktionale Blockade dar."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}]</t>
+          <t>[{"fall_id": "8", "text": "Frontmaske hat matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend. Muss poliert/nachlackiert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend"}, "cot_begruendung": "Fehler beim Auftragen des Lacks ('Klarlack teilweise nicht deckend') weisen auf einen Verarbeitungs- bzw. Prozessfehler direkt in der Werksfertigung hin. Dies erfordert eine optische Nacharbeit, stellt aber keine funktionale Blockade dar."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "109", "text": "Isolationsmatte hinter Türvoute LWS falsch zugeschnitten. Werker hat statt der Schablone B die Schablone A verwendet. Matte deckt den Kältebereich nicht vollständig ab.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat statt der Schablone B die Schablone A verwendet."}, "cot_begruendung": "Die Verwendung einer falschen Schablone durch den internen Werker beim Zuschnitt ist ein Verarbeitungs- bzw. Montagefehler im Werk. Die falsche Matte muss entfernt und durch eine korrekt zugeschnittene ersetzt werden (Nacharbeit)."}]</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>[{"fall_id": "2", "text": "Seitenwandverkleidung RWS im Einstiegsbereich weist tiefe Kratzer auf. Betrifft die letzten 5 angelieferten Wagen. Falsche Stapelung in Transportbox durch Spedition.", "zielvariablen": {"grundursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Betrifft die letzten 5 angelieferten Wagen. Falsche Stapelung in Transportbox"}, "cot_begruendung": "Der Schaden entstand explizit durch 'Falsche Stapelung in Transportbox' durch die Spedition, woraus sich Transport/Logistik als Verursacher ableiten lässt. Der Hinweis 'letzten 5 angelieferten Wagen' ist ein klarer Indikator für einen Serienfehler. Der Kratzer muss nachgearbeitet werden, stoppt aber nicht sofort die gesamte Produktion."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}, {"fall_id": "21", "text": "Spaltmaß bei Übergangstür WE2 zu groß (&gt;8mm). Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3"}, "cot_begruendung": "Wenn Scharniere physisch nicht weiter justierbar sind, liegt oft ein Toleranz- oder Konstruktionsproblem (Engineering) vor, weniger ein Montagefehler. Der explizite Hinweis auf 'Wagen 1, 2 und 3' ist ein eindeutiger Indikator für einen Serienfehler. Ein falsches Spaltmaß erfordert Nacharbeit."}]</t>
+          <t>[{"fall_id": "2", "text": "Seitenwandverkleidung RWS im Einstiegsbereich weist tiefe Kratzer auf. Betrifft die letzten 5 angelieferten Wagen. Falsche Stapelung in Transportbox durch Spedition.", "zielvariablen": {"ursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Betrifft die letzten 5 angelieferten Wagen. Falsche Stapelung in Transportbox"}, "cot_begruendung": "Der Schaden entstand explizit durch 'Falsche Stapelung in Transportbox' durch die Spedition, woraus sich Transport/Logistik als Verursacher ableiten lässt. Der Hinweis 'letzten 5 angelieferten Wagen' ist ein klarer Indikator für einen Serienfehler. Der Kratzer muss nachgearbeitet werden, stoppt aber nicht sofort die gesamte Produktion."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}, {"fall_id": "106", "text": "Spaltmaß zwischen den Dachpaneelen im FGR RWS zu gering. Dehnungsausgleich nicht möglich. Laut 3D-Modell in Revision E ist das Paneel 5mm zu lang gezeichnet. QA sperrt den weiteren Deckenausbau.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Laut 3D-Modell in Revision E ist das Paneel 5mm zu lang gezeichnet. QA sperrt den weiteren Deckenausbau."}, "cot_begruendung": "Eine fehlerhafte Längenangabe im 3D-Modell verweist auf einen Konstruktionsfehler durch das Engineering. Die explizite Sperrung des weiteren Deckenausbaus durch die Qualitätsabteilung (QA) stuft dieses Problem als Blocker ein."}]</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}, {"fall_id": "61", "text": "Schrauben an der Bugnase WE1 mit 40Nm statt 25Nm angezogen. Gewinde teilweise überdreht. Vorgabe im Arbeitsplan wurde von Schicht 1 missachtet.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "mit 40Nm statt 25Nm angezogen. Vorgabe im Arbeitsplan wurde von Schicht 1 missachtet."}, "cot_begruendung": "Das Missachten der Drehmoment-Vorgaben aus dem Arbeitsplan durch die interne Schicht ist ein prozessualer bzw. Montagefehler im Werk. Beschädigte Gewinde müssen nachgearbeitet/ersetzt werden (Nacharbeit)."}]</t>
+          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"ursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}, {"fall_id": "152", "text": "Abdeckbleche für die Heizkanäle LWS aus unserer eigenen Stanzerei sind an der Kante um 10 Grad zu wenig abgekantet. Betrifft alle 40 Bleche von heute. Können so nicht montiert werden, Kante steht ab.", "zielvariablen": {"ursache": "Fertigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "aus unserer eigenen Stanzerei sind an der Kante um 10 Grad zu wenig abgekantet. Betrifft alle 40 Bleche"}, "cot_begruendung": "Ein Biegefehler aus der 'eigenen Stanzerei' ist ein interner Fertigungsfehler (Werk). Da 'alle 40 Bleche von heute' betroffen sind, liegt ein Serienfehler vor. Die Bleche müssen nachgebogen werden (Nacharbeit), stoppen aber nicht den kompletten Wagenausbau."}]</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>[{"fall_id": "44", "text": "Befestigung der Haltestange im FGR LWS lose. Werker hat vergessen, die Kontermutter anzubringen. Muss dringend nachgezogen werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, die Kontermutter anzubringen"}, "cot_begruendung": "Das explizite Vergessen der Kontermutter durch den Werker ist ein klassischer Montagefehler, der im eigenen Werk entstanden ist. Das Nachziehen der Mutter ist eine unkritische Nacharbeit."}, {"fall_id": "27", "text": "Scheibe RWS im FGR schmierig. Putzkolonne hat falsches Reinigungsmittel verwendet, Schlieren lassen sich schwer entfernen.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Putzkolonne hat falsches Reinigungsmittel verwendet"}, "cot_begruendung": "Die Verschmutzung wurde explizit durch die Putzkolonne ('falsches Reinigungsmittel') verursacht. Dies ist ein Reinigungsfehler im Werk. Da dies weder die Montage aufhält noch ein Bauteil zerstört, wird es als reine Nacharbeit/Info eingestuft."}, {"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}]</t>
+          <t>[{"fall_id": "44", "text": "Befestigung der Haltestange im FGR LWS lose. Werker hat vergessen, die Kontermutter anzubringen. Muss dringend nachgezogen werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, die Kontermutter anzubringen"}, "cot_begruendung": "Das explizite Vergessen der Kontermutter durch den Werker ist ein klassischer Montagefehler, der im eigenen Werk entstanden ist. Das Nachziehen der Mutter ist eine unkritische Nacharbeit."}, {"fall_id": "117", "text": "Befestigung der Sitzkiste RWS im FGR wackelt. Werker hat statt der M8x25 eine M8x40 Schraube mit Gewalt reingedreht und das Gewinde im Boden zerstört. Gewindeeinsatz muss neu gesetzt werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat statt der M8x25 eine M8x40 Schraube mit Gewalt reingedreht"}, "cot_begruendung": "Die Zerstörung des Gewindes durch den Werker (falsche Schraube, Gewaltanwendung) ist ein klarer Montage- und Handhabungsfehler im eigenen Werk. Die Reparatur des Gewindes ist zwar aufwendig, stellt aber einen lokalen Eingriff dar (Nacharbeit)."}, {"fall_id": "179", "text": "Notbrems-Zugschalter im FGR LWS löst bei Betätigung nicht aus. Werker der Schicht 3 hat Pin 1 und Pin 2 am Stecker X4 vertauscht. Bremsschleife ist dadurch dauerhaft überbrückt. Lebensgefahr!", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker der Schicht 3 hat Pin 1 und Pin 2 am Stecker X4 vertauscht."}, "cot_begruendung": "Vertauschte Pins durch einen Werker der internen Schicht sind ein Montagefehler im Werk. Da eine defekte Notbremse ein sicherheitskritischer Mangel ist, der die Streckenzulassung unmöglich macht, wird dies als Blocker kategorisiert."}]</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>[{"fall_id": "58", "text": "Lack zerkratzt.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Lack zerkratzt."}, "cot_begruendung": "Der Text beschreibt lediglich das Symptom 'Lack zerkratzt', liefert jedoch keinen Kontext zur Entstehung (z. B. Transport, unachtsamer Werker, Reinigung). Zur Vermeidung von Halluzinationen muss die Abstention-Logik angewandt und 'Unbekannt' ausgegeben werden."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
+          <t>[{"fall_id": "58", "text": "Lack zerkratzt.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Lack zerkratzt."}, "cot_begruendung": "Der Text beschreibt lediglich das Symptom 'Lack zerkratzt', liefert jedoch keinen Kontext zur Entstehung (z. B. Transport, unachtsamer Werker, Reinigung). Zur Vermeidung von Halluzinationen muss die Abstention-Logik angewandt und 'Unbekannt' ausgegeben werden."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
         </is>
       </c>
     </row>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>[{"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "62", "text": "Kabelkanal unterflur kollidiert mit der Druckluftleitung für die Bremsanlage. Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich."}, "cot_begruendung": "Eine Überlappung im 3D-Modell/Zeichnung ist ein Konstruktionsfehler aus dem Engineering. Da die Druckluftleitung für die Bremsen essenziell ist und die 'Rohrverlegung aktuell unmöglich' ist, handelt es sich um einen harten Blocker."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
+          <t>[{"fall_id": "104", "text": "Wischwasserbehälter WE1 undicht. Schweißnaht am Kunststoffgehäuse hat Haarrisse. Offenbar Produktionsfehler vom Hersteller. Tropft auf die darunterliegende Elektrik. Sofortiger Tausch nötig.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Schweißnaht am Kunststoffgehäuse hat Haarrisse. Offenbar Produktionsfehler vom Hersteller."}, "cot_begruendung": "Ein undichter Behälter aufgrund von Haarrissen in der Schweißnaht ab Werk ist ein Materialfehler, der vom Hersteller (Lieferant) verursacht wurde. Da das Wasser auf die Elektrik tropft und ein sofortiger Tausch gefordert wird, liegt eine hohe Kritikalität (Blocker) vor."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "62", "text": "Kabelkanal unterflur kollidiert mit der Druckluftleitung für die Bremsanlage. Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich."}, "cot_begruendung": "Eine Überlappung im 3D-Modell/Zeichnung ist ein Konstruktionsfehler aus dem Engineering. Da die Druckluftleitung für die Bremsen essenziell ist und die 'Rohrverlegung aktuell unmöglich' ist, handelt es sich um einen harten Blocker."}]</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>[{"fall_id": "48", "text": "Sensorkabel am Drehgestell WE1 abgerissen. Wurde beim Einziehen durch die enge Tülle vom Montage-Team überdehnt.", "zielvariablen": {"grundursache": "Handhabung", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Wurde beim Einziehen durch die enge Tülle vom Montage-Team überdehnt."}, "cot_begruendung": "Das Überdehnen des Kabels durch das interne Montage-Team ist ein Handhabungsfehler im Werk. Da ein abgerissenes Sensorkabel am sicherheitsrelevanten Drehgestell die Inbetriebnahme verhindert, ist es als Blocker einzustufen."}, {"fall_id": "61", "text": "Schrauben an der Bugnase WE1 mit 40Nm statt 25Nm angezogen. Gewinde teilweise überdreht. Vorgabe im Arbeitsplan wurde von Schicht 1 missachtet.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "mit 40Nm statt 25Nm angezogen. Vorgabe im Arbeitsplan wurde von Schicht 1 missachtet."}, "cot_begruendung": "Das Missachten der Drehmoment-Vorgaben aus dem Arbeitsplan durch die interne Schicht ist ein prozessualer bzw. Montagefehler im Werk. Beschädigte Gewinde müssen nachgearbeitet/ersetzt werden (Nacharbeit)."}, {"fall_id": "100", "text": "Schraube M8x20 an Haltestange im FGR WE2 rundgedreht. Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden."}, "cot_begruendung": "Das Runddrehen einer Schraube durch Nutzung eines falschen Bits durch den Werker ist ein Montagefehler im Werk. Das Ausbohren der defekten Schraube ist zeitintensiv, aber eine klassische Nacharbeit, die den Fertigungsablauf nicht komplett stoppt."}]</t>
+          <t>[{"fall_id": "48", "text": "Sensorkabel am Drehgestell WE1 abgerissen. Wurde beim Einziehen durch die enge Tülle vom Montage-Team überdehnt.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Wurde beim Einziehen durch die enge Tülle vom Montage-Team überdehnt."}, "cot_begruendung": "Das Überdehnen des Kabels durch das interne Montage-Team ist ein Handhabungsfehler im Werk. Da ein abgerissenes Sensorkabel am sicherheitsrelevanten Drehgestell die Inbetriebnahme verhindert, ist es als Blocker einzustufen."}, {"fall_id": "179", "text": "Notbrems-Zugschalter im FGR LWS löst bei Betätigung nicht aus. Werker der Schicht 3 hat Pin 1 und Pin 2 am Stecker X4 vertauscht. Bremsschleife ist dadurch dauerhaft überbrückt. Lebensgefahr!", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker der Schicht 3 hat Pin 1 und Pin 2 am Stecker X4 vertauscht."}, "cot_begruendung": "Vertauschte Pins durch einen Werker der internen Schicht sind ein Montagefehler im Werk. Da eine defekte Notbremse ein sicherheitskritischer Mangel ist, der die Streckenzulassung unmöglich macht, wird dies als Blocker kategorisiert."}, {"fall_id": "61", "text": "Schrauben an der Bugnase WE1 mit 40Nm statt 25Nm angezogen. Gewinde teilweise überdreht. Vorgabe im Arbeitsplan wurde von Schicht 1 missachtet.", "zielvariablen": {"ursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "mit 40Nm statt 25Nm angezogen. Vorgabe im Arbeitsplan wurde von Schicht 1 missachtet."}, "cot_begruendung": "Das Missachten der Drehmoment-Vorgaben aus dem Arbeitsplan durch die interne Schicht ist ein prozessualer bzw. Montagefehler im Werk. Beschädigte Gewinde müssen nachgearbeitet/ersetzt werden (Nacharbeit)."}]</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2076,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>[{"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "82", "text": "Tiefer Kratzer auf dem Führerpult. IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen.", "zielvariablen": {"grundursache": "Handhabung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen."}, "cot_begruendung": "Das Fallenlassen des Laptops durch den Mitarbeiter ist ein Handhabungsfehler im eigenen Werk. Optische Kratzer erfordern Nacharbeit (Austausch oder Politur)."}]</t>
+          <t>[{"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "82", "text": "Tiefer Kratzer auf dem Führerpult. IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen."}, "cot_begruendung": "Das Fallenlassen des Laptops durch den Mitarbeiter ist ein Handhabungsfehler im eigenen Werk. Optische Kratzer erfordern Nacharbeit (Austausch oder Politur)."}]</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>[{"fall_id": "75", "text": "Großer Spiegel in der Nasszelle komplett zersplittert. Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang.", "zielvariablen": {"grundursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang."}, "cot_begruendung": "Der durchstoßene Karton im Wareneingang durch einen Gabelstapler ist ein eindeutiger Transportschaden (Logistik). Ein kaputter Spiegel muss bestellt und nachgearbeitet werden, hält den Zugbau aber nicht auf."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}]</t>
+          <t>[{"fall_id": "133", "text": "Kiste mit den WC-Spiegeln wurde vom Zulieferer [Platzhalter] stark beschädigt angeliefert. Spiegel innen sind zerkratzt. Wareneingang hat die Palette leider ungeprüft angenommen.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "vom Zulieferer [Platzhalter] stark beschädigt angeliefert. Spiegel innen sind zerkratzt."}, "cot_begruendung": "Der Schaden wird explizit dem Zulieferer zugeschrieben, der die Palette bereits beschädigt angeliefert hat (Handhabung/Lieferant). Zerkratzte Spiegel müssen ausgetauscht werden, stellen aber eine einfache Nacharbeit dar."}, {"fall_id": "75", "text": "Großer Spiegel in der Nasszelle komplett zersplittert. Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang.", "zielvariablen": {"ursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang."}, "cot_begruendung": "Der durchstoßene Karton im Wareneingang durch einen Gabelstapler ist ein eindeutiger Transportschaden (Logistik). Ein kaputter Spiegel muss bestellt und nachgearbeitet werden, hält den Zugbau aber nicht auf."}, {"fall_id": "104", "text": "Wischwasserbehälter WE1 undicht. Schweißnaht am Kunststoffgehäuse hat Haarrisse. Offenbar Produktionsfehler vom Hersteller. Tropft auf die darunterliegende Elektrik. Sofortiger Tausch nötig.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Schweißnaht am Kunststoffgehäuse hat Haarrisse. Offenbar Produktionsfehler vom Hersteller."}, "cot_begruendung": "Ein undichter Behälter aufgrund von Haarrissen in der Schweißnaht ab Werk ist ein Materialfehler, der vom Hersteller (Lieferant) verursacht wurde. Da das Wasser auf die Elektrik tropft und ein sofortiger Tausch gefordert wird, liegt eine hohe Kritikalität (Blocker) vor."}]</t>
         </is>
       </c>
     </row>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>[{"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}, {"fall_id": "46", "text": "Großer Kratzer auf Trennglas im FGR. Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen"}, "cot_begruendung": "Die Beschädigung wurde direkt durch die Reinigungskraft beim Wischen verursacht (Reinigung/Werk). Ein zerkratztes Glas in der Trennwand muss getauscht werden (Nacharbeit), stoppt aber nicht die Produktion."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
+          <t>[{"fall_id": "187", "text": "Haltebleche für alle 12 Mülleimer im FGR aus unserer Schlosserei sind um 15 Grad zu wenig gebogen. Mülleimer rutschen aus der Halterung. Kantpresse war falsch programmiert. Bleche müssen neu gemacht werden.", "zielvariablen": {"ursache": "Fertigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "aus unserer Schlosserei sind um 15 Grad zu wenig gebogen. [...] Kantpresse war falsch programmiert."}, "cot_begruendung": "Eine falsch programmierte Kantpresse in der 'eigenen Schlosserei' ist ein interner Fertigungsfehler (Werk). Da 'alle 12 Mülleimer' betroffen sind, liegt ein Serienfehler vor. Die Bleche müssen neu produziert werden (Nacharbeit)."}, {"fall_id": "104", "text": "Wischwasserbehälter WE1 undicht. Schweißnaht am Kunststoffgehäuse hat Haarrisse. Offenbar Produktionsfehler vom Hersteller. Tropft auf die darunterliegende Elektrik. Sofortiger Tausch nötig.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Schweißnaht am Kunststoffgehäuse hat Haarrisse. Offenbar Produktionsfehler vom Hersteller."}, "cot_begruendung": "Ein undichter Behälter aufgrund von Haarrissen in der Schweißnaht ab Werk ist ein Materialfehler, der vom Hersteller (Lieferant) verursacht wurde. Da das Wasser auf die Elektrik tropft und ein sofortiger Tausch gefordert wird, liegt eine hohe Kritikalität (Blocker) vor."}, {"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"ursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}]</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>[{"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "75", "text": "Großer Spiegel in der Nasszelle komplett zersplittert. Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang.", "zielvariablen": {"grundursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang."}, "cot_begruendung": "Der durchstoßene Karton im Wareneingang durch einen Gabelstapler ist ein eindeutiger Transportschaden (Logistik). Ein kaputter Spiegel muss bestellt und nachgearbeitet werden, hält den Zugbau aber nicht auf."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
+          <t>[{"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "75", "text": "Großer Spiegel in der Nasszelle komplett zersplittert. Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang.", "zielvariablen": {"ursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang."}, "cot_begruendung": "Der durchstoßene Karton im Wareneingang durch einen Gabelstapler ist ein eindeutiger Transportschaden (Logistik). Ein kaputter Spiegel muss bestellt und nachgearbeitet werden, hält den Zugbau aber nicht auf."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>[{"fall_id": "44", "text": "Befestigung der Haltestange im FGR LWS lose. Werker hat vergessen, die Kontermutter anzubringen. Muss dringend nachgezogen werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, die Kontermutter anzubringen"}, "cot_begruendung": "Das explizite Vergessen der Kontermutter durch den Werker ist ein klassischer Montagefehler, der im eigenen Werk entstanden ist. Das Nachziehen der Mutter ist eine unkritische Nacharbeit."}, {"fall_id": "100", "text": "Schraube M8x20 an Haltestange im FGR WE2 rundgedreht. Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden."}, "cot_begruendung": "Das Runddrehen einer Schraube durch Nutzung eines falschen Bits durch den Werker ist ein Montagefehler im Werk. Das Ausbohren der defekten Schraube ist zeitintensiv, aber eine klassische Nacharbeit, die den Fertigungsablauf nicht komplett stoppt."}, {"fall_id": "13", "text": "Hauptschalter am Dach WE1 löst bei 100A aus, Spezifikation fordert 150A. Alle Schalter der aktuellen Charge von Fa. [Platzhalter] sind betroffen. IBS kann nicht fortgesetzt werden.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Alle Schalter der aktuellen Charge von Fa. [Platzhalter] sind betroffen"}, "cot_begruendung": "Das Bauteil erfüllt nicht die geforderte Spezifikation, was auf einen Materialfehler des externen Lieferanten ('Fa. [Platzhalter]') hinweist. Da die IBS (Inbetriebsetzung) nicht fortgesetzt werden kann, ist dies ein harter Blocker. Der Hinweis 'Alle Schalter der aktuellen Charge' markiert es klar als Serienfehler."}]</t>
+          <t>[{"fall_id": "101", "text": "Klemmschutz an Fahrgasttür 3 LWS löst viel zu früh aus. Schließvorgang bricht bei leichtem Windstoß ab. Sensorik-Parameter in der neuen Türsoftware (V1.4) von Fa. [Platzhalter] sind zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte angefordert.", "zielvariablen": {"ursache": "Software", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Sensorik-Parameter in der neuen Türsoftware [...] zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte"}, "cot_begruendung": "Der Text beschreibt ein funktionales Problem der Fahrgasttür aufgrund zu empfindlicher Parameter in der 'neuen Türsoftware', welche von einem externen Lieferanten stammt. Da die 'gesamte Flotte' ein Update benötigt, handelt es sich um einen Serienfehler. Ein fehlerhafter Klemmschutz betrifft die Sicherheit und Zuverlässigkeit der Türen, was die Inbetriebnahme blockiert."}, {"fall_id": "128", "text": "Brandschottung an Kabeldurchführung zum Fahrerstand fehlt komplett. Schicht 2 hat die Durchführung offen gelassen und mit dem Innenausbau weitergemacht. Akute Brandgefahr, keine Zulassung möglich.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Schicht 2 hat die Durchführung offen gelassen und mit dem Innenausbau weitergemacht. Akute Brandgefahr"}, "cot_begruendung": "Das Vergessen der Brandschottung durch die interne Schicht ist ein grober Montagefehler. Eine fehlende Brandschottung stellt eine Gefahr für Leib und Leben dar und verhindert die Zulassung zwingend, weshalb es sich um einen harten Blocker handelt."}, {"fall_id": "44", "text": "Befestigung der Haltestange im FGR LWS lose. Werker hat vergessen, die Kontermutter anzubringen. Muss dringend nachgezogen werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, die Kontermutter anzubringen"}, "cot_begruendung": "Das explizite Vergessen der Kontermutter durch den Werker ist ein klassischer Montagefehler, der im eigenen Werk entstanden ist. Das Nachziehen der Mutter ist eine unkritische Nacharbeit."}]</t>
         </is>
       </c>
     </row>
@@ -2451,7 +2451,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>[{"fall_id": "69", "text": "HVAC-Einheit für WE2 mit tiefen Kratzern und verbogenen Lamellen angeliefert worden. Verpackung war aufgerissen. Eindeutiger Handhabungsschaden durch Zulieferer Fa. [Platzhalter] vor Versand.", "zielvariablen": {"grundursache": "Handhabung", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Eindeutiger Handhabungsschaden durch Zulieferer Fa. [Platzhalter] vor Versand."}, "cot_begruendung": "Der Schaden wird explizit als Handhabungsfehler durch den externen Zulieferer vor dem Versand identifiziert (Handhabung/Lieferant). Verborgene Lamellen erfordern eine Nacharbeit, stoppen aber die generelle Produktion des Wagens meist nicht sofort."}, {"fall_id": "44", "text": "Befestigung der Haltestange im FGR LWS lose. Werker hat vergessen, die Kontermutter anzubringen. Muss dringend nachgezogen werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, die Kontermutter anzubringen"}, "cot_begruendung": "Das explizite Vergessen der Kontermutter durch den Werker ist ein klassischer Montagefehler, der im eigenen Werk entstanden ist. Das Nachziehen der Mutter ist eine unkritische Nacharbeit."}, {"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}]</t>
+          <t>[{"fall_id": "69", "text": "HVAC-Einheit für WE2 mit tiefen Kratzern und verbogenen Lamellen angeliefert worden. Verpackung war aufgerissen. Eindeutiger Handhabungsschaden durch Zulieferer Fa. [Platzhalter] vor Versand.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Eindeutiger Handhabungsschaden durch Zulieferer Fa. [Platzhalter] vor Versand."}, "cot_begruendung": "Der Schaden wird explizit als Handhabungsfehler durch den externen Zulieferer vor dem Versand identifiziert (Handhabung/Lieferant). Verborgene Lamellen erfordern eine Nacharbeit, stoppen aber die generelle Produktion des Wagens meist nicht sofort."}, {"fall_id": "44", "text": "Befestigung der Haltestange im FGR LWS lose. Werker hat vergessen, die Kontermutter anzubringen. Muss dringend nachgezogen werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, die Kontermutter anzubringen"}, "cot_begruendung": "Das explizite Vergessen der Kontermutter durch den Werker ist ein klassischer Montagefehler, der im eigenen Werk entstanden ist. Das Nachziehen der Mutter ist eine unkritische Nacharbeit."}, {"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"ursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}]</t>
         </is>
       </c>
     </row>
@@ -2526,7 +2526,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>[{"fall_id": "100", "text": "Schraube M8x20 an Haltestange im FGR WE2 rundgedreht. Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden."}, "cot_begruendung": "Das Runddrehen einer Schraube durch Nutzung eines falschen Bits durch den Werker ist ein Montagefehler im Werk. Das Ausbohren der defekten Schraube ist zeitintensiv, aber eine klassische Nacharbeit, die den Fertigungsablauf nicht komplett stoppt."}, {"fall_id": "82", "text": "Tiefer Kratzer auf dem Führerpult. IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen.", "zielvariablen": {"grundursache": "Handhabung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen."}, "cot_begruendung": "Das Fallenlassen des Laptops durch den Mitarbeiter ist ein Handhabungsfehler im eigenen Werk. Optische Kratzer erfordern Nacharbeit (Austausch oder Politur)."}, {"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}]</t>
+          <t>[{"fall_id": "197", "text": "Türen lassen sich nach der IBS nicht zentral schließen. Werker hat versehentlich die veraltete Tür-Software V1.0 von seinem lokalen USB-Stick geflasht, anstatt die freigegebene V1.2 vom Server zu ziehen. Alle Türen am Wagen müssen neu bespielt werden.", "zielvariablen": {"ursache": "Software", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker hat versehentlich die veraltete Tür-Software V1.0 von seinem lokalen USB-Stick geflasht"}, "cot_begruendung": "Das Aufspielen einer falschen/veralteten Software durch den Werker ist ein softwareseitiger und prozessualer Fehler, der direkt im Werk entstanden ist (Software/Werk). Da die sicherheitskritische zentrale Türschließung nicht funktioniert, ist die Inbetriebnahme hart blockiert."}, {"fall_id": "100", "text": "Schraube M8x20 an Haltestange im FGR WE2 rundgedreht. Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden."}, "cot_begruendung": "Das Runddrehen einer Schraube durch Nutzung eines falschen Bits durch den Werker ist ein Montagefehler im Werk. Das Ausbohren der defekten Schraube ist zeitintensiv, aber eine klassische Nacharbeit, die den Fertigungsablauf nicht komplett stoppt."}, {"fall_id": "82", "text": "Tiefer Kratzer auf dem Führerpult. IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen."}, "cot_begruendung": "Das Fallenlassen des Laptops durch den Mitarbeiter ist ein Handhabungsfehler im eigenen Werk. Optische Kratzer erfordern Nacharbeit (Austausch oder Politur)."}]</t>
         </is>
       </c>
     </row>
@@ -2601,7 +2601,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>[{"fall_id": "42", "text": "Zugsteuerung ZSG bootet nicht. Laut Herrn [Platzhalter] fehlt das gestrige Software-Patch für den CAN-Bus. Gesamte IBS steht aktuell.", "zielvariablen": {"grundursache": "Software", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "fehlt das gestrige Software-Patch für den CAN-Bus. Gesamte IBS steht aktuell"}, "cot_begruendung": "Ein fehlendes Software-Patch für ein Steuergerät, das zentral entwickelt wird, fällt in den Bereich Software/Engineering. Da die 'Gesamte IBS steht', ist der Fehler funktionskritisch und somit eindeutig ein Blocker."}, {"fall_id": "82", "text": "Tiefer Kratzer auf dem Führerpult. IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen.", "zielvariablen": {"grundursache": "Handhabung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen."}, "cot_begruendung": "Das Fallenlassen des Laptops durch den Mitarbeiter ist ein Handhabungsfehler im eigenen Werk. Optische Kratzer erfordern Nacharbeit (Austausch oder Politur)."}, {"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}]</t>
+          <t>[{"fall_id": "42", "text": "Zugsteuerung ZSG bootet nicht. Laut Herrn [Platzhalter] fehlt das gestrige Software-Patch für den CAN-Bus. Gesamte IBS steht aktuell.", "zielvariablen": {"ursache": "Software", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "fehlt das gestrige Software-Patch für den CAN-Bus. Gesamte IBS steht aktuell"}, "cot_begruendung": "Ein fehlendes Software-Patch für ein Steuergerät, das zentral entwickelt wird, fällt in den Bereich Software/Engineering. Da die 'Gesamte IBS steht', ist der Fehler funktionskritisch und somit eindeutig ein Blocker."}, {"fall_id": "197", "text": "Türen lassen sich nach der IBS nicht zentral schließen. Werker hat versehentlich die veraltete Tür-Software V1.0 von seinem lokalen USB-Stick geflasht, anstatt die freigegebene V1.2 vom Server zu ziehen. Alle Türen am Wagen müssen neu bespielt werden.", "zielvariablen": {"ursache": "Software", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker hat versehentlich die veraltete Tür-Software V1.0 von seinem lokalen USB-Stick geflasht"}, "cot_begruendung": "Das Aufspielen einer falschen/veralteten Software durch den Werker ist ein softwareseitiger und prozessualer Fehler, der direkt im Werk entstanden ist (Software/Werk). Da die sicherheitskritische zentrale Türschließung nicht funktioniert, ist die Inbetriebnahme hart blockiert."}, {"fall_id": "188", "text": "Diagnose-Software (ZSG) meldet 'Drehgestell 2 fehlt'. Code-Fehler im letzten Software-Update V4.1 des Engineering-Teams unterdrückt die CAN-ID des zweiten Bogies. Zug darf so nicht bewegt werden.", "zielvariablen": {"ursache": "Software", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Code-Fehler im letzten Software-Update V4.1 des Engineering-Teams unterdrückt die CAN-ID"}, "cot_begruendung": "Ein fehlerhafter Code in einem Software-Update durch das Engineering-Team ist ein klassischer Software/Engineering-Fehler. Da eine falsche Diagnose zu einem Bewegungsverbot ('Zug darf so nicht bewegt werden') führt, ist es ein Blocker."}]</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>[{"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}, {"fall_id": "57", "text": "Zwei Halterungen am Mülleimer in der Nasszelle WE2 fehlen. Werker hat vergessen sie anzunieten.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen sie anzunieten."}, "cot_begruendung": "Das Vergessen des Annietens durch den Werker ist ein klarer Montagefehler im Werk. Fehlende Halterungen am Mülleimer stoppen die Produktion nicht und sind als einfache Nacharbeit zu werten."}, {"fall_id": "44", "text": "Befestigung der Haltestange im FGR LWS lose. Werker hat vergessen, die Kontermutter anzubringen. Muss dringend nachgezogen werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, die Kontermutter anzubringen"}, "cot_begruendung": "Das explizite Vergessen der Kontermutter durch den Werker ist ein klassischer Montagefehler, der im eigenen Werk entstanden ist. Das Nachziehen der Mutter ist eine unkritische Nacharbeit."}]</t>
+          <t>[{"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"ursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}, {"fall_id": "169", "text": "Delle in der weißen Deckenverkleidung FGR RWS. IBS-Techniker ist beim Versuch, an den Rauchmelder zu kommen, mit seiner Alu-Leiter dagegen gestoßen.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "IBS-Techniker ist beim Versuch, an den Rauchmelder zu kommen, mit seiner Alu-Leiter dagegen gestoßen."}, "cot_begruendung": "Das Verursachen einer Delle durch Unachtsamkeit mit einer Leiter durch den internen IBS-Techniker ist ein Handhabungsfehler im Werk. Das optisch beschädigte Deckenelement muss ausgetauscht werden (Nacharbeit)."}, {"fall_id": "57", "text": "Zwei Halterungen am Mülleimer in der Nasszelle WE2 fehlen. Werker hat vergessen sie anzunieten.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen sie anzunieten."}, "cot_begruendung": "Das Vergessen des Annietens durch den Werker ist ein klarer Montagefehler im Werk. Fehlende Halterungen am Mülleimer stoppen die Produktion nicht und sind als einfache Nacharbeit zu werten."}]</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>[{"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}, {"fall_id": "44", "text": "Befestigung der Haltestange im FGR LWS lose. Werker hat vergessen, die Kontermutter anzubringen. Muss dringend nachgezogen werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, die Kontermutter anzubringen"}, "cot_begruendung": "Das explizite Vergessen der Kontermutter durch den Werker ist ein klassischer Montagefehler, der im eigenen Werk entstanden ist. Das Nachziehen der Mutter ist eine unkritische Nacharbeit."}, {"fall_id": "42", "text": "Zugsteuerung ZSG bootet nicht. Laut Herrn [Platzhalter] fehlt das gestrige Software-Patch für den CAN-Bus. Gesamte IBS steht aktuell.", "zielvariablen": {"grundursache": "Software", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "fehlt das gestrige Software-Patch für den CAN-Bus. Gesamte IBS steht aktuell"}, "cot_begruendung": "Ein fehlendes Software-Patch für ein Steuergerät, das zentral entwickelt wird, fällt in den Bereich Software/Engineering. Da die 'Gesamte IBS steht', ist der Fehler funktionskritisch und somit eindeutig ein Blocker."}]</t>
+          <t>[{"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"ursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}, {"fall_id": "197", "text": "Türen lassen sich nach der IBS nicht zentral schließen. Werker hat versehentlich die veraltete Tür-Software V1.0 von seinem lokalen USB-Stick geflasht, anstatt die freigegebene V1.2 vom Server zu ziehen. Alle Türen am Wagen müssen neu bespielt werden.", "zielvariablen": {"ursache": "Software", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker hat versehentlich die veraltete Tür-Software V1.0 von seinem lokalen USB-Stick geflasht"}, "cot_begruendung": "Das Aufspielen einer falschen/veralteten Software durch den Werker ist ein softwareseitiger und prozessualer Fehler, der direkt im Werk entstanden ist (Software/Werk). Da die sicherheitskritische zentrale Türschließung nicht funktioniert, ist die Inbetriebnahme hart blockiert."}, {"fall_id": "44", "text": "Befestigung der Haltestange im FGR LWS lose. Werker hat vergessen, die Kontermutter anzubringen. Muss dringend nachgezogen werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, die Kontermutter anzubringen"}, "cot_begruendung": "Das explizite Vergessen der Kontermutter durch den Werker ist ein klassischer Montagefehler, der im eigenen Werk entstanden ist. Das Nachziehen der Mutter ist eine unkritische Nacharbeit."}]</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "58", "text": "Lack zerkratzt.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Lack zerkratzt."}, "cot_begruendung": "Der Text beschreibt lediglich das Symptom 'Lack zerkratzt', liefert jedoch keinen Kontext zur Entstehung (z. B. Transport, unachtsamer Werker, Reinigung). Zur Vermeidung von Halluzinationen muss die Abstention-Logik angewandt und 'Unbekannt' ausgegeben werden."}]</t>
+          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "58", "text": "Lack zerkratzt.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Lack zerkratzt."}, "cot_begruendung": "Der Text beschreibt lediglich das Symptom 'Lack zerkratzt', liefert jedoch keinen Kontext zur Entstehung (z. B. Transport, unachtsamer Werker, Reinigung). Zur Vermeidung von Halluzinationen muss die Abstention-Logik angewandt und 'Unbekannt' ausgegeben werden."}]</t>
         </is>
       </c>
     </row>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>[{"fall_id": "42", "text": "Zugsteuerung ZSG bootet nicht. Laut Herrn [Platzhalter] fehlt das gestrige Software-Patch für den CAN-Bus. Gesamte IBS steht aktuell.", "zielvariablen": {"grundursache": "Software", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "fehlt das gestrige Software-Patch für den CAN-Bus. Gesamte IBS steht aktuell"}, "cot_begruendung": "Ein fehlendes Software-Patch für ein Steuergerät, das zentral entwickelt wird, fällt in den Bereich Software/Engineering. Da die 'Gesamte IBS steht', ist der Fehler funktionskritisch und somit eindeutig ein Blocker."}, {"fall_id": "26", "text": "Hauptkabelstrang HKS-3 unterflur am Drehgestell WE2 durchtrennt. Staplerfahrer hat beim Abladen der Palette reingestochen. Kabelbaum muss komplett neu.", "zielvariablen": {"grundursache": "Handhabung", "ursprung": "Logistik", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Staplerfahrer hat beim Abladen der Palette reingestochen"}, "cot_begruendung": "Der Text beschreibt eindeutig eine mechanische Beschädigung durch einen Staplerfahrer beim Abladen. Dies ist ein Handhabungsfehler, der der Logistik zuzuordnen ist. Da der Hauptkabelstrang komplett neu muss, kann das Fahrzeug elektrisch nicht in Betrieb genommen werden (Blocker)."}, {"fall_id": "31", "text": "DCU Tür 4 lässt sich nicht flashen. Falsches Skript auf dem Programmiergerät der IBS-Schichtleitung. Keine Tür am Wagen ansteuerbar.", "zielvariablen": {"grundursache": "Software", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Falsches Skript auf dem Programmiergerät der IBS-Schichtleitung. Keine Tür am Wagen ansteuerbar."}, "cot_begruendung": "Ein falsches Skript auf einem internen Programmiergerät ('IBS-Schichtleitung') ist ein lokaler Software/Prozessfehler im Werk. Da keine Tür am Wagen ansteuerbar ist, ist die Inbetriebnahme massiv gestört, was den Fehler als Blocker klassifiziert."}]</t>
+          <t>[{"fall_id": "197", "text": "Türen lassen sich nach der IBS nicht zentral schließen. Werker hat versehentlich die veraltete Tür-Software V1.0 von seinem lokalen USB-Stick geflasht, anstatt die freigegebene V1.2 vom Server zu ziehen. Alle Türen am Wagen müssen neu bespielt werden.", "zielvariablen": {"ursache": "Software", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker hat versehentlich die veraltete Tür-Software V1.0 von seinem lokalen USB-Stick geflasht"}, "cot_begruendung": "Das Aufspielen einer falschen/veralteten Software durch den Werker ist ein softwareseitiger und prozessualer Fehler, der direkt im Werk entstanden ist (Software/Werk). Da die sicherheitskritische zentrale Türschließung nicht funktioniert, ist die Inbetriebnahme hart blockiert."}, {"fall_id": "42", "text": "Zugsteuerung ZSG bootet nicht. Laut Herrn [Platzhalter] fehlt das gestrige Software-Patch für den CAN-Bus. Gesamte IBS steht aktuell.", "zielvariablen": {"ursache": "Software", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "fehlt das gestrige Software-Patch für den CAN-Bus. Gesamte IBS steht aktuell"}, "cot_begruendung": "Ein fehlendes Software-Patch für ein Steuergerät, das zentral entwickelt wird, fällt in den Bereich Software/Engineering. Da die 'Gesamte IBS steht', ist der Fehler funktionskritisch und somit eindeutig ein Blocker."}, {"fall_id": "179", "text": "Notbrems-Zugschalter im FGR LWS löst bei Betätigung nicht aus. Werker der Schicht 3 hat Pin 1 und Pin 2 am Stecker X4 vertauscht. Bremsschleife ist dadurch dauerhaft überbrückt. Lebensgefahr!", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker der Schicht 3 hat Pin 1 und Pin 2 am Stecker X4 vertauscht."}, "cot_begruendung": "Vertauschte Pins durch einen Werker der internen Schicht sind ein Montagefehler im Werk. Da eine defekte Notbremse ein sicherheitskritischer Mangel ist, der die Streckenzulassung unmöglich macht, wird dies als Blocker kategorisiert."}]</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>[{"fall_id": "8", "text": "Frontmaske hat matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend. Muss poliert/nachlackiert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend"}, "cot_begruendung": "Fehler beim Auftragen des Lacks ('Klarlack teilweise nicht deckend') weisen auf einen Verarbeitungs- bzw. Prozessfehler direkt in der Werksfertigung hin. Dies erfordert eine optische Nacharbeit, stellt aber keine funktionale Blockade dar."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "16", "text": "Klebereste von Schutzfolie an Fensterscheibe WE2 links. Wurde beim Abziehen nicht sauber gereinigt.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Wurde beim Abziehen nicht sauber gereinigt"}, "cot_begruendung": "Klebereste von Schutzfolien sind ein typischer Fehler aus der Endreinigung im Werk. Da der Fehler schnell behebbar ist und keine Bauteile beschädigt sind, wird er als 'Info' oder sehr leichte Nacharbeit eingestuft."}]</t>
+          <t>[{"fall_id": "8", "text": "Frontmaske hat matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend. Muss poliert/nachlackiert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend"}, "cot_begruendung": "Fehler beim Auftragen des Lacks ('Klarlack teilweise nicht deckend') weisen auf einen Verarbeitungs- bzw. Prozessfehler direkt in der Werksfertigung hin. Dies erfordert eine optische Nacharbeit, stellt aber keine funktionale Blockade dar."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "157", "text": "Palette mit Seitenverkleidungen ist beim Transport im Lager umgekippt, da sie nicht mit Folie gesichert war. Ecken der Paneele leicht eingedrückt, können aber vermutlich gerichtet werden.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "beim Transport im Lager umgekippt, da sie nicht mit Folie gesichert war."}, "cot_begruendung": "Das Umkippen einer ungesicherten Palette während des innerbetrieblichen Transports ist ein Handhabungsfehler der Logistik. Die leichten Beschädigungen können durch Richten behoben werden (Nacharbeit)."}]</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>[{"fall_id": "85", "text": "Haltegriffe an allen Sitzen im FGR falsch herum montiert. Schicht 3 hat die Einbauanleitung falsch verstanden. Müssen alle gedreht werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "an allen Sitzen im FGR falsch herum montiert. Schicht 3 hat die Einbauanleitung falsch verstanden."}, "cot_begruendung": "Ein Montagefehler durch eine interne Schicht, die die Anleitung falsch verstand, ist eindeutig Montage/Werk. Da 'alle Sitze' betroffen sind, handelt es sich um einen Serienfehler. Das Drehen der Griffe ist eine typische Nacharbeit."}, {"fall_id": "100", "text": "Schraube M8x20 an Haltestange im FGR WE2 rundgedreht. Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden."}, "cot_begruendung": "Das Runddrehen einer Schraube durch Nutzung eines falschen Bits durch den Werker ist ein Montagefehler im Werk. Das Ausbohren der defekten Schraube ist zeitintensiv, aber eine klassische Nacharbeit, die den Fertigungsablauf nicht komplett stoppt."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
+          <t>[{"fall_id": "106", "text": "Spaltmaß zwischen den Dachpaneelen im FGR RWS zu gering. Dehnungsausgleich nicht möglich. Laut 3D-Modell in Revision E ist das Paneel 5mm zu lang gezeichnet. QA sperrt den weiteren Deckenausbau.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Laut 3D-Modell in Revision E ist das Paneel 5mm zu lang gezeichnet. QA sperrt den weiteren Deckenausbau."}, "cot_begruendung": "Eine fehlerhafte Längenangabe im 3D-Modell verweist auf einen Konstruktionsfehler durch das Engineering. Die explizite Sperrung des weiteren Deckenausbaus durch die Qualitätsabteilung (QA) stuft dieses Problem als Blocker ein."}, {"fall_id": "85", "text": "Haltegriffe an allen Sitzen im FGR falsch herum montiert. Schicht 3 hat die Einbauanleitung falsch verstanden. Müssen alle gedreht werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "an allen Sitzen im FGR falsch herum montiert. Schicht 3 hat die Einbauanleitung falsch verstanden."}, "cot_begruendung": "Ein Montagefehler durch eine interne Schicht, die die Anleitung falsch verstand, ist eindeutig Montage/Werk. Da 'alle Sitze' betroffen sind, handelt es sich um einen Serienfehler. Das Drehen der Griffe ist eine typische Nacharbeit."}, {"fall_id": "100", "text": "Schraube M8x20 an Haltestange im FGR WE2 rundgedreht. Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden."}, "cot_begruendung": "Das Runddrehen einer Schraube durch Nutzung eines falschen Bits durch den Werker ist ein Montagefehler im Werk. Das Ausbohren der defekten Schraube ist zeitintensiv, aber eine klassische Nacharbeit, die den Fertigungsablauf nicht komplett stoppt."}]</t>
         </is>
       </c>
     </row>
@@ -3126,7 +3126,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>[{"fall_id": "38", "text": "Farbnebel auf Haltestange RWS im FGR. Wurde beim Lackieren der Wand nicht richtig abgeklebt.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Wurde beim Lackieren der Wand nicht richtig abgeklebt."}, "cot_begruendung": "Nicht richtiges Abkleben vor dem Lackieren ist ein Verarbeitungs- bzw. Prozessfehler, der direkt in der eigenen Werkstatt passiert ist. Der Farbnebel lässt sich meist einfach entfernen (Info/leichte Nacharbeit)."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "27", "text": "Scheibe RWS im FGR schmierig. Putzkolonne hat falsches Reinigungsmittel verwendet, Schlieren lassen sich schwer entfernen.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Putzkolonne hat falsches Reinigungsmittel verwendet"}, "cot_begruendung": "Die Verschmutzung wurde explizit durch die Putzkolonne ('falsches Reinigungsmittel') verursacht. Dies ist ein Reinigungsfehler im Werk. Da dies weder die Montage aufhält noch ein Bauteil zerstört, wird es als reine Nacharbeit/Info eingestuft."}]</t>
+          <t>[{"fall_id": "38", "text": "Farbnebel auf Haltestange RWS im FGR. Wurde beim Lackieren der Wand nicht richtig abgeklebt.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Wurde beim Lackieren der Wand nicht richtig abgeklebt."}, "cot_begruendung": "Nicht richtiges Abkleben vor dem Lackieren ist ein Verarbeitungs- bzw. Prozessfehler, der direkt in der eigenen Werkstatt passiert ist. Der Farbnebel lässt sich meist einfach entfernen (Info/leichte Nacharbeit)."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "27", "text": "Scheibe RWS im FGR schmierig. Putzkolonne hat falsches Reinigungsmittel verwendet, Schlieren lassen sich schwer entfernen.", "zielvariablen": {"ursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Putzkolonne hat falsches Reinigungsmittel verwendet"}, "cot_begruendung": "Die Verschmutzung wurde explizit durch die Putzkolonne ('falsches Reinigungsmittel') verursacht. Dies ist ein Reinigungsfehler im Werk. Da dies weder die Montage aufhält noch ein Bauteil zerstört, wird es als reine Nacharbeit/Info eingestuft."}]</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3201,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>[{"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "46", "text": "Großer Kratzer auf Trennglas im FGR. Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen"}, "cot_begruendung": "Die Beschädigung wurde direkt durch die Reinigungskraft beim Wischen verursacht (Reinigung/Werk). Ein zerkratztes Glas in der Trennwand muss getauscht werden (Nacharbeit), stoppt aber nicht die Produktion."}, {"fall_id": "27", "text": "Scheibe RWS im FGR schmierig. Putzkolonne hat falsches Reinigungsmittel verwendet, Schlieren lassen sich schwer entfernen.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Putzkolonne hat falsches Reinigungsmittel verwendet"}, "cot_begruendung": "Die Verschmutzung wurde explizit durch die Putzkolonne ('falsches Reinigungsmittel') verursacht. Dies ist ein Reinigungsfehler im Werk. Da dies weder die Montage aufhält noch ein Bauteil zerstört, wird es als reine Nacharbeit/Info eingestuft."}]</t>
+          <t>[{"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "46", "text": "Großer Kratzer auf Trennglas im FGR. Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen.", "zielvariablen": {"ursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen"}, "cot_begruendung": "Die Beschädigung wurde direkt durch die Reinigungskraft beim Wischen verursacht (Reinigung/Werk). Ein zerkratztes Glas in der Trennwand muss getauscht werden (Nacharbeit), stoppt aber nicht die Produktion."}, {"fall_id": "162", "text": "Graue Flecken auf dem neuen Fußbodenbelag im FGR. Reinigungskraft hat den Spezialreiniger nicht richtig verdünnt, wodurch Rückstände beim Trocknen entstanden sind. Einmal feucht nachwischen behebt das Problem.", "zielvariablen": {"ursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Reinigungskraft hat den Spezialreiniger nicht richtig verdünnt"}, "cot_begruendung": "Falsche Dosierung des Reinigungsmittels durch die Reinigungskraft ist ein klassischer Fehler der internen Reinigung (Werk). Da sich der Mangel durch simples Nachwischen beheben lässt, wird er als 'Info' oder sehr leichte Nacharbeit deklariert."}]</t>
         </is>
       </c>
     </row>
@@ -3276,7 +3276,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>[{"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "46", "text": "Großer Kratzer auf Trennglas im FGR. Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen"}, "cot_begruendung": "Die Beschädigung wurde direkt durch die Reinigungskraft beim Wischen verursacht (Reinigung/Werk). Ein zerkratztes Glas in der Trennwand muss getauscht werden (Nacharbeit), stoppt aber nicht die Produktion."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}]</t>
+          <t>[{"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "104", "text": "Wischwasserbehälter WE1 undicht. Schweißnaht am Kunststoffgehäuse hat Haarrisse. Offenbar Produktionsfehler vom Hersteller. Tropft auf die darunterliegende Elektrik. Sofortiger Tausch nötig.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Schweißnaht am Kunststoffgehäuse hat Haarrisse. Offenbar Produktionsfehler vom Hersteller."}, "cot_begruendung": "Ein undichter Behälter aufgrund von Haarrissen in der Schweißnaht ab Werk ist ein Materialfehler, der vom Hersteller (Lieferant) verursacht wurde. Da das Wasser auf die Elektrik tropft und ein sofortiger Tausch gefordert wird, liegt eine hohe Kritikalität (Blocker) vor."}, {"fall_id": "194", "text": "Massive Klarlacknasen am unteren Rand der Bugmaske WE2. Werker in der Lackierkabine hat die Spritzpistole zu nah gehalten und zu viel Lack aufgetragen. Muss komplett abgeschliffen und neu lackiert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker in der Lackierkabine hat die Spritzpistole zu nah gehalten und zu viel Lack aufgetragen."}, "cot_begruendung": "Falscher Umgang mit der Lackierpistole durch den Werker ist ein handwerklicher Verarbeitungsfehler im eigenen Werk. Abschleifen und Neulackieren ist zwar ärgerlich, aber eine reguläre Nacharbeit."}]</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>[{"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "4", "text": "Erdungsband am Triebdrehgestell WE1 links vergessen anzuschrauben. Schraube liegt lose auf dem Rahmen.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "vergessen anzuschrauben"}, "cot_begruendung": "Das vergessene Anschrauben ('Schraube liegt lose auf dem Rahmen') ist ein eindeutiger Montage- und Ausführungsfehler im Werk. Da eine fehlende Erdung am Triebdrehgestell ein massives Sicherheitsrisiko darstellt und die Inbetriebnahme verhindert, ist dies ein Blocker."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}]</t>
+          <t>[{"fall_id": "148", "text": "Sitzgestell wackelt.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Sitzgestell wackelt."}, "cot_begruendung": "Nur das Symptom 'wackelt' ist gegeben. Ob der Werker Schrauben vergessen hat, die Bohrungen falsch gesetzt sind oder das Gestell vom Lieferanten verzogen ist, ist nicht ersichtlich. Causal Faithfulness verlangt hier die Abstention (Unbekannt)."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "4", "text": "Erdungsband am Triebdrehgestell WE1 links vergessen anzuschrauben. Schraube liegt lose auf dem Rahmen.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "vergessen anzuschrauben"}, "cot_begruendung": "Das vergessene Anschrauben ('Schraube liegt lose auf dem Rahmen') ist ein eindeutiger Montage- und Ausführungsfehler im Werk. Da eine fehlende Erdung am Triebdrehgestell ein massives Sicherheitsrisiko darstellt und die Inbetriebnahme verhindert, ist dies ein Blocker."}]</t>
         </is>
       </c>
     </row>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>[{"fall_id": "30", "text": "Gummiprofil an Einstiegstür WE1 rissig. Betrifft Lieferung von ABC-Gummi der KW12 komplett. Material ist spröde.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Betrifft Lieferung von ABC-Gummi der KW12 komplett. Material ist spröde."}, "cot_begruendung": "Das spröde Gummiprofil ist auf eine fehlerhafte Materiallieferung von 'ABC-Gummi' zurückzuführen (Material/Lieferant). Der Hinweis 'Lieferung [...] komplett' markiert dies eindeutig als Serienfehler. Ein rissiges Gummi muss getauscht werden (Nacharbeit)."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "8", "text": "Frontmaske hat matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend. Muss poliert/nachlackiert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend"}, "cot_begruendung": "Fehler beim Auftragen des Lacks ('Klarlack teilweise nicht deckend') weisen auf einen Verarbeitungs- bzw. Prozessfehler direkt in der Werksfertigung hin. Dies erfordert eine optische Nacharbeit, stellt aber keine funktionale Blockade dar."}]</t>
+          <t>[{"fall_id": "30", "text": "Gummiprofil an Einstiegstür WE1 rissig. Betrifft Lieferung von ABC-Gummi der KW12 komplett. Material ist spröde.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Betrifft Lieferung von ABC-Gummi der KW12 komplett. Material ist spröde."}, "cot_begruendung": "Das spröde Gummiprofil ist auf eine fehlerhafte Materiallieferung von 'ABC-Gummi' zurückzuführen (Material/Lieferant). Der Hinweis 'Lieferung [...] komplett' markiert dies eindeutig als Serienfehler. Ein rissiges Gummi muss getauscht werden (Nacharbeit)."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "8", "text": "Frontmaske hat matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend. Muss poliert/nachlackiert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend"}, "cot_begruendung": "Fehler beim Auftragen des Lacks ('Klarlack teilweise nicht deckend') weisen auf einen Verarbeitungs- bzw. Prozessfehler direkt in der Werksfertigung hin. Dies erfordert eine optische Nacharbeit, stellt aber keine funktionale Blockade dar."}]</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>[{"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}]</t>
+          <t>[{"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}]</t>
         </is>
       </c>
     </row>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>[{"fall_id": "85", "text": "Haltegriffe an allen Sitzen im FGR falsch herum montiert. Schicht 3 hat die Einbauanleitung falsch verstanden. Müssen alle gedreht werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "an allen Sitzen im FGR falsch herum montiert. Schicht 3 hat die Einbauanleitung falsch verstanden."}, "cot_begruendung": "Ein Montagefehler durch eine interne Schicht, die die Anleitung falsch verstand, ist eindeutig Montage/Werk. Da 'alle Sitze' betroffen sind, handelt es sich um einen Serienfehler. Das Drehen der Griffe ist eine typische Nacharbeit."}, {"fall_id": "27", "text": "Scheibe RWS im FGR schmierig. Putzkolonne hat falsches Reinigungsmittel verwendet, Schlieren lassen sich schwer entfernen.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Putzkolonne hat falsches Reinigungsmittel verwendet"}, "cot_begruendung": "Die Verschmutzung wurde explizit durch die Putzkolonne ('falsches Reinigungsmittel') verursacht. Dies ist ein Reinigungsfehler im Werk. Da dies weder die Montage aufhält noch ein Bauteil zerstört, wird es als reine Nacharbeit/Info eingestuft."}, {"fall_id": "53", "text": "FIS-Displays für den FGR kamen mit gesprungenen Scheiben an. Betrifft Palette 1 bis 4. Transportsicherung des Spediteurs war gerissen.", "zielvariablen": {"grundursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Betrifft Palette 1 bis 4. Transportsicherung des Spediteurs war gerissen."}, "cot_begruendung": "Gerissene Transportsicherungen des Spediteurs verweisen auf einen Transportschaden (Logistik). Da gleich 4 Paletten ('Palette 1 bis 4') betroffen sind, liegt ein klarer Serienfehler vor. Die Displays müssen nachgearbeitet/ersetzt werden."}]</t>
+          <t>[{"fall_id": "106", "text": "Spaltmaß zwischen den Dachpaneelen im FGR RWS zu gering. Dehnungsausgleich nicht möglich. Laut 3D-Modell in Revision E ist das Paneel 5mm zu lang gezeichnet. QA sperrt den weiteren Deckenausbau.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Laut 3D-Modell in Revision E ist das Paneel 5mm zu lang gezeichnet. QA sperrt den weiteren Deckenausbau."}, "cot_begruendung": "Eine fehlerhafte Längenangabe im 3D-Modell verweist auf einen Konstruktionsfehler durch das Engineering. Die explizite Sperrung des weiteren Deckenausbaus durch die Qualitätsabteilung (QA) stuft dieses Problem als Blocker ein."}, {"fall_id": "85", "text": "Haltegriffe an allen Sitzen im FGR falsch herum montiert. Schicht 3 hat die Einbauanleitung falsch verstanden. Müssen alle gedreht werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "an allen Sitzen im FGR falsch herum montiert. Schicht 3 hat die Einbauanleitung falsch verstanden."}, "cot_begruendung": "Ein Montagefehler durch eine interne Schicht, die die Anleitung falsch verstand, ist eindeutig Montage/Werk. Da 'alle Sitze' betroffen sind, handelt es sich um einen Serienfehler. Das Drehen der Griffe ist eine typische Nacharbeit."}, {"fall_id": "27", "text": "Scheibe RWS im FGR schmierig. Putzkolonne hat falsches Reinigungsmittel verwendet, Schlieren lassen sich schwer entfernen.", "zielvariablen": {"ursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Putzkolonne hat falsches Reinigungsmittel verwendet"}, "cot_begruendung": "Die Verschmutzung wurde explizit durch die Putzkolonne ('falsches Reinigungsmittel') verursacht. Dies ist ein Reinigungsfehler im Werk. Da dies weder die Montage aufhält noch ein Bauteil zerstört, wird es als reine Nacharbeit/Info eingestuft."}]</t>
         </is>
       </c>
     </row>
@@ -3651,7 +3651,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>[{"fall_id": "85", "text": "Haltegriffe an allen Sitzen im FGR falsch herum montiert. Schicht 3 hat die Einbauanleitung falsch verstanden. Müssen alle gedreht werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "an allen Sitzen im FGR falsch herum montiert. Schicht 3 hat die Einbauanleitung falsch verstanden."}, "cot_begruendung": "Ein Montagefehler durch eine interne Schicht, die die Anleitung falsch verstand, ist eindeutig Montage/Werk. Da 'alle Sitze' betroffen sind, handelt es sich um einen Serienfehler. Das Drehen der Griffe ist eine typische Nacharbeit."}, {"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}, {"fall_id": "53", "text": "FIS-Displays für den FGR kamen mit gesprungenen Scheiben an. Betrifft Palette 1 bis 4. Transportsicherung des Spediteurs war gerissen.", "zielvariablen": {"grundursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Betrifft Palette 1 bis 4. Transportsicherung des Spediteurs war gerissen."}, "cot_begruendung": "Gerissene Transportsicherungen des Spediteurs verweisen auf einen Transportschaden (Logistik). Da gleich 4 Paletten ('Palette 1 bis 4') betroffen sind, liegt ein klarer Serienfehler vor. Die Displays müssen nachgearbeitet/ersetzt werden."}]</t>
+          <t>[{"fall_id": "179", "text": "Notbrems-Zugschalter im FGR LWS löst bei Betätigung nicht aus. Werker der Schicht 3 hat Pin 1 und Pin 2 am Stecker X4 vertauscht. Bremsschleife ist dadurch dauerhaft überbrückt. Lebensgefahr!", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker der Schicht 3 hat Pin 1 und Pin 2 am Stecker X4 vertauscht."}, "cot_begruendung": "Vertauschte Pins durch einen Werker der internen Schicht sind ein Montagefehler im Werk. Da eine defekte Notbremse ein sicherheitskritischer Mangel ist, der die Streckenzulassung unmöglich macht, wird dies als Blocker kategorisiert."}, {"fall_id": "85", "text": "Haltegriffe an allen Sitzen im FGR falsch herum montiert. Schicht 3 hat die Einbauanleitung falsch verstanden. Müssen alle gedreht werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "an allen Sitzen im FGR falsch herum montiert. Schicht 3 hat die Einbauanleitung falsch verstanden."}, "cot_begruendung": "Ein Montagefehler durch eine interne Schicht, die die Anleitung falsch verstand, ist eindeutig Montage/Werk. Da 'alle Sitze' betroffen sind, handelt es sich um einen Serienfehler. Das Drehen der Griffe ist eine typische Nacharbeit."}, {"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}]</t>
         </is>
       </c>
     </row>
@@ -3726,7 +3726,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>[{"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}]</t>
+          <t>[{"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "109", "text": "Isolationsmatte hinter Türvoute LWS falsch zugeschnitten. Werker hat statt der Schablone B die Schablone A verwendet. Matte deckt den Kältebereich nicht vollständig ab.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat statt der Schablone B die Schablone A verwendet."}, "cot_begruendung": "Die Verwendung einer falschen Schablone durch den internen Werker beim Zuschnitt ist ein Verarbeitungs- bzw. Montagefehler im Werk. Die falsche Matte muss entfernt und durch eine korrekt zugeschnittene ersetzt werden (Nacharbeit)."}]</t>
         </is>
       </c>
     </row>
@@ -3801,7 +3801,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>[{"fall_id": "30", "text": "Gummiprofil an Einstiegstür WE1 rissig. Betrifft Lieferung von ABC-Gummi der KW12 komplett. Material ist spröde.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Betrifft Lieferung von ABC-Gummi der KW12 komplett. Material ist spröde."}, "cot_begruendung": "Das spröde Gummiprofil ist auf eine fehlerhafte Materiallieferung von 'ABC-Gummi' zurückzuführen (Material/Lieferant). Der Hinweis 'Lieferung [...] komplett' markiert dies eindeutig als Serienfehler. Ein rissiges Gummi muss getauscht werden (Nacharbeit)."}, {"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}]</t>
+          <t>[{"fall_id": "101", "text": "Klemmschutz an Fahrgasttür 3 LWS löst viel zu früh aus. Schließvorgang bricht bei leichtem Windstoß ab. Sensorik-Parameter in der neuen Türsoftware (V1.4) von Fa. [Platzhalter] sind zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte angefordert.", "zielvariablen": {"ursache": "Software", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Sensorik-Parameter in der neuen Türsoftware [...] zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte"}, "cot_begruendung": "Der Text beschreibt ein funktionales Problem der Fahrgasttür aufgrund zu empfindlicher Parameter in der 'neuen Türsoftware', welche von einem externen Lieferanten stammt. Da die 'gesamte Flotte' ein Update benötigt, handelt es sich um einen Serienfehler. Ein fehlerhafter Klemmschutz betrifft die Sicherheit und Zuverlässigkeit der Türen, was die Inbetriebnahme blockiert."}, {"fall_id": "30", "text": "Gummiprofil an Einstiegstür WE1 rissig. Betrifft Lieferung von ABC-Gummi der KW12 komplett. Material ist spröde.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Betrifft Lieferung von ABC-Gummi der KW12 komplett. Material ist spröde."}, "cot_begruendung": "Das spröde Gummiprofil ist auf eine fehlerhafte Materiallieferung von 'ABC-Gummi' zurückzuführen (Material/Lieferant). Der Hinweis 'Lieferung [...] komplett' markiert dies eindeutig als Serienfehler. Ein rissiges Gummi muss getauscht werden (Nacharbeit)."}, {"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}]</t>
         </is>
       </c>
     </row>
@@ -3876,7 +3876,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>[{"fall_id": "27", "text": "Scheibe RWS im FGR schmierig. Putzkolonne hat falsches Reinigungsmittel verwendet, Schlieren lassen sich schwer entfernen.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Putzkolonne hat falsches Reinigungsmittel verwendet"}, "cot_begruendung": "Die Verschmutzung wurde explizit durch die Putzkolonne ('falsches Reinigungsmittel') verursacht. Dies ist ein Reinigungsfehler im Werk. Da dies weder die Montage aufhält noch ein Bauteil zerstört, wird es als reine Nacharbeit/Info eingestuft."}, {"fall_id": "76", "text": "Türen LWS öffnen sich, wenn Taster für RWS gedrückt wird. Software-Mapping in der DCU vom Engineering komplett vertauscht. Gefahr für Leib und Leben, IBS abgebrochen.", "zielvariablen": {"grundursache": "Software", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Software-Mapping in der DCU vom Engineering komplett vertauscht. Gefahr für Leib und Leben, IBS abgebrochen."}, "cot_begruendung": "Vertauschtes Software-Mapping durch das Engineering ist ein Software/Konstruktions-Fehler. Ein sicherheitskritisches Türproblem mit Abbruch der IBS ist der Inbegriff eines harten Blockers."}, {"fall_id": "46", "text": "Großer Kratzer auf Trennglas im FGR. Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen"}, "cot_begruendung": "Die Beschädigung wurde direkt durch die Reinigungskraft beim Wischen verursacht (Reinigung/Werk). Ein zerkratztes Glas in der Trennwand muss getauscht werden (Nacharbeit), stoppt aber nicht die Produktion."}]</t>
+          <t>[{"fall_id": "27", "text": "Scheibe RWS im FGR schmierig. Putzkolonne hat falsches Reinigungsmittel verwendet, Schlieren lassen sich schwer entfernen.", "zielvariablen": {"ursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Putzkolonne hat falsches Reinigungsmittel verwendet"}, "cot_begruendung": "Die Verschmutzung wurde explizit durch die Putzkolonne ('falsches Reinigungsmittel') verursacht. Dies ist ein Reinigungsfehler im Werk. Da dies weder die Montage aufhält noch ein Bauteil zerstört, wird es als reine Nacharbeit/Info eingestuft."}, {"fall_id": "117", "text": "Befestigung der Sitzkiste RWS im FGR wackelt. Werker hat statt der M8x25 eine M8x40 Schraube mit Gewalt reingedreht und das Gewinde im Boden zerstört. Gewindeeinsatz muss neu gesetzt werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat statt der M8x25 eine M8x40 Schraube mit Gewalt reingedreht"}, "cot_begruendung": "Die Zerstörung des Gewindes durch den Werker (falsche Schraube, Gewaltanwendung) ist ein klarer Montage- und Handhabungsfehler im eigenen Werk. Die Reparatur des Gewindes ist zwar aufwendig, stellt aber einen lokalen Eingriff dar (Nacharbeit)."}, {"fall_id": "106", "text": "Spaltmaß zwischen den Dachpaneelen im FGR RWS zu gering. Dehnungsausgleich nicht möglich. Laut 3D-Modell in Revision E ist das Paneel 5mm zu lang gezeichnet. QA sperrt den weiteren Deckenausbau.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Laut 3D-Modell in Revision E ist das Paneel 5mm zu lang gezeichnet. QA sperrt den weiteren Deckenausbau."}, "cot_begruendung": "Eine fehlerhafte Längenangabe im 3D-Modell verweist auf einen Konstruktionsfehler durch das Engineering. Die explizite Sperrung des weiteren Deckenausbaus durch die Qualitätsabteilung (QA) stuft dieses Problem als Blocker ein."}]</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "4", "text": "Erdungsband am Triebdrehgestell WE1 links vergessen anzuschrauben. Schraube liegt lose auf dem Rahmen.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "vergessen anzuschrauben"}, "cot_begruendung": "Das vergessene Anschrauben ('Schraube liegt lose auf dem Rahmen') ist ein eindeutiger Montage- und Ausführungsfehler im Werk. Da eine fehlende Erdung am Triebdrehgestell ein massives Sicherheitsrisiko darstellt und die Inbetriebnahme verhindert, ist dies ein Blocker."}, {"fall_id": "2", "text": "Seitenwandverkleidung RWS im Einstiegsbereich weist tiefe Kratzer auf. Betrifft die letzten 5 angelieferten Wagen. Falsche Stapelung in Transportbox durch Spedition.", "zielvariablen": {"grundursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Betrifft die letzten 5 angelieferten Wagen. Falsche Stapelung in Transportbox"}, "cot_begruendung": "Der Schaden entstand explizit durch 'Falsche Stapelung in Transportbox' durch die Spedition, woraus sich Transport/Logistik als Verursacher ableiten lässt. Der Hinweis 'letzten 5 angelieferten Wagen' ist ein klarer Indikator für einen Serienfehler. Der Kratzer muss nachgearbeitet werden, stoppt aber nicht sofort die gesamte Produktion."}]</t>
+          <t>[{"fall_id": "135", "text": "Alle Haltegriffe an der Decke im Wagen 5 sind um 180 Grad verdreht montiert. Die Piktogramme stehen auf dem Kopf. Montage-Crew hat die Zeichnung falsch gelesen.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Alle Haltegriffe [...] Montage-Crew hat die Zeichnung falsch gelesen."}, "cot_begruendung": "Die interne Montage-Crew hat die Zeichnung falsch interpretiert, was einen klaren Montagefehler im Werk darstellt. Da 'Alle Haltegriffe' im Wagen betroffen sind, liegt ein Serienfehler vor. Die Griffe müssen demontiert und richtig herum angeschraubt werden (Nacharbeit)."}, {"fall_id": "106", "text": "Spaltmaß zwischen den Dachpaneelen im FGR RWS zu gering. Dehnungsausgleich nicht möglich. Laut 3D-Modell in Revision E ist das Paneel 5mm zu lang gezeichnet. QA sperrt den weiteren Deckenausbau.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Laut 3D-Modell in Revision E ist das Paneel 5mm zu lang gezeichnet. QA sperrt den weiteren Deckenausbau."}, "cot_begruendung": "Eine fehlerhafte Längenangabe im 3D-Modell verweist auf einen Konstruktionsfehler durch das Engineering. Die explizite Sperrung des weiteren Deckenausbaus durch die Qualitätsabteilung (QA) stuft dieses Problem als Blocker ein."}, {"fall_id": "152", "text": "Abdeckbleche für die Heizkanäle LWS aus unserer eigenen Stanzerei sind an der Kante um 10 Grad zu wenig abgekantet. Betrifft alle 40 Bleche von heute. Können so nicht montiert werden, Kante steht ab.", "zielvariablen": {"ursache": "Fertigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "aus unserer eigenen Stanzerei sind an der Kante um 10 Grad zu wenig abgekantet. Betrifft alle 40 Bleche"}, "cot_begruendung": "Ein Biegefehler aus der 'eigenen Stanzerei' ist ein interner Fertigungsfehler (Werk). Da 'alle 40 Bleche von heute' betroffen sind, liegt ein Serienfehler vor. Die Bleche müssen nachgebogen werden (Nacharbeit), stoppen aber nicht den kompletten Wagenausbau."}]</t>
         </is>
       </c>
     </row>
@@ -4026,7 +4026,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>[{"fall_id": "26", "text": "Hauptkabelstrang HKS-3 unterflur am Drehgestell WE2 durchtrennt. Staplerfahrer hat beim Abladen der Palette reingestochen. Kabelbaum muss komplett neu.", "zielvariablen": {"grundursache": "Handhabung", "ursprung": "Logistik", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Staplerfahrer hat beim Abladen der Palette reingestochen"}, "cot_begruendung": "Der Text beschreibt eindeutig eine mechanische Beschädigung durch einen Staplerfahrer beim Abladen. Dies ist ein Handhabungsfehler, der der Logistik zuzuordnen ist. Da der Hauptkabelstrang komplett neu muss, kann das Fahrzeug elektrisch nicht in Betrieb genommen werden (Blocker)."}, {"fall_id": "4", "text": "Erdungsband am Triebdrehgestell WE1 links vergessen anzuschrauben. Schraube liegt lose auf dem Rahmen.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "vergessen anzuschrauben"}, "cot_begruendung": "Das vergessene Anschrauben ('Schraube liegt lose auf dem Rahmen') ist ein eindeutiger Montage- und Ausführungsfehler im Werk. Da eine fehlende Erdung am Triebdrehgestell ein massives Sicherheitsrisiko darstellt und die Inbetriebnahme verhindert, ist dies ein Blocker."}, {"fall_id": "82", "text": "Tiefer Kratzer auf dem Führerpult. IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen.", "zielvariablen": {"grundursache": "Handhabung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen."}, "cot_begruendung": "Das Fallenlassen des Laptops durch den Mitarbeiter ist ein Handhabungsfehler im eigenen Werk. Optische Kratzer erfordern Nacharbeit (Austausch oder Politur)."}]</t>
+          <t>[{"fall_id": "26", "text": "Hauptkabelstrang HKS-3 unterflur am Drehgestell WE2 durchtrennt. Staplerfahrer hat beim Abladen der Palette reingestochen. Kabelbaum muss komplett neu.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Logistik", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Staplerfahrer hat beim Abladen der Palette reingestochen"}, "cot_begruendung": "Der Text beschreibt eindeutig eine mechanische Beschädigung durch einen Staplerfahrer beim Abladen. Dies ist ein Handhabungsfehler, der der Logistik zuzuordnen ist. Da der Hauptkabelstrang komplett neu muss, kann das Fahrzeug elektrisch nicht in Betrieb genommen werden (Blocker)."}, {"fall_id": "4", "text": "Erdungsband am Triebdrehgestell WE1 links vergessen anzuschrauben. Schraube liegt lose auf dem Rahmen.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "vergessen anzuschrauben"}, "cot_begruendung": "Das vergessene Anschrauben ('Schraube liegt lose auf dem Rahmen') ist ein eindeutiger Montage- und Ausführungsfehler im Werk. Da eine fehlende Erdung am Triebdrehgestell ein massives Sicherheitsrisiko darstellt und die Inbetriebnahme verhindert, ist dies ein Blocker."}, {"fall_id": "82", "text": "Tiefer Kratzer auf dem Führerpult. IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen."}, "cot_begruendung": "Das Fallenlassen des Laptops durch den Mitarbeiter ist ein Handhabungsfehler im eigenen Werk. Optische Kratzer erfordern Nacharbeit (Austausch oder Politur)."}]</t>
         </is>
       </c>
     </row>
@@ -4101,7 +4101,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>[{"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "44", "text": "Befestigung der Haltestange im FGR LWS lose. Werker hat vergessen, die Kontermutter anzubringen. Muss dringend nachgezogen werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, die Kontermutter anzubringen"}, "cot_begruendung": "Das explizite Vergessen der Kontermutter durch den Werker ist ein klassischer Montagefehler, der im eigenen Werk entstanden ist. Das Nachziehen der Mutter ist eine unkritische Nacharbeit."}]</t>
+          <t>[{"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "44", "text": "Befestigung der Haltestange im FGR LWS lose. Werker hat vergessen, die Kontermutter anzubringen. Muss dringend nachgezogen werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, die Kontermutter anzubringen"}, "cot_begruendung": "Das explizite Vergessen der Kontermutter durch den Werker ist ein klassischer Montagefehler, der im eigenen Werk entstanden ist. Das Nachziehen der Mutter ist eine unkritische Nacharbeit."}]</t>
         </is>
       </c>
     </row>
@@ -4176,7 +4176,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>[{"fall_id": "4", "text": "Erdungsband am Triebdrehgestell WE1 links vergessen anzuschrauben. Schraube liegt lose auf dem Rahmen.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "vergessen anzuschrauben"}, "cot_begruendung": "Das vergessene Anschrauben ('Schraube liegt lose auf dem Rahmen') ist ein eindeutiger Montage- und Ausführungsfehler im Werk. Da eine fehlende Erdung am Triebdrehgestell ein massives Sicherheitsrisiko darstellt und die Inbetriebnahme verhindert, ist dies ein Blocker."}, {"fall_id": "14", "text": "Notbremsschleife falsch gepinnt an Stecker X12 im Fahrerpult. Pin 3 und Pin 5 vertauscht, Funktion nicht gegeben. Fehler bei Verkabelung durch Schicht 2.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Fehler bei Verkabelung durch Schicht 2"}, "cot_begruendung": "Die falsch gepinnte Notbremsschleife wurde explizit durch eine interne Schicht ('Verkabelung durch Schicht 2') verursacht, was Montage/Werk als Ursprung festlegt. Da die Notbremse eine sicherheitskritische Funktion ist und nicht funktioniert, handelt es sich um einen Blocker."}, {"fall_id": "100", "text": "Schraube M8x20 an Haltestange im FGR WE2 rundgedreht. Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden."}, "cot_begruendung": "Das Runddrehen einer Schraube durch Nutzung eines falschen Bits durch den Werker ist ein Montagefehler im Werk. Das Ausbohren der defekten Schraube ist zeitintensiv, aber eine klassische Nacharbeit, die den Fertigungsablauf nicht komplett stoppt."}]</t>
+          <t>[{"fall_id": "4", "text": "Erdungsband am Triebdrehgestell WE1 links vergessen anzuschrauben. Schraube liegt lose auf dem Rahmen.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "vergessen anzuschrauben"}, "cot_begruendung": "Das vergessene Anschrauben ('Schraube liegt lose auf dem Rahmen') ist ein eindeutiger Montage- und Ausführungsfehler im Werk. Da eine fehlende Erdung am Triebdrehgestell ein massives Sicherheitsrisiko darstellt und die Inbetriebnahme verhindert, ist dies ein Blocker."}, {"fall_id": "14", "text": "Notbremsschleife falsch gepinnt an Stecker X12 im Fahrerpult. Pin 3 und Pin 5 vertauscht, Funktion nicht gegeben. Fehler bei Verkabelung durch Schicht 2.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Fehler bei Verkabelung durch Schicht 2"}, "cot_begruendung": "Die falsch gepinnte Notbremsschleife wurde explizit durch eine interne Schicht ('Verkabelung durch Schicht 2') verursacht, was Montage/Werk als Ursprung festlegt. Da die Notbremse eine sicherheitskritische Funktion ist und nicht funktioniert, handelt es sich um einen Blocker."}, {"fall_id": "100", "text": "Schraube M8x20 an Haltestange im FGR WE2 rundgedreht. Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden."}, "cot_begruendung": "Das Runddrehen einer Schraube durch Nutzung eines falschen Bits durch den Werker ist ein Montagefehler im Werk. Das Ausbohren der defekten Schraube ist zeitintensiv, aber eine klassische Nacharbeit, die den Fertigungsablauf nicht komplett stoppt."}]</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "58", "text": "Lack zerkratzt.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Lack zerkratzt."}, "cot_begruendung": "Der Text beschreibt lediglich das Symptom 'Lack zerkratzt', liefert jedoch keinen Kontext zur Entstehung (z. B. Transport, unachtsamer Werker, Reinigung). Zur Vermeidung von Halluzinationen muss die Abstention-Logik angewandt und 'Unbekannt' ausgegeben werden."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
+          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "58", "text": "Lack zerkratzt.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Lack zerkratzt."}, "cot_begruendung": "Der Text beschreibt lediglich das Symptom 'Lack zerkratzt', liefert jedoch keinen Kontext zur Entstehung (z. B. Transport, unachtsamer Werker, Reinigung). Zur Vermeidung von Halluzinationen muss die Abstention-Logik angewandt und 'Unbekannt' ausgegeben werden."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
         </is>
       </c>
     </row>
@@ -4326,7 +4326,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>[{"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "70", "text": "Anschlusskabel für Notbremsschalter im FGR zu kurz geschnitten. Werker hat den Kabelstrang nicht wie vorgeschrieben in Schleife gelegt, sondern direkt gezogen. Neuverkabelung der halben Seite LWS nötig.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker hat den Kabelstrang nicht wie vorgeschrieben in Schleife gelegt, sondern direkt gezogen. Neuverkabelung der halben Seite LWS nötig."}, "cot_begruendung": "Der Werker hat den Kabelstrang falsch verlegt (nicht in Schleife), was einen Montagefehler im Werk darstellt. Da sicherheitsrelevante Notbremsschalter betroffen sind und die halbe Seite neu verkabelt werden muss, ist dies ein massiver Verzug und somit ein Blocker."}, {"fall_id": "62", "text": "Kabelkanal unterflur kollidiert mit der Druckluftleitung für die Bremsanlage. Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich."}, "cot_begruendung": "Eine Überlappung im 3D-Modell/Zeichnung ist ein Konstruktionsfehler aus dem Engineering. Da die Druckluftleitung für die Bremsen essenziell ist und die 'Rohrverlegung aktuell unmöglich' ist, handelt es sich um einen harten Blocker."}]</t>
+          <t>[{"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "70", "text": "Anschlusskabel für Notbremsschalter im FGR zu kurz geschnitten. Werker hat den Kabelstrang nicht wie vorgeschrieben in Schleife gelegt, sondern direkt gezogen. Neuverkabelung der halben Seite LWS nötig.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker hat den Kabelstrang nicht wie vorgeschrieben in Schleife gelegt, sondern direkt gezogen. Neuverkabelung der halben Seite LWS nötig."}, "cot_begruendung": "Der Werker hat den Kabelstrang falsch verlegt (nicht in Schleife), was einen Montagefehler im Werk darstellt. Da sicherheitsrelevante Notbremsschalter betroffen sind und die halbe Seite neu verkabelt werden muss, ist dies ein massiver Verzug und somit ein Blocker."}, {"fall_id": "62", "text": "Kabelkanal unterflur kollidiert mit der Druckluftleitung für die Bremsanlage. Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich."}, "cot_begruendung": "Eine Überlappung im 3D-Modell/Zeichnung ist ein Konstruktionsfehler aus dem Engineering. Da die Druckluftleitung für die Bremsen essenziell ist und die 'Rohrverlegung aktuell unmöglich' ist, handelt es sich um einen harten Blocker."}]</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4401,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>[{"fall_id": "79", "text": "Sitzbezüge im gesamten Wagen reißen an der Naht ein. Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge müssen getauscht werden.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge"}, "cot_begruendung": "Die mangelhafte Stoffqualität eines externen Lieferanten ist ein Materialfehler. Die Bemerkungen 'gesamter Wagen' und 'neuen Serie' verweisen auf einen Serienfehler. Das Austauschen der Bezüge ist Nacharbeit, aber kein Blocker für Inbetriebsetzungen."}, {"fall_id": "22", "text": "Fahrgasttür RWS öffnet nicht bei Tasterbetätigung. DCU gibt keinen Befehl raus. Ersatzteil aus Lager geholt, Tür funktioniert wieder. Defekte DCU geht an Lieferant retour.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "DCU gibt keinen Befehl raus. [...] Defekte DCU geht an Lieferant retour"}, "cot_begruendung": "Die Door Control Unit (DCU) ist intern defekt, was auf einen Materialfehler des Lieferanten schließen lässt. Da das Ersatzteil sofort aus dem Lager verfügbar war und die Produktion nicht gestoppt wurde, bleibt es bei einer Nacharbeit."}, {"fall_id": "44", "text": "Befestigung der Haltestange im FGR LWS lose. Werker hat vergessen, die Kontermutter anzubringen. Muss dringend nachgezogen werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, die Kontermutter anzubringen"}, "cot_begruendung": "Das explizite Vergessen der Kontermutter durch den Werker ist ein klassischer Montagefehler, der im eigenen Werk entstanden ist. Das Nachziehen der Mutter ist eine unkritische Nacharbeit."}]</t>
+          <t>[{"fall_id": "79", "text": "Sitzbezüge im gesamten Wagen reißen an der Naht ein. Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge müssen getauscht werden.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge"}, "cot_begruendung": "Die mangelhafte Stoffqualität eines externen Lieferanten ist ein Materialfehler. Die Bemerkungen 'gesamter Wagen' und 'neuen Serie' verweisen auf einen Serienfehler. Das Austauschen der Bezüge ist Nacharbeit, aber kein Blocker für Inbetriebsetzungen."}, {"fall_id": "22", "text": "Fahrgasttür RWS öffnet nicht bei Tasterbetätigung. DCU gibt keinen Befehl raus. Ersatzteil aus Lager geholt, Tür funktioniert wieder. Defekte DCU geht an Lieferant retour.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "DCU gibt keinen Befehl raus. [...] Defekte DCU geht an Lieferant retour"}, "cot_begruendung": "Die Door Control Unit (DCU) ist intern defekt, was auf einen Materialfehler des Lieferanten schließen lässt. Da das Ersatzteil sofort aus dem Lager verfügbar war und die Produktion nicht gestoppt wurde, bleibt es bei einer Nacharbeit."}, {"fall_id": "126", "text": "Alle C-Schienen zur Befestigung der Sitze aus unserer internen Fräserei sind um 5mm zu schmal gefräst worden. Maß in der Maschine war falsch eingestellt. Keine Sitze im Wagen 3 montierbar.", "zielvariablen": {"ursache": "Fertigung", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "aus unserer internen Fräserei sind um 5mm zu schmal gefräst worden. Maß in der Maschine war falsch eingestellt."}, "cot_begruendung": "Falsch gefräste Bauteile aus der 'internen Fräserei' aufgrund einer falsch eingestellten Maschine sind ein Fertigungsfehler im Werk. Da 'Alle C-Schienen' betroffen sind, ist es ein Serienproblem. Dass keine Sitze verbaut werden können, zieht einen Produktionsstopp nach sich (Blocker)."}]</t>
         </is>
       </c>
     </row>
@@ -4476,7 +4476,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>[{"fall_id": "69", "text": "HVAC-Einheit für WE2 mit tiefen Kratzern und verbogenen Lamellen angeliefert worden. Verpackung war aufgerissen. Eindeutiger Handhabungsschaden durch Zulieferer Fa. [Platzhalter] vor Versand.", "zielvariablen": {"grundursache": "Handhabung", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Eindeutiger Handhabungsschaden durch Zulieferer Fa. [Platzhalter] vor Versand."}, "cot_begruendung": "Der Schaden wird explizit als Handhabungsfehler durch den externen Zulieferer vor dem Versand identifiziert (Handhabung/Lieferant). Verborgene Lamellen erfordern eine Nacharbeit, stoppen aber die generelle Produktion des Wagens meist nicht sofort."}, {"fall_id": "54", "text": "Kühlleistung HVAC 2 ungenügend. Prüfung ergab, dass Lieferant ABC versehentlich das falsche Kältemittel eingefüllt hat. Muss abgesaugt und neu befüllt werden.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Lieferant ABC versehentlich das falsche Kältemittel eingefüllt"}, "cot_begruendung": "Das falsche Kältemittel wurde explizit vom Lieferanten eingefüllt, was als Materialfehler des Lieferanten gewertet wird. Die Absaugung und Neubefüllung ist eine aufwendige, aber standardisierbare Nacharbeit, die nicht den gesamten Wagenbau stoppt."}, {"fall_id": "13", "text": "Hauptschalter am Dach WE1 löst bei 100A aus, Spezifikation fordert 150A. Alle Schalter der aktuellen Charge von Fa. [Platzhalter] sind betroffen. IBS kann nicht fortgesetzt werden.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Alle Schalter der aktuellen Charge von Fa. [Platzhalter] sind betroffen"}, "cot_begruendung": "Das Bauteil erfüllt nicht die geforderte Spezifikation, was auf einen Materialfehler des externen Lieferanten ('Fa. [Platzhalter]') hinweist. Da die IBS (Inbetriebsetzung) nicht fortgesetzt werden kann, ist dies ein harter Blocker. Der Hinweis 'Alle Schalter der aktuellen Charge' markiert es klar als Serienfehler."}]</t>
+          <t>[{"fall_id": "136", "text": "Kühlmittelleitung der HVAC kollidiert mit dem Kabelkanal RWS am Dach. Laut DMU-Modell Version 4.1 gibt es hier keine Überlappung, in der Realität fehlen jedoch 15mm Freigang. Das Rohr-Routing muss vom EN dringend überarbeitet werden. Deckenausbau gestoppt.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Laut DMU-Modell Version 4.1 gibt es hier keine Überlappung [...] Das Rohr-Routing muss vom EN dringend überarbeitet werden."}, "cot_begruendung": "Eine Diskrepanz zwischen dem 3D-Modell (DMU) und der Realität, die eine Änderung des Routings durch das Engineering (EN) erfordert, ist ein Konstruktionsfehler. Die Kollision verhindert den weiteren Ausbau ('Deckenausbau gestoppt'), was den Fehler als Blocker einstuft."}, {"fall_id": "69", "text": "HVAC-Einheit für WE2 mit tiefen Kratzern und verbogenen Lamellen angeliefert worden. Verpackung war aufgerissen. Eindeutiger Handhabungsschaden durch Zulieferer Fa. [Platzhalter] vor Versand.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Eindeutiger Handhabungsschaden durch Zulieferer Fa. [Platzhalter] vor Versand."}, "cot_begruendung": "Der Schaden wird explizit als Handhabungsfehler durch den externen Zulieferer vor dem Versand identifiziert (Handhabung/Lieferant). Verborgene Lamellen erfordern eine Nacharbeit, stoppen aber die generelle Produktion des Wagens meist nicht sofort."}, {"fall_id": "197", "text": "Türen lassen sich nach der IBS nicht zentral schließen. Werker hat versehentlich die veraltete Tür-Software V1.0 von seinem lokalen USB-Stick geflasht, anstatt die freigegebene V1.2 vom Server zu ziehen. Alle Türen am Wagen müssen neu bespielt werden.", "zielvariablen": {"ursache": "Software", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker hat versehentlich die veraltete Tür-Software V1.0 von seinem lokalen USB-Stick geflasht"}, "cot_begruendung": "Das Aufspielen einer falschen/veralteten Software durch den Werker ist ein softwareseitiger und prozessualer Fehler, der direkt im Werk entstanden ist (Software/Werk). Da die sicherheitskritische zentrale Türschließung nicht funktioniert, ist die Inbetriebnahme hart blockiert."}]</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4551,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>[{"fall_id": "17", "text": "Drehmomentmarkierungen an allen Dachklappen HVAC1 bis HVAC4 verwischt. Werker hat falschen Lackstift benutzt. Gesamter Wagen 6 muss neu abgeknackt werden.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Werker hat falschen Lackstift benutzt. Gesamter Wagen 6"}, "cot_begruendung": "Die Nutzung eines falschen Lackstifts für Sicherheitsmarkierungen durch den Werker ist ein prozessualer Fehler in der Werkstatt. Da 'alle Dachklappen' am 'gesamten Wagen 6' betroffen sind, liegt ein Serienfehler vor. Die erneute Prüfung (Abknacken) erfordert Nacharbeit."}, {"fall_id": "44", "text": "Befestigung der Haltestange im FGR LWS lose. Werker hat vergessen, die Kontermutter anzubringen. Muss dringend nachgezogen werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, die Kontermutter anzubringen"}, "cot_begruendung": "Das explizite Vergessen der Kontermutter durch den Werker ist ein klassischer Montagefehler, der im eigenen Werk entstanden ist. Das Nachziehen der Mutter ist eine unkritische Nacharbeit."}, {"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}]</t>
+          <t>[{"fall_id": "169", "text": "Delle in der weißen Deckenverkleidung FGR RWS. IBS-Techniker ist beim Versuch, an den Rauchmelder zu kommen, mit seiner Alu-Leiter dagegen gestoßen.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "IBS-Techniker ist beim Versuch, an den Rauchmelder zu kommen, mit seiner Alu-Leiter dagegen gestoßen."}, "cot_begruendung": "Das Verursachen einer Delle durch Unachtsamkeit mit einer Leiter durch den internen IBS-Techniker ist ein Handhabungsfehler im Werk. Das optisch beschädigte Deckenelement muss ausgetauscht werden (Nacharbeit)."}, {"fall_id": "173", "text": "Sika-Fuge an der Nasszelle Tür LWS ist komplett verschmiert. Werker hat vergessen, vor dem Spritzen der Dichtmasse abzukleben.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, vor dem Spritzen der Dichtmasse abzukleben."}, "cot_begruendung": "Das Vergessen des Abklebens durch den Werker führt zu einer unsauberen Fuge, was einen Verarbeitungsfehler im eigenen Werk darstellt. Das Entfernen der Schmierer und Neuverfugen ist eine Nacharbeit."}, {"fall_id": "147", "text": "Leistungsschütz K12 im Hauptschalterkasten brennt sofort nach Anlegen der 110V Steuerspannung durch. Interne Spule hat ab Werk einen Kurzschluss. Betrifft Bauteil von Zulieferer ABC. Hauptstromkreis kann nicht zugeschaltet werden.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Interne Spule hat ab Werk einen Kurzschluss. Betrifft Bauteil von Zulieferer ABC. Hauptstromkreis kann nicht zugeschaltet werden."}, "cot_begruendung": "Ein Kurzschluss in der Spule ab Werk ist ein Materialfehler, der vom Zulieferer (Lieferant) verschuldet wurde. Da der Hauptstromkreis nicht zugeschaltet werden kann, ist die Inbetriebsetzung hart blockiert."}]</t>
         </is>
       </c>
     </row>
@@ -4626,7 +4626,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>[{"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "3", "text": "Kabelbaum für MFA-Display im Fahrerpult ist um 15cm zu kurz. Anschluss an Stecker X45 nicht möglich. Zeichnung laut Herrn [Platzhalter] fehlerhaft, Verlängerung nötig.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Zeichnung laut Herrn [Platzhalter] fehlerhaft"}, "cot_begruendung": "Die Aussage 'Zeichnung [...] fehlerhaft' verweist direkt auf einen Konstruktionsfehler aus dem Engineering. Da das Kabel zum MFA-Display (Fahrerpult) nicht angeschlossen werden kann, ist die Funktion des Zuges nicht gegeben und die Montage blockiert."}, {"fall_id": "61", "text": "Schrauben an der Bugnase WE1 mit 40Nm statt 25Nm angezogen. Gewinde teilweise überdreht. Vorgabe im Arbeitsplan wurde von Schicht 1 missachtet.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "mit 40Nm statt 25Nm angezogen. Vorgabe im Arbeitsplan wurde von Schicht 1 missachtet."}, "cot_begruendung": "Das Missachten der Drehmoment-Vorgaben aus dem Arbeitsplan durch die interne Schicht ist ein prozessualer bzw. Montagefehler im Werk. Beschädigte Gewinde müssen nachgearbeitet/ersetzt werden (Nacharbeit)."}]</t>
+          <t>[{"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "3", "text": "Kabelbaum für MFA-Display im Fahrerpult ist um 15cm zu kurz. Anschluss an Stecker X45 nicht möglich. Zeichnung laut Herrn [Platzhalter] fehlerhaft, Verlängerung nötig.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Zeichnung laut Herrn [Platzhalter] fehlerhaft"}, "cot_begruendung": "Die Aussage 'Zeichnung [...] fehlerhaft' verweist direkt auf einen Konstruktionsfehler aus dem Engineering. Da das Kabel zum MFA-Display (Fahrerpult) nicht angeschlossen werden kann, ist die Funktion des Zuges nicht gegeben und die Montage blockiert."}, {"fall_id": "172", "text": "Kabelbinder (schwarz, 300mm) fehlen komplett am Arbeitsplatz für die Unterflurverkabelung. Dispo hat im System den Meldebestand nicht richtig gepflegt, Lager ist leer. Kommen erst am Nachmittag.", "zielvariablen": {"ursache": "Software", "ursprung": "Logistik", "kritikalitaet": "Info", "serie": false, "text_snippet": "Dispo hat im System den Meldebestand nicht richtig gepflegt, Lager ist leer."}, "cot_begruendung": "Das Fehlen von C-Teilen aufgrund einer fehlerhaften Systempflege im ERP/Dispo-System ist ein softwareseitiges bzw. administratives Problem der internen Logistik. Kabelbinder sind temporär ersetzbar oder leicht nachzurüsten, weshalb der Ausbau meist nicht komplett steht (Info)."}]</t>
         </is>
       </c>
     </row>
@@ -4701,7 +4701,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>[{"fall_id": "8", "text": "Frontmaske hat matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend. Muss poliert/nachlackiert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend"}, "cot_begruendung": "Fehler beim Auftragen des Lacks ('Klarlack teilweise nicht deckend') weisen auf einen Verarbeitungs- bzw. Prozessfehler direkt in der Werksfertigung hin. Dies erfordert eine optische Nacharbeit, stellt aber keine funktionale Blockade dar."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
+          <t>[{"fall_id": "8", "text": "Frontmaske hat matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend. Muss poliert/nachlackiert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend"}, "cot_begruendung": "Fehler beim Auftragen des Lacks ('Klarlack teilweise nicht deckend') weisen auf einen Verarbeitungs- bzw. Prozessfehler direkt in der Werksfertigung hin. Dies erfordert eine optische Nacharbeit, stellt aber keine funktionale Blockade dar."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>[{"fall_id": "51", "text": "Schweißnaht an der Frontmaske unten links (SN-12) nur punktiert, nicht durchgeschweißt. Schweißer hat diesen Bereich scheinbar übersehen. Sonderfreigabe nicht möglich.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Schweißer hat diesen Bereich scheinbar übersehen. Sonderfreigabe nicht möglich."}, "cot_begruendung": "Ein Übersehen einer Schweißnaht durch den Werker ist ein schwerer Prozess- bzw. Fertigungsfehler im Werk. Da eine fehlende Schweißnaht am Rohbau/Frontmaske die statische Integrität gefährdet und keine Sonderfreigabe möglich ist, ist es ein absoluter Blocker."}, {"fall_id": "67", "text": "Versteifungsrippe RWS im Unterflur nicht verschweißt, nur geheftet. Schweißer hat die finale Naht komplett vergessen. Fahrzeug darf so nicht aufgebockt werden.", "zielvariablen": {"grundursache": "Fertigung", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Schweißer hat die finale Naht komplett vergessen. Fahrzeug darf so nicht aufgebockt werden."}, "cot_begruendung": "Das Vergessen der finalen Schweißnaht durch den Schweißer ist ein schwerer Fertigungsfehler im Rohbau (Werk). Da die Statik gefährdet ist ('Fahrzeug darf so nicht aufgebockt werden'), liegt ein kritischer Blocker vor."}, {"fall_id": "95", "text": "Halter für Feuerlöscher aus interner Schweißerei sind um 10mm zu schmal. Feuerlöscher passt nicht rein. Betrifft alle 20 Halter der heutigen Tagesproduktion.", "zielvariablen": {"grundursache": "Fertigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "aus interner Schweißerei sind um 10mm zu schmal. [...] Betrifft alle 20 Halter der heutigen Tagesproduktion."}, "cot_begruendung": "Falsch gefertigte Halter aus der 'internen Schweißerei' sind ein Fertigungsfehler im Werk. Der Hinweis auf 'alle 20 Halter' flaggt den Fehler als Serie. Die Halter müssen nachgearbeitet/neu produziert werden, stoppen aber den Waggonbau nicht komplett."}]</t>
+          <t>[{"fall_id": "165", "text": "Schweißnaht an allen 10 Halteblechen für die HBU unterflur fehlerhaft ausgeführt (zu wenig Einbrand). Aus unserer internen Schweißerei. QA sperrt Wagen für jegliche Weiterarbeit unter dem Fahrzeug.", "zielvariablen": {"ursache": "Fertigung", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "an allen 10 Halteblechen [...] zu wenig Einbrand). Aus unserer internen Schweißerei. QA sperrt Wagen"}, "cot_begruendung": "Mangelhafte Schweißnähte aus der 'internen Schweißerei' sind ein Fertigungsfehler im Werk. Der Vermerk 'allen 10 Halteblechen' kennzeichnet die Serie. Da die QA den Wagen für den weiteren Unterflurausbau sperrt, liegt eine hohe Kritikalität (Blocker) vor."}, {"fall_id": "51", "text": "Schweißnaht an der Frontmaske unten links (SN-12) nur punktiert, nicht durchgeschweißt. Schweißer hat diesen Bereich scheinbar übersehen. Sonderfreigabe nicht möglich.", "zielvariablen": {"ursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Schweißer hat diesen Bereich scheinbar übersehen. Sonderfreigabe nicht möglich."}, "cot_begruendung": "Ein Übersehen einer Schweißnaht durch den Werker ist ein schwerer Prozess- bzw. Fertigungsfehler im Werk. Da eine fehlende Schweißnaht am Rohbau/Frontmaske die statische Integrität gefährdet und keine Sonderfreigabe möglich ist, ist es ein absoluter Blocker."}, {"fall_id": "67", "text": "Versteifungsrippe RWS im Unterflur nicht verschweißt, nur geheftet. Schweißer hat die finale Naht komplett vergessen. Fahrzeug darf so nicht aufgebockt werden.", "zielvariablen": {"ursache": "Fertigung", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Schweißer hat die finale Naht komplett vergessen. Fahrzeug darf so nicht aufgebockt werden."}, "cot_begruendung": "Das Vergessen der finalen Schweißnaht durch den Schweißer ist ein schwerer Fertigungsfehler im Rohbau (Werk). Da die Statik gefährdet ist ('Fahrzeug darf so nicht aufgebockt werden'), liegt ein kritischer Blocker vor."}]</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>[{"fall_id": "16", "text": "Klebereste von Schutzfolie an Fensterscheibe WE2 links. Wurde beim Abziehen nicht sauber gereinigt.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Wurde beim Abziehen nicht sauber gereinigt"}, "cot_begruendung": "Klebereste von Schutzfolien sind ein typischer Fehler aus der Endreinigung im Werk. Da der Fehler schnell behebbar ist und keine Bauteile beschädigt sind, wird er als 'Info' oder sehr leichte Nacharbeit eingestuft."}, {"fall_id": "30", "text": "Gummiprofil an Einstiegstür WE1 rissig. Betrifft Lieferung von ABC-Gummi der KW12 komplett. Material ist spröde.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Betrifft Lieferung von ABC-Gummi der KW12 komplett. Material ist spröde."}, "cot_begruendung": "Das spröde Gummiprofil ist auf eine fehlerhafte Materiallieferung von 'ABC-Gummi' zurückzuführen (Material/Lieferant). Der Hinweis 'Lieferung [...] komplett' markiert dies eindeutig als Serienfehler. Ein rissiges Gummi muss getauscht werden (Nacharbeit)."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
+          <t>[{"fall_id": "16", "text": "Klebereste von Schutzfolie an Fensterscheibe WE2 links. Wurde beim Abziehen nicht sauber gereinigt.", "zielvariablen": {"ursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Wurde beim Abziehen nicht sauber gereinigt"}, "cot_begruendung": "Klebereste von Schutzfolien sind ein typischer Fehler aus der Endreinigung im Werk. Da der Fehler schnell behebbar ist und keine Bauteile beschädigt sind, wird er als 'Info' oder sehr leichte Nacharbeit eingestuft."}, {"fall_id": "30", "text": "Gummiprofil an Einstiegstür WE1 rissig. Betrifft Lieferung von ABC-Gummi der KW12 komplett. Material ist spröde.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Betrifft Lieferung von ABC-Gummi der KW12 komplett. Material ist spröde."}, "cot_begruendung": "Das spröde Gummiprofil ist auf eine fehlerhafte Materiallieferung von 'ABC-Gummi' zurückzuführen (Material/Lieferant). Der Hinweis 'Lieferung [...] komplett' markiert dies eindeutig als Serienfehler. Ein rissiges Gummi muss getauscht werden (Nacharbeit)."}, {"fall_id": "164", "text": "Lackschaden an der Innenseite der WC-Tür. Staubeinschlüsse sind deutlich sichtbar. Passierte bei der manuellen Nachlackierung im internen Lackierbereich.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Staubeinschlüsse sind deutlich sichtbar. Passierte bei der manuellen Nachlackierung im internen Lackierbereich."}, "cot_begruendung": "Staubeinschlüsse durch unsaubere Umgebungsbedingungen bei der manuellen internen Lackierung sind Verarbeitungs- und Prozessfehler im Werk. Die Tür muss abgeschliffen und poliert werden (Nacharbeit)."}]</t>
         </is>
       </c>
     </row>
@@ -4926,7 +4926,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>[{"fall_id": "27", "text": "Scheibe RWS im FGR schmierig. Putzkolonne hat falsches Reinigungsmittel verwendet, Schlieren lassen sich schwer entfernen.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Putzkolonne hat falsches Reinigungsmittel verwendet"}, "cot_begruendung": "Die Verschmutzung wurde explizit durch die Putzkolonne ('falsches Reinigungsmittel') verursacht. Dies ist ein Reinigungsfehler im Werk. Da dies weder die Montage aufhält noch ein Bauteil zerstört, wird es als reine Nacharbeit/Info eingestuft."}, {"fall_id": "22", "text": "Fahrgasttür RWS öffnet nicht bei Tasterbetätigung. DCU gibt keinen Befehl raus. Ersatzteil aus Lager geholt, Tür funktioniert wieder. Defekte DCU geht an Lieferant retour.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "DCU gibt keinen Befehl raus. [...] Defekte DCU geht an Lieferant retour"}, "cot_begruendung": "Die Door Control Unit (DCU) ist intern defekt, was auf einen Materialfehler des Lieferanten schließen lässt. Da das Ersatzteil sofort aus dem Lager verfügbar war und die Produktion nicht gestoppt wurde, bleibt es bei einer Nacharbeit."}, {"fall_id": "76", "text": "Türen LWS öffnen sich, wenn Taster für RWS gedrückt wird. Software-Mapping in der DCU vom Engineering komplett vertauscht. Gefahr für Leib und Leben, IBS abgebrochen.", "zielvariablen": {"grundursache": "Software", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Software-Mapping in der DCU vom Engineering komplett vertauscht. Gefahr für Leib und Leben, IBS abgebrochen."}, "cot_begruendung": "Vertauschtes Software-Mapping durch das Engineering ist ein Software/Konstruktions-Fehler. Ein sicherheitskritisches Türproblem mit Abbruch der IBS ist der Inbegriff eines harten Blockers."}]</t>
+          <t>[{"fall_id": "27", "text": "Scheibe RWS im FGR schmierig. Putzkolonne hat falsches Reinigungsmittel verwendet, Schlieren lassen sich schwer entfernen.", "zielvariablen": {"ursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Putzkolonne hat falsches Reinigungsmittel verwendet"}, "cot_begruendung": "Die Verschmutzung wurde explizit durch die Putzkolonne ('falsches Reinigungsmittel') verursacht. Dies ist ein Reinigungsfehler im Werk. Da dies weder die Montage aufhält noch ein Bauteil zerstört, wird es als reine Nacharbeit/Info eingestuft."}, {"fall_id": "117", "text": "Befestigung der Sitzkiste RWS im FGR wackelt. Werker hat statt der M8x25 eine M8x40 Schraube mit Gewalt reingedreht und das Gewinde im Boden zerstört. Gewindeeinsatz muss neu gesetzt werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat statt der M8x25 eine M8x40 Schraube mit Gewalt reingedreht"}, "cot_begruendung": "Die Zerstörung des Gewindes durch den Werker (falsche Schraube, Gewaltanwendung) ist ein klarer Montage- und Handhabungsfehler im eigenen Werk. Die Reparatur des Gewindes ist zwar aufwendig, stellt aber einen lokalen Eingriff dar (Nacharbeit)."}, {"fall_id": "22", "text": "Fahrgasttür RWS öffnet nicht bei Tasterbetätigung. DCU gibt keinen Befehl raus. Ersatzteil aus Lager geholt, Tür funktioniert wieder. Defekte DCU geht an Lieferant retour.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "DCU gibt keinen Befehl raus. [...] Defekte DCU geht an Lieferant retour"}, "cot_begruendung": "Die Door Control Unit (DCU) ist intern defekt, was auf einen Materialfehler des Lieferanten schließen lässt. Da das Ersatzteil sofort aus dem Lager verfügbar war und die Produktion nicht gestoppt wurde, bleibt es bei einer Nacharbeit."}]</t>
         </is>
       </c>
     </row>
@@ -5001,7 +5001,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>[{"fall_id": "62", "text": "Kabelkanal unterflur kollidiert mit der Druckluftleitung für die Bremsanlage. Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich."}, "cot_begruendung": "Eine Überlappung im 3D-Modell/Zeichnung ist ein Konstruktionsfehler aus dem Engineering. Da die Druckluftleitung für die Bremsen essenziell ist und die 'Rohrverlegung aktuell unmöglich' ist, handelt es sich um einen harten Blocker."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}]</t>
+          <t>[{"fall_id": "62", "text": "Kabelkanal unterflur kollidiert mit der Druckluftleitung für die Bremsanlage. Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich."}, "cot_begruendung": "Eine Überlappung im 3D-Modell/Zeichnung ist ein Konstruktionsfehler aus dem Engineering. Da die Druckluftleitung für die Bremsen essenziell ist und die 'Rohrverlegung aktuell unmöglich' ist, handelt es sich um einen harten Blocker."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}]</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5076,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "4", "text": "Erdungsband am Triebdrehgestell WE1 links vergessen anzuschrauben. Schraube liegt lose auf dem Rahmen.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "vergessen anzuschrauben"}, "cot_begruendung": "Das vergessene Anschrauben ('Schraube liegt lose auf dem Rahmen') ist ein eindeutiger Montage- und Ausführungsfehler im Werk. Da eine fehlende Erdung am Triebdrehgestell ein massives Sicherheitsrisiko darstellt und die Inbetriebnahme verhindert, ist dies ein Blocker."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
+          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "121", "text": "Kollision des Sandungsrohrs mit dem Drehgestellrahmen bei Ausdrehwinkel &gt; 5 Grad. Das EN hat den Schwenkbereich des Drehgestells im 3D-Modell nicht korrekt simuliert. Verrohrung muss komplett geändert werden. Fahrtests untersagt.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Das EN hat den Schwenkbereich des Drehgestells im 3D-Modell nicht korrekt simuliert. [...] Fahrtests untersagt."}, "cot_begruendung": "Die fehlende Simulation des Schwenkbereichs durch das Engineering (EN) ist ein eindeutiger Konstruktionsfehler. Eine statische Kollision am sicherheitsrelevanten Drehgestell, die zu einem Testverbot führt, macht dieses Problem zu einem absoluten Blocker."}, {"fall_id": "4", "text": "Erdungsband am Triebdrehgestell WE1 links vergessen anzuschrauben. Schraube liegt lose auf dem Rahmen.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "vergessen anzuschrauben"}, "cot_begruendung": "Das vergessene Anschrauben ('Schraube liegt lose auf dem Rahmen') ist ein eindeutiger Montage- und Ausführungsfehler im Werk. Da eine fehlende Erdung am Triebdrehgestell ein massives Sicherheitsrisiko darstellt und die Inbetriebnahme verhindert, ist dies ein Blocker."}]</t>
         </is>
       </c>
     </row>
@@ -5151,7 +5151,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>[{"fall_id": "26", "text": "Hauptkabelstrang HKS-3 unterflur am Drehgestell WE2 durchtrennt. Staplerfahrer hat beim Abladen der Palette reingestochen. Kabelbaum muss komplett neu.", "zielvariablen": {"grundursache": "Handhabung", "ursprung": "Logistik", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Staplerfahrer hat beim Abladen der Palette reingestochen"}, "cot_begruendung": "Der Text beschreibt eindeutig eine mechanische Beschädigung durch einen Staplerfahrer beim Abladen. Dies ist ein Handhabungsfehler, der der Logistik zuzuordnen ist. Da der Hauptkabelstrang komplett neu muss, kann das Fahrzeug elektrisch nicht in Betrieb genommen werden (Blocker)."}, {"fall_id": "62", "text": "Kabelkanal unterflur kollidiert mit der Druckluftleitung für die Bremsanlage. Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich."}, "cot_begruendung": "Eine Überlappung im 3D-Modell/Zeichnung ist ein Konstruktionsfehler aus dem Engineering. Da die Druckluftleitung für die Bremsen essenziell ist und die 'Rohrverlegung aktuell unmöglich' ist, handelt es sich um einen harten Blocker."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}]</t>
+          <t>[{"fall_id": "154", "text": "Kabelstrang für Notbremsschleife LWS auf einer Länge von 2 Metern gequetscht. Ein Gabelstapler ist im Gang über das Kabel gefahren, bevor es in die Kabelkanäle gelegt wurde.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Logistik", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Ein Gabelstapler ist im Gang über das Kabel gefahren, bevor es in die Kabelkanäle gelegt wurde."}, "cot_begruendung": "Das Überfahren eines Bauteils durch einen Gabelstapler ist ein Handhabungs- bzw. Intralogistik-Fehler (Logistik). Da das Kabel der sicherheitsrelevanten Notbremsschleife komplett getauscht werden muss, was zeitintensiv ist und Folgegewerke stoppt, ist es ein Blocker."}, {"fall_id": "26", "text": "Hauptkabelstrang HKS-3 unterflur am Drehgestell WE2 durchtrennt. Staplerfahrer hat beim Abladen der Palette reingestochen. Kabelbaum muss komplett neu.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Logistik", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Staplerfahrer hat beim Abladen der Palette reingestochen"}, "cot_begruendung": "Der Text beschreibt eindeutig eine mechanische Beschädigung durch einen Staplerfahrer beim Abladen. Dies ist ein Handhabungsfehler, der der Logistik zuzuordnen ist. Da der Hauptkabelstrang komplett neu muss, kann das Fahrzeug elektrisch nicht in Betrieb genommen werden (Blocker)."}, {"fall_id": "102", "text": "Bohrung für Erdungskabel am Drehgestell WE2 ist mit dicker Lackschicht verschlossen. Gewinde muss mühsam nachgeschnitten werden. Vorfertigung hat die Gewindeschoner vor dem Lackieren vergessen.", "zielvariablen": {"ursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Vorfertigung hat die Gewindeschoner vor dem Lackieren vergessen."}, "cot_begruendung": "Das Vergessen der Gewindeschoner durch die interne Vorfertigung vor dem Lackieren ist ein prozessualer Verarbeitungsfehler im eigenen Werk. Das Nachschneiden des Gewindes ist eine typische, lokal behebbare Nacharbeit."}]</t>
         </is>
       </c>
     </row>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>[{"fall_id": "79", "text": "Sitzbezüge im gesamten Wagen reißen an der Naht ein. Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge müssen getauscht werden.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge"}, "cot_begruendung": "Die mangelhafte Stoffqualität eines externen Lieferanten ist ein Materialfehler. Die Bemerkungen 'gesamter Wagen' und 'neuen Serie' verweisen auf einen Serienfehler. Das Austauschen der Bezüge ist Nacharbeit, aber kein Blocker für Inbetriebsetzungen."}, {"fall_id": "17", "text": "Drehmomentmarkierungen an allen Dachklappen HVAC1 bis HVAC4 verwischt. Werker hat falschen Lackstift benutzt. Gesamter Wagen 6 muss neu abgeknackt werden.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Werker hat falschen Lackstift benutzt. Gesamter Wagen 6"}, "cot_begruendung": "Die Nutzung eines falschen Lackstifts für Sicherheitsmarkierungen durch den Werker ist ein prozessualer Fehler in der Werkstatt. Da 'alle Dachklappen' am 'gesamten Wagen 6' betroffen sind, liegt ein Serienfehler vor. Die erneute Prüfung (Abknacken) erfordert Nacharbeit."}, {"fall_id": "21", "text": "Spaltmaß bei Übergangstür WE2 zu groß (&gt;8mm). Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3"}, "cot_begruendung": "Wenn Scharniere physisch nicht weiter justierbar sind, liegt oft ein Toleranz- oder Konstruktionsproblem (Engineering) vor, weniger ein Montagefehler. Der explizite Hinweis auf 'Wagen 1, 2 und 3' ist ein eindeutiger Indikator für einen Serienfehler. Ein falsches Spaltmaß erfordert Nacharbeit."}]</t>
+          <t>[{"fall_id": "79", "text": "Sitzbezüge im gesamten Wagen reißen an der Naht ein. Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge müssen getauscht werden.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge"}, "cot_begruendung": "Die mangelhafte Stoffqualität eines externen Lieferanten ist ein Materialfehler. Die Bemerkungen 'gesamter Wagen' und 'neuen Serie' verweisen auf einen Serienfehler. Das Austauschen der Bezüge ist Nacharbeit, aber kein Blocker für Inbetriebsetzungen."}, {"fall_id": "110", "text": "Zugsteuerung erkennt das zweite Drehgestell nicht. Fehlerhafter Crimp am Stecker X75 unterflur. Leitungen haben Wackelkontakt. Montage-Team muss Crimpung erneuern.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Fehlerhafter Crimp am Stecker X75 unterflur. [...] Montage-Team muss Crimpung erneuern."}, "cot_begruendung": "Ein fehlerhafter Crimp durch das Montage-Team führt zu einem Wackelkontakt, was einen Ausführungsfehler (Montage) im Werk darstellt. Da die Zugsteuerung das Drehgestell nicht erkennt, ist keine Fahrtübersicht gegeben, was eine Inbetriebnahme blockiert (Blocker)."}, {"fall_id": "107", "text": "Piktogramme für Feuerlöscher und Notbremse im gesamten Wagen 4 fehlen komplett. Wurden bei der Materialausgabe nicht kommissioniert. Bitte per Bote an die Linie schicken.", "zielvariablen": {"ursache": "Logistik", "ursprung": "Logistik", "kritikalitaet": "Info", "serie": false, "text_snippet": "Wurden bei der Materialausgabe nicht kommissioniert."}, "cot_begruendung": "Das Fehlen von Piktogrammen aufgrund eines Kommissionierungsfehlers in der Materialausgabe ist ein prozessuales Problem der Logistik. Aufkleber blockieren die technische Fertigung und Inbetriebnahme nicht, daher als 'Info' verbucht."}]</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>[{"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}, {"fall_id": "65", "text": "Tür geht nicht.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Tür geht nicht."}, "cot_begruendung": "Der Text 'Tür geht nicht' ist maximal unspezifisch. Es fehlen jegliche Hinweise auf mechanische, elektrische, softwareseitige oder prozessuale Ursachen. Gemäß Abstention-Vorgabe muss Unbekannt ausgegeben werden."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}]</t>
+          <t>[{"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}, {"fall_id": "197", "text": "Türen lassen sich nach der IBS nicht zentral schließen. Werker hat versehentlich die veraltete Tür-Software V1.0 von seinem lokalen USB-Stick geflasht, anstatt die freigegebene V1.2 vom Server zu ziehen. Alle Türen am Wagen müssen neu bespielt werden.", "zielvariablen": {"ursache": "Software", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker hat versehentlich die veraltete Tür-Software V1.0 von seinem lokalen USB-Stick geflasht"}, "cot_begruendung": "Das Aufspielen einer falschen/veralteten Software durch den Werker ist ein softwareseitiger und prozessualer Fehler, der direkt im Werk entstanden ist (Software/Werk). Da die sicherheitskritische zentrale Türschließung nicht funktioniert, ist die Inbetriebnahme hart blockiert."}, {"fall_id": "65", "text": "Tür geht nicht.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Tür geht nicht."}, "cot_begruendung": "Der Text 'Tür geht nicht' ist maximal unspezifisch. Es fehlen jegliche Hinweise auf mechanische, elektrische, softwareseitige oder prozessuale Ursachen. Gemäß Abstention-Vorgabe muss Unbekannt ausgegeben werden."}]</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5376,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>[{"fall_id": "16", "text": "Klebereste von Schutzfolie an Fensterscheibe WE2 links. Wurde beim Abziehen nicht sauber gereinigt.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Wurde beim Abziehen nicht sauber gereinigt"}, "cot_begruendung": "Klebereste von Schutzfolien sind ein typischer Fehler aus der Endreinigung im Werk. Da der Fehler schnell behebbar ist und keine Bauteile beschädigt sind, wird er als 'Info' oder sehr leichte Nacharbeit eingestuft."}, {"fall_id": "40", "text": "PMA-Schlauch am Unterflur WE1 links kollidiert leicht mit der Achse. Kabelbinder wurde vom Werker zu locker gezogen.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Kabelbinder wurde vom Werker zu locker gezogen."}, "cot_begruendung": "Ein zu locker gezogener Kabelbinder durch den Werker ist ein klassischer Montagefehler im Werk. Die leichte Kollision des Schlauchs muss durch Setzen eines neuen Kabelbinders nachgearbeitet werden, hält die Produktion aber nicht an."}, {"fall_id": "75", "text": "Großer Spiegel in der Nasszelle komplett zersplittert. Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang.", "zielvariablen": {"grundursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang."}, "cot_begruendung": "Der durchstoßene Karton im Wareneingang durch einen Gabelstapler ist ein eindeutiger Transportschaden (Logistik). Ein kaputter Spiegel muss bestellt und nachgearbeitet werden, hält den Zugbau aber nicht auf."}]</t>
+          <t>[{"fall_id": "16", "text": "Klebereste von Schutzfolie an Fensterscheibe WE2 links. Wurde beim Abziehen nicht sauber gereinigt.", "zielvariablen": {"ursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Wurde beim Abziehen nicht sauber gereinigt"}, "cot_begruendung": "Klebereste von Schutzfolien sind ein typischer Fehler aus der Endreinigung im Werk. Da der Fehler schnell behebbar ist und keine Bauteile beschädigt sind, wird er als 'Info' oder sehr leichte Nacharbeit eingestuft."}, {"fall_id": "40", "text": "PMA-Schlauch am Unterflur WE1 links kollidiert leicht mit der Achse. Kabelbinder wurde vom Werker zu locker gezogen.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Kabelbinder wurde vom Werker zu locker gezogen."}, "cot_begruendung": "Ein zu locker gezogener Kabelbinder durch den Werker ist ein klassischer Montagefehler im Werk. Die leichte Kollision des Schlauchs muss durch Setzen eines neuen Kabelbinders nachgearbeitet werden, hält die Produktion aber nicht an."}, {"fall_id": "75", "text": "Großer Spiegel in der Nasszelle komplett zersplittert. Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang.", "zielvariablen": {"ursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang."}, "cot_begruendung": "Der durchstoßene Karton im Wareneingang durch einen Gabelstapler ist ein eindeutiger Transportschaden (Logistik). Ein kaputter Spiegel muss bestellt und nachgearbeitet werden, hält den Zugbau aber nicht auf."}]</t>
         </is>
       </c>
     </row>
@@ -5451,7 +5451,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>[{"fall_id": "26", "text": "Hauptkabelstrang HKS-3 unterflur am Drehgestell WE2 durchtrennt. Staplerfahrer hat beim Abladen der Palette reingestochen. Kabelbaum muss komplett neu.", "zielvariablen": {"grundursache": "Handhabung", "ursprung": "Logistik", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Staplerfahrer hat beim Abladen der Palette reingestochen"}, "cot_begruendung": "Der Text beschreibt eindeutig eine mechanische Beschädigung durch einen Staplerfahrer beim Abladen. Dies ist ein Handhabungsfehler, der der Logistik zuzuordnen ist. Da der Hauptkabelstrang komplett neu muss, kann das Fahrzeug elektrisch nicht in Betrieb genommen werden (Blocker)."}, {"fall_id": "70", "text": "Anschlusskabel für Notbremsschalter im FGR zu kurz geschnitten. Werker hat den Kabelstrang nicht wie vorgeschrieben in Schleife gelegt, sondern direkt gezogen. Neuverkabelung der halben Seite LWS nötig.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker hat den Kabelstrang nicht wie vorgeschrieben in Schleife gelegt, sondern direkt gezogen. Neuverkabelung der halben Seite LWS nötig."}, "cot_begruendung": "Der Werker hat den Kabelstrang falsch verlegt (nicht in Schleife), was einen Montagefehler im Werk darstellt. Da sicherheitsrelevante Notbremsschalter betroffen sind und die halbe Seite neu verkabelt werden muss, ist dies ein massiver Verzug und somit ein Blocker."}, {"fall_id": "62", "text": "Kabelkanal unterflur kollidiert mit der Druckluftleitung für die Bremsanlage. Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich."}, "cot_begruendung": "Eine Überlappung im 3D-Modell/Zeichnung ist ein Konstruktionsfehler aus dem Engineering. Da die Druckluftleitung für die Bremsen essenziell ist und die 'Rohrverlegung aktuell unmöglich' ist, handelt es sich um einen harten Blocker."}]</t>
+          <t>[{"fall_id": "154", "text": "Kabelstrang für Notbremsschleife LWS auf einer Länge von 2 Metern gequetscht. Ein Gabelstapler ist im Gang über das Kabel gefahren, bevor es in die Kabelkanäle gelegt wurde.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Logistik", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Ein Gabelstapler ist im Gang über das Kabel gefahren, bevor es in die Kabelkanäle gelegt wurde."}, "cot_begruendung": "Das Überfahren eines Bauteils durch einen Gabelstapler ist ein Handhabungs- bzw. Intralogistik-Fehler (Logistik). Da das Kabel der sicherheitsrelevanten Notbremsschleife komplett getauscht werden muss, was zeitintensiv ist und Folgegewerke stoppt, ist es ein Blocker."}, {"fall_id": "26", "text": "Hauptkabelstrang HKS-3 unterflur am Drehgestell WE2 durchtrennt. Staplerfahrer hat beim Abladen der Palette reingestochen. Kabelbaum muss komplett neu.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Logistik", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Staplerfahrer hat beim Abladen der Palette reingestochen"}, "cot_begruendung": "Der Text beschreibt eindeutig eine mechanische Beschädigung durch einen Staplerfahrer beim Abladen. Dies ist ein Handhabungsfehler, der der Logistik zuzuordnen ist. Da der Hauptkabelstrang komplett neu muss, kann das Fahrzeug elektrisch nicht in Betrieb genommen werden (Blocker)."}, {"fall_id": "102", "text": "Bohrung für Erdungskabel am Drehgestell WE2 ist mit dicker Lackschicht verschlossen. Gewinde muss mühsam nachgeschnitten werden. Vorfertigung hat die Gewindeschoner vor dem Lackieren vergessen.", "zielvariablen": {"ursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Vorfertigung hat die Gewindeschoner vor dem Lackieren vergessen."}, "cot_begruendung": "Das Vergessen der Gewindeschoner durch die interne Vorfertigung vor dem Lackieren ist ein prozessualer Verarbeitungsfehler im eigenen Werk. Das Nachschneiden des Gewindes ist eine typische, lokal behebbare Nacharbeit."}]</t>
         </is>
       </c>
     </row>
@@ -5526,7 +5526,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>[{"fall_id": "26", "text": "Hauptkabelstrang HKS-3 unterflur am Drehgestell WE2 durchtrennt. Staplerfahrer hat beim Abladen der Palette reingestochen. Kabelbaum muss komplett neu.", "zielvariablen": {"grundursache": "Handhabung", "ursprung": "Logistik", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Staplerfahrer hat beim Abladen der Palette reingestochen"}, "cot_begruendung": "Der Text beschreibt eindeutig eine mechanische Beschädigung durch einen Staplerfahrer beim Abladen. Dies ist ein Handhabungsfehler, der der Logistik zuzuordnen ist. Da der Hauptkabelstrang komplett neu muss, kann das Fahrzeug elektrisch nicht in Betrieb genommen werden (Blocker)."}, {"fall_id": "70", "text": "Anschlusskabel für Notbremsschalter im FGR zu kurz geschnitten. Werker hat den Kabelstrang nicht wie vorgeschrieben in Schleife gelegt, sondern direkt gezogen. Neuverkabelung der halben Seite LWS nötig.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker hat den Kabelstrang nicht wie vorgeschrieben in Schleife gelegt, sondern direkt gezogen. Neuverkabelung der halben Seite LWS nötig."}, "cot_begruendung": "Der Werker hat den Kabelstrang falsch verlegt (nicht in Schleife), was einen Montagefehler im Werk darstellt. Da sicherheitsrelevante Notbremsschalter betroffen sind und die halbe Seite neu verkabelt werden muss, ist dies ein massiver Verzug und somit ein Blocker."}, {"fall_id": "62", "text": "Kabelkanal unterflur kollidiert mit der Druckluftleitung für die Bremsanlage. Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich."}, "cot_begruendung": "Eine Überlappung im 3D-Modell/Zeichnung ist ein Konstruktionsfehler aus dem Engineering. Da die Druckluftleitung für die Bremsen essenziell ist und die 'Rohrverlegung aktuell unmöglich' ist, handelt es sich um einen harten Blocker."}]</t>
+          <t>[{"fall_id": "141", "text": "Erdungsband am Hochspannungsschrank WE1 nicht verschraubt, hängt lose herab. Werker hat es vergessen anzuschließen. Lebensgefahr beim Einschalten der Fahrleitungsspannung!", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker hat es vergessen anzuschließen. Lebensgefahr beim Einschalten"}, "cot_begruendung": "Das Vergessen des Erdungsbandes durch den Werker ist ein klassischer Montagefehler im eigenen Werk. Da eine lose Erdung an einem Hochspannungsschrank absolute Lebensgefahr bedeutet und die IBS verhindert, ist es ein kritischer Blocker."}, {"fall_id": "26", "text": "Hauptkabelstrang HKS-3 unterflur am Drehgestell WE2 durchtrennt. Staplerfahrer hat beim Abladen der Palette reingestochen. Kabelbaum muss komplett neu.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Logistik", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Staplerfahrer hat beim Abladen der Palette reingestochen"}, "cot_begruendung": "Der Text beschreibt eindeutig eine mechanische Beschädigung durch einen Staplerfahrer beim Abladen. Dies ist ein Handhabungsfehler, der der Logistik zuzuordnen ist. Da der Hauptkabelstrang komplett neu muss, kann das Fahrzeug elektrisch nicht in Betrieb genommen werden (Blocker)."}, {"fall_id": "172", "text": "Kabelbinder (schwarz, 300mm) fehlen komplett am Arbeitsplatz für die Unterflurverkabelung. Dispo hat im System den Meldebestand nicht richtig gepflegt, Lager ist leer. Kommen erst am Nachmittag.", "zielvariablen": {"ursache": "Software", "ursprung": "Logistik", "kritikalitaet": "Info", "serie": false, "text_snippet": "Dispo hat im System den Meldebestand nicht richtig gepflegt, Lager ist leer."}, "cot_begruendung": "Das Fehlen von C-Teilen aufgrund einer fehlerhaften Systempflege im ERP/Dispo-System ist ein softwareseitiges bzw. administratives Problem der internen Logistik. Kabelbinder sind temporär ersetzbar oder leicht nachzurüsten, weshalb der Ausbau meist nicht komplett steht (Info)."}]</t>
         </is>
       </c>
     </row>
@@ -5601,7 +5601,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>[{"fall_id": "63", "text": "Kurzschluss im Taster für WC-Spülung WE2. Reinigungstrupp hat mit Hochdruckreiniger direkt in den Taster gesprüht, Wasser im Gehäuse.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Reinigungstrupp hat mit Hochdruckreiniger direkt in den Taster gesprüht"}, "cot_begruendung": "Die Zerstörung des Tasters durch unsachgemäßen Einsatz eines Hochdruckreinigers ist eindeutig der Reinigung im Werk (Verursacher) zuzuschreiben. Ein defekter Spülungstaster muss getauscht werden (Nacharbeit)."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "74", "text": "Fugenabdichtung im WC WE2 unsauber gezogen. Werker hat Silikon statt PU-Dichtmasse verwendet. Fuge muss komplett rausgekratzt und neu gemacht werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat Silikon statt PU-Dichtmasse verwendet."}, "cot_begruendung": "Die Verwendung des falschen Dichtmittels durch den Werker ist ein Verarbeitungs- und Prozessfehler im Werk. Das Auskratzen und Erneuern der Fuge ist eine typische Nacharbeit."}]</t>
+          <t>[{"fall_id": "164", "text": "Lackschaden an der Innenseite der WC-Tür. Staubeinschlüsse sind deutlich sichtbar. Passierte bei der manuellen Nachlackierung im internen Lackierbereich.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Staubeinschlüsse sind deutlich sichtbar. Passierte bei der manuellen Nachlackierung im internen Lackierbereich."}, "cot_begruendung": "Staubeinschlüsse durch unsaubere Umgebungsbedingungen bei der manuellen internen Lackierung sind Verarbeitungs- und Prozessfehler im Werk. Die Tür muss abgeschliffen und poliert werden (Nacharbeit)."}, {"fall_id": "133", "text": "Kiste mit den WC-Spiegeln wurde vom Zulieferer [Platzhalter] stark beschädigt angeliefert. Spiegel innen sind zerkratzt. Wareneingang hat die Palette leider ungeprüft angenommen.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "vom Zulieferer [Platzhalter] stark beschädigt angeliefert. Spiegel innen sind zerkratzt."}, "cot_begruendung": "Der Schaden wird explizit dem Zulieferer zugeschrieben, der die Palette bereits beschädigt angeliefert hat (Handhabung/Lieferant). Zerkratzte Spiegel müssen ausgetauscht werden, stellen aber eine einfache Nacharbeit dar."}, {"fall_id": "143", "text": "Bodenbelag im WC WE2 ist extrem stumpf und weist weiße Schlieren auf. Reinigungspersonal hat statt des Neutralreinigers einen stark alkalischen Grundreiniger unverdünnt benutzt.", "zielvariablen": {"ursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Reinigungspersonal hat statt des Neutralreinigers einen stark alkalischen Grundreiniger unverdünnt benutzt."}, "cot_begruendung": "Die falsche Dosierung und Wahl des Reinigungsmittels durch das interne Reinigungspersonal ist ein Verursacher in Reinigung/Werk. Optische Schlieren am Boden sind als Info/leichte Nacharbeit zu bewerten."}]</t>
         </is>
       </c>
     </row>
@@ -5676,7 +5676,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "21", "text": "Spaltmaß bei Übergangstür WE2 zu groß (&gt;8mm). Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3"}, "cot_begruendung": "Wenn Scharniere physisch nicht weiter justierbar sind, liegt oft ein Toleranz- oder Konstruktionsproblem (Engineering) vor, weniger ein Montagefehler. Der explizite Hinweis auf 'Wagen 1, 2 und 3' ist ein eindeutiger Indikator für einen Serienfehler. Ein falsches Spaltmaß erfordert Nacharbeit."}]</t>
+          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "21", "text": "Spaltmaß bei Übergangstür WE2 zu groß (&gt;8mm). Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3"}, "cot_begruendung": "Wenn Scharniere physisch nicht weiter justierbar sind, liegt oft ein Toleranz- oder Konstruktionsproblem (Engineering) vor, weniger ein Montagefehler. Der explizite Hinweis auf 'Wagen 1, 2 und 3' ist ein eindeutiger Indikator für einen Serienfehler. Ein falsches Spaltmaß erfordert Nacharbeit."}]</t>
         </is>
       </c>
     </row>
@@ -5751,7 +5751,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>[{"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}, {"fall_id": "61", "text": "Schrauben an der Bugnase WE1 mit 40Nm statt 25Nm angezogen. Gewinde teilweise überdreht. Vorgabe im Arbeitsplan wurde von Schicht 1 missachtet.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "mit 40Nm statt 25Nm angezogen. Vorgabe im Arbeitsplan wurde von Schicht 1 missachtet."}, "cot_begruendung": "Das Missachten der Drehmoment-Vorgaben aus dem Arbeitsplan durch die interne Schicht ist ein prozessualer bzw. Montagefehler im Werk. Beschädigte Gewinde müssen nachgearbeitet/ersetzt werden (Nacharbeit)."}, {"fall_id": "13", "text": "Hauptschalter am Dach WE1 löst bei 100A aus, Spezifikation fordert 150A. Alle Schalter der aktuellen Charge von Fa. [Platzhalter] sind betroffen. IBS kann nicht fortgesetzt werden.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Alle Schalter der aktuellen Charge von Fa. [Platzhalter] sind betroffen"}, "cot_begruendung": "Das Bauteil erfüllt nicht die geforderte Spezifikation, was auf einen Materialfehler des externen Lieferanten ('Fa. [Platzhalter]') hinweist. Da die IBS (Inbetriebsetzung) nicht fortgesetzt werden kann, ist dies ein harter Blocker. Der Hinweis 'Alle Schalter der aktuellen Charge' markiert es klar als Serienfehler."}]</t>
+          <t>[{"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"ursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}, {"fall_id": "188", "text": "Diagnose-Software (ZSG) meldet 'Drehgestell 2 fehlt'. Code-Fehler im letzten Software-Update V4.1 des Engineering-Teams unterdrückt die CAN-ID des zweiten Bogies. Zug darf so nicht bewegt werden.", "zielvariablen": {"ursache": "Software", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Code-Fehler im letzten Software-Update V4.1 des Engineering-Teams unterdrückt die CAN-ID"}, "cot_begruendung": "Ein fehlerhafter Code in einem Software-Update durch das Engineering-Team ist ein klassischer Software/Engineering-Fehler. Da eine falsche Diagnose zu einem Bewegungsverbot ('Zug darf so nicht bewegt werden') führt, ist es ein Blocker."}, {"fall_id": "116", "text": "Bremssystem meldet permanent Störung 'Druckverlust', obwohl System dicht ist. Laut Engineering ist die Threshold-Variable in der Brems-Software V3.0 falsch parametriert. Betrifft alle Wagen der aktuellen Tranche. Software-Rollback auf V2.9 zwingend erforderlich, sonst keine Streckenfreigabe.", "zielvariablen": {"ursache": "Software", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Threshold-Variable in der Brems-Software V3.0 falsch parametriert. Betrifft alle Wagen"}, "cot_begruendung": "Der Text beschreibt ein Softwareproblem im Bremssystem, das explizit vom Engineering (falsch parametrierte Variable) verursacht wurde. Da 'alle Wagen der aktuellen Tranche' betroffen sind, liegt ein Serienfehler vor. Ohne funktionierendes Bremssystem gibt es 'keine Streckenfreigabe', weshalb der Fehler als Blocker klassifiziert wird."}]</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>[{"fall_id": "31", "text": "DCU Tür 4 lässt sich nicht flashen. Falsches Skript auf dem Programmiergerät der IBS-Schichtleitung. Keine Tür am Wagen ansteuerbar.", "zielvariablen": {"grundursache": "Software", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Falsches Skript auf dem Programmiergerät der IBS-Schichtleitung. Keine Tür am Wagen ansteuerbar."}, "cot_begruendung": "Ein falsches Skript auf einem internen Programmiergerät ('IBS-Schichtleitung') ist ein lokaler Software/Prozessfehler im Werk. Da keine Tür am Wagen ansteuerbar ist, ist die Inbetriebnahme massiv gestört, was den Fehler als Blocker klassifiziert."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "3", "text": "Kabelbaum für MFA-Display im Fahrerpult ist um 15cm zu kurz. Anschluss an Stecker X45 nicht möglich. Zeichnung laut Herrn [Platzhalter] fehlerhaft, Verlängerung nötig.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Zeichnung laut Herrn [Platzhalter] fehlerhaft"}, "cot_begruendung": "Die Aussage 'Zeichnung [...] fehlerhaft' verweist direkt auf einen Konstruktionsfehler aus dem Engineering. Da das Kabel zum MFA-Display (Fahrerpult) nicht angeschlossen werden kann, ist die Funktion des Zuges nicht gegeben und die Montage blockiert."}]</t>
+          <t>[{"fall_id": "31", "text": "DCU Tür 4 lässt sich nicht flashen. Falsches Skript auf dem Programmiergerät der IBS-Schichtleitung. Keine Tür am Wagen ansteuerbar.", "zielvariablen": {"ursache": "Software", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Falsches Skript auf dem Programmiergerät der IBS-Schichtleitung. Keine Tür am Wagen ansteuerbar."}, "cot_begruendung": "Ein falsches Skript auf einem internen Programmiergerät ('IBS-Schichtleitung') ist ein lokaler Software/Prozessfehler im Werk. Da keine Tür am Wagen ansteuerbar ist, ist die Inbetriebnahme massiv gestört, was den Fehler als Blocker klassifiziert."}, {"fall_id": "101", "text": "Klemmschutz an Fahrgasttür 3 LWS löst viel zu früh aus. Schließvorgang bricht bei leichtem Windstoß ab. Sensorik-Parameter in der neuen Türsoftware (V1.4) von Fa. [Platzhalter] sind zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte angefordert.", "zielvariablen": {"ursache": "Software", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Sensorik-Parameter in der neuen Türsoftware [...] zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte"}, "cot_begruendung": "Der Text beschreibt ein funktionales Problem der Fahrgasttür aufgrund zu empfindlicher Parameter in der 'neuen Türsoftware', welche von einem externen Lieferanten stammt. Da die 'gesamte Flotte' ein Update benötigt, handelt es sich um einen Serienfehler. Ein fehlerhafter Klemmschutz betrifft die Sicherheit und Zuverlässigkeit der Türen, was die Inbetriebnahme blockiert."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}]</t>
         </is>
       </c>
     </row>
@@ -5901,7 +5901,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>[{"fall_id": "85", "text": "Haltegriffe an allen Sitzen im FGR falsch herum montiert. Schicht 3 hat die Einbauanleitung falsch verstanden. Müssen alle gedreht werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "an allen Sitzen im FGR falsch herum montiert. Schicht 3 hat die Einbauanleitung falsch verstanden."}, "cot_begruendung": "Ein Montagefehler durch eine interne Schicht, die die Anleitung falsch verstand, ist eindeutig Montage/Werk. Da 'alle Sitze' betroffen sind, handelt es sich um einen Serienfehler. Das Drehen der Griffe ist eine typische Nacharbeit."}, {"fall_id": "27", "text": "Scheibe RWS im FGR schmierig. Putzkolonne hat falsches Reinigungsmittel verwendet, Schlieren lassen sich schwer entfernen.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Putzkolonne hat falsches Reinigungsmittel verwendet"}, "cot_begruendung": "Die Verschmutzung wurde explizit durch die Putzkolonne ('falsches Reinigungsmittel') verursacht. Dies ist ein Reinigungsfehler im Werk. Da dies weder die Montage aufhält noch ein Bauteil zerstört, wird es als reine Nacharbeit/Info eingestuft."}, {"fall_id": "100", "text": "Schraube M8x20 an Haltestange im FGR WE2 rundgedreht. Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden."}, "cot_begruendung": "Das Runddrehen einer Schraube durch Nutzung eines falschen Bits durch den Werker ist ein Montagefehler im Werk. Das Ausbohren der defekten Schraube ist zeitintensiv, aber eine klassische Nacharbeit, die den Fertigungsablauf nicht komplett stoppt."}]</t>
+          <t>[{"fall_id": "85", "text": "Haltegriffe an allen Sitzen im FGR falsch herum montiert. Schicht 3 hat die Einbauanleitung falsch verstanden. Müssen alle gedreht werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "an allen Sitzen im FGR falsch herum montiert. Schicht 3 hat die Einbauanleitung falsch verstanden."}, "cot_begruendung": "Ein Montagefehler durch eine interne Schicht, die die Anleitung falsch verstand, ist eindeutig Montage/Werk. Da 'alle Sitze' betroffen sind, handelt es sich um einen Serienfehler. Das Drehen der Griffe ist eine typische Nacharbeit."}, {"fall_id": "117", "text": "Befestigung der Sitzkiste RWS im FGR wackelt. Werker hat statt der M8x25 eine M8x40 Schraube mit Gewalt reingedreht und das Gewinde im Boden zerstört. Gewindeeinsatz muss neu gesetzt werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat statt der M8x25 eine M8x40 Schraube mit Gewalt reingedreht"}, "cot_begruendung": "Die Zerstörung des Gewindes durch den Werker (falsche Schraube, Gewaltanwendung) ist ein klarer Montage- und Handhabungsfehler im eigenen Werk. Die Reparatur des Gewindes ist zwar aufwendig, stellt aber einen lokalen Eingriff dar (Nacharbeit)."}, {"fall_id": "27", "text": "Scheibe RWS im FGR schmierig. Putzkolonne hat falsches Reinigungsmittel verwendet, Schlieren lassen sich schwer entfernen.", "zielvariablen": {"ursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Putzkolonne hat falsches Reinigungsmittel verwendet"}, "cot_begruendung": "Die Verschmutzung wurde explizit durch die Putzkolonne ('falsches Reinigungsmittel') verursacht. Dies ist ein Reinigungsfehler im Werk. Da dies weder die Montage aufhält noch ein Bauteil zerstört, wird es als reine Nacharbeit/Info eingestuft."}]</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>[{"fall_id": "8", "text": "Frontmaske hat matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend. Muss poliert/nachlackiert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend"}, "cot_begruendung": "Fehler beim Auftragen des Lacks ('Klarlack teilweise nicht deckend') weisen auf einen Verarbeitungs- bzw. Prozessfehler direkt in der Werksfertigung hin. Dies erfordert eine optische Nacharbeit, stellt aber keine funktionale Blockade dar."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}]</t>
+          <t>[{"fall_id": "152", "text": "Abdeckbleche für die Heizkanäle LWS aus unserer eigenen Stanzerei sind an der Kante um 10 Grad zu wenig abgekantet. Betrifft alle 40 Bleche von heute. Können so nicht montiert werden, Kante steht ab.", "zielvariablen": {"ursache": "Fertigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "aus unserer eigenen Stanzerei sind an der Kante um 10 Grad zu wenig abgekantet. Betrifft alle 40 Bleche"}, "cot_begruendung": "Ein Biegefehler aus der 'eigenen Stanzerei' ist ein interner Fertigungsfehler (Werk). Da 'alle 40 Bleche von heute' betroffen sind, liegt ein Serienfehler vor. Die Bleche müssen nachgebogen werden (Nacharbeit), stoppen aber nicht den kompletten Wagenausbau."}, {"fall_id": "106", "text": "Spaltmaß zwischen den Dachpaneelen im FGR RWS zu gering. Dehnungsausgleich nicht möglich. Laut 3D-Modell in Revision E ist das Paneel 5mm zu lang gezeichnet. QA sperrt den weiteren Deckenausbau.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Laut 3D-Modell in Revision E ist das Paneel 5mm zu lang gezeichnet. QA sperrt den weiteren Deckenausbau."}, "cot_begruendung": "Eine fehlerhafte Längenangabe im 3D-Modell verweist auf einen Konstruktionsfehler durch das Engineering. Die explizite Sperrung des weiteren Deckenausbaus durch die Qualitätsabteilung (QA) stuft dieses Problem als Blocker ein."}, {"fall_id": "8", "text": "Frontmaske hat matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend. Muss poliert/nachlackiert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend"}, "cot_begruendung": "Fehler beim Auftragen des Lacks ('Klarlack teilweise nicht deckend') weisen auf einen Verarbeitungs- bzw. Prozessfehler direkt in der Werksfertigung hin. Dies erfordert eine optische Nacharbeit, stellt aber keine funktionale Blockade dar."}]</t>
         </is>
       </c>
     </row>
@@ -6051,7 +6051,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>[{"fall_id": "58", "text": "Lack zerkratzt.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Lack zerkratzt."}, "cot_begruendung": "Der Text beschreibt lediglich das Symptom 'Lack zerkratzt', liefert jedoch keinen Kontext zur Entstehung (z. B. Transport, unachtsamer Werker, Reinigung). Zur Vermeidung von Halluzinationen muss die Abstention-Logik angewandt und 'Unbekannt' ausgegeben werden."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "75", "text": "Großer Spiegel in der Nasszelle komplett zersplittert. Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang.", "zielvariablen": {"grundursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang."}, "cot_begruendung": "Der durchstoßene Karton im Wareneingang durch einen Gabelstapler ist ein eindeutiger Transportschaden (Logistik). Ein kaputter Spiegel muss bestellt und nachgearbeitet werden, hält den Zugbau aber nicht auf."}]</t>
+          <t>[{"fall_id": "58", "text": "Lack zerkratzt.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Lack zerkratzt."}, "cot_begruendung": "Der Text beschreibt lediglich das Symptom 'Lack zerkratzt', liefert jedoch keinen Kontext zur Entstehung (z. B. Transport, unachtsamer Werker, Reinigung). Zur Vermeidung von Halluzinationen muss die Abstention-Logik angewandt und 'Unbekannt' ausgegeben werden."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "75", "text": "Großer Spiegel in der Nasszelle komplett zersplittert. Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang.", "zielvariablen": {"ursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang."}, "cot_begruendung": "Der durchstoßene Karton im Wareneingang durch einen Gabelstapler ist ein eindeutiger Transportschaden (Logistik). Ein kaputter Spiegel muss bestellt und nachgearbeitet werden, hält den Zugbau aber nicht auf."}]</t>
         </is>
       </c>
     </row>
@@ -6126,7 +6126,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>[{"fall_id": "82", "text": "Tiefer Kratzer auf dem Führerpult. IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen.", "zielvariablen": {"grundursache": "Handhabung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen."}, "cot_begruendung": "Das Fallenlassen des Laptops durch den Mitarbeiter ist ein Handhabungsfehler im eigenen Werk. Optische Kratzer erfordern Nacharbeit (Austausch oder Politur)."}, {"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}, {"fall_id": "42", "text": "Zugsteuerung ZSG bootet nicht. Laut Herrn [Platzhalter] fehlt das gestrige Software-Patch für den CAN-Bus. Gesamte IBS steht aktuell.", "zielvariablen": {"grundursache": "Software", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "fehlt das gestrige Software-Patch für den CAN-Bus. Gesamte IBS steht aktuell"}, "cot_begruendung": "Ein fehlendes Software-Patch für ein Steuergerät, das zentral entwickelt wird, fällt in den Bereich Software/Engineering. Da die 'Gesamte IBS steht', ist der Fehler funktionskritisch und somit eindeutig ein Blocker."}]</t>
+          <t>[{"fall_id": "82", "text": "Tiefer Kratzer auf dem Führerpult. IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "IBS-Mitarbeiter hat sein Diagnose-Laptop versehentlich drauf fallen lassen."}, "cot_begruendung": "Das Fallenlassen des Laptops durch den Mitarbeiter ist ein Handhabungsfehler im eigenen Werk. Optische Kratzer erfordern Nacharbeit (Austausch oder Politur)."}, {"fall_id": "197", "text": "Türen lassen sich nach der IBS nicht zentral schließen. Werker hat versehentlich die veraltete Tür-Software V1.0 von seinem lokalen USB-Stick geflasht, anstatt die freigegebene V1.2 vom Server zu ziehen. Alle Türen am Wagen müssen neu bespielt werden.", "zielvariablen": {"ursache": "Software", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker hat versehentlich die veraltete Tür-Software V1.0 von seinem lokalen USB-Stick geflasht"}, "cot_begruendung": "Das Aufspielen einer falschen/veralteten Software durch den Werker ist ein softwareseitiger und prozessualer Fehler, der direkt im Werk entstanden ist (Software/Werk). Da die sicherheitskritische zentrale Türschließung nicht funktioniert, ist die Inbetriebnahme hart blockiert."}, {"fall_id": "179", "text": "Notbrems-Zugschalter im FGR LWS löst bei Betätigung nicht aus. Werker der Schicht 3 hat Pin 1 und Pin 2 am Stecker X4 vertauscht. Bremsschleife ist dadurch dauerhaft überbrückt. Lebensgefahr!", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker der Schicht 3 hat Pin 1 und Pin 2 am Stecker X4 vertauscht."}, "cot_begruendung": "Vertauschte Pins durch einen Werker der internen Schicht sind ein Montagefehler im Werk. Da eine defekte Notbremse ein sicherheitskritischer Mangel ist, der die Streckenzulassung unmöglich macht, wird dies als Blocker kategorisiert."}]</t>
         </is>
       </c>
     </row>
@@ -6201,7 +6201,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>[{"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}, {"fall_id": "4", "text": "Erdungsband am Triebdrehgestell WE1 links vergessen anzuschrauben. Schraube liegt lose auf dem Rahmen.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "vergessen anzuschrauben"}, "cot_begruendung": "Das vergessene Anschrauben ('Schraube liegt lose auf dem Rahmen') ist ein eindeutiger Montage- und Ausführungsfehler im Werk. Da eine fehlende Erdung am Triebdrehgestell ein massives Sicherheitsrisiko darstellt und die Inbetriebnahme verhindert, ist dies ein Blocker."}, {"fall_id": "21", "text": "Spaltmaß bei Übergangstür WE2 zu groß (&gt;8mm). Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3"}, "cot_begruendung": "Wenn Scharniere physisch nicht weiter justierbar sind, liegt oft ein Toleranz- oder Konstruktionsproblem (Engineering) vor, weniger ein Montagefehler. Der explizite Hinweis auf 'Wagen 1, 2 und 3' ist ein eindeutiger Indikator für einen Serienfehler. Ein falsches Spaltmaß erfordert Nacharbeit."}]</t>
+          <t>[{"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}, {"fall_id": "194", "text": "Massive Klarlacknasen am unteren Rand der Bugmaske WE2. Werker in der Lackierkabine hat die Spritzpistole zu nah gehalten und zu viel Lack aufgetragen. Muss komplett abgeschliffen und neu lackiert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker in der Lackierkabine hat die Spritzpistole zu nah gehalten und zu viel Lack aufgetragen."}, "cot_begruendung": "Falscher Umgang mit der Lackierpistole durch den Werker ist ein handwerklicher Verarbeitungsfehler im eigenen Werk. Abschleifen und Neulackieren ist zwar ärgerlich, aber eine reguläre Nacharbeit."}, {"fall_id": "115", "text": "WLAN-Antenne am Dach schief montiert. Werker hat die Unterlegscheiben asymmetrisch angebracht. Kann im Finish behoben werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat die Unterlegscheiben asymmetrisch angebracht."}, "cot_begruendung": "Das asymmetrische Anbringen von Unterlegscheiben durch den Werker ist ein klarer Montagefehler im Werk. Das Geraderichten im IBS-Finish ist unkritisch und erfordert lediglich Nacharbeit."}]</t>
         </is>
       </c>
     </row>
@@ -6276,7 +6276,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "27", "text": "Scheibe RWS im FGR schmierig. Putzkolonne hat falsches Reinigungsmittel verwendet, Schlieren lassen sich schwer entfernen.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Putzkolonne hat falsches Reinigungsmittel verwendet"}, "cot_begruendung": "Die Verschmutzung wurde explizit durch die Putzkolonne ('falsches Reinigungsmittel') verursacht. Dies ist ein Reinigungsfehler im Werk. Da dies weder die Montage aufhält noch ein Bauteil zerstört, wird es als reine Nacharbeit/Info eingestuft."}, {"fall_id": "38", "text": "Farbnebel auf Haltestange RWS im FGR. Wurde beim Lackieren der Wand nicht richtig abgeklebt.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Wurde beim Lackieren der Wand nicht richtig abgeklebt."}, "cot_begruendung": "Nicht richtiges Abkleben vor dem Lackieren ist ein Verarbeitungs- bzw. Prozessfehler, der direkt in der eigenen Werkstatt passiert ist. Der Farbnebel lässt sich meist einfach entfernen (Info/leichte Nacharbeit)."}]</t>
+          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "27", "text": "Scheibe RWS im FGR schmierig. Putzkolonne hat falsches Reinigungsmittel verwendet, Schlieren lassen sich schwer entfernen.", "zielvariablen": {"ursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Putzkolonne hat falsches Reinigungsmittel verwendet"}, "cot_begruendung": "Die Verschmutzung wurde explizit durch die Putzkolonne ('falsches Reinigungsmittel') verursacht. Dies ist ein Reinigungsfehler im Werk. Da dies weder die Montage aufhält noch ein Bauteil zerstört, wird es als reine Nacharbeit/Info eingestuft."}, {"fall_id": "38", "text": "Farbnebel auf Haltestange RWS im FGR. Wurde beim Lackieren der Wand nicht richtig abgeklebt.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Wurde beim Lackieren der Wand nicht richtig abgeklebt."}, "cot_begruendung": "Nicht richtiges Abkleben vor dem Lackieren ist ein Verarbeitungs- bzw. Prozessfehler, der direkt in der eigenen Werkstatt passiert ist. Der Farbnebel lässt sich meist einfach entfernen (Info/leichte Nacharbeit)."}]</t>
         </is>
       </c>
     </row>
@@ -6351,7 +6351,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>[{"fall_id": "44", "text": "Befestigung der Haltestange im FGR LWS lose. Werker hat vergessen, die Kontermutter anzubringen. Muss dringend nachgezogen werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, die Kontermutter anzubringen"}, "cot_begruendung": "Das explizite Vergessen der Kontermutter durch den Werker ist ein klassischer Montagefehler, der im eigenen Werk entstanden ist. Das Nachziehen der Mutter ist eine unkritische Nacharbeit."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}, {"fall_id": "84", "text": "Isolationsprüfprotokoll für Schaltschrank WE1 unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg. Muss neu gemessen werden.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Isolationsprüfprotokoll [...] unauffindbar. Prüfer hat es gestern unterschrieben abgelegt, aber Dokument ist weg."}, "cot_begruendung": "Ein verschwundenes Prüfprotokoll ist ein administrativer Prozessfehler im Werk. Da das Bauteil selbst funktioniert und nur die Dokumentation fehlt, wird es mit 'Info' flaggt, bis die Neumessung vorliegt."}]</t>
+          <t>[{"fall_id": "44", "text": "Befestigung der Haltestange im FGR LWS lose. Werker hat vergessen, die Kontermutter anzubringen. Muss dringend nachgezogen werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, die Kontermutter anzubringen"}, "cot_begruendung": "Das explizite Vergessen der Kontermutter durch den Werker ist ein klassischer Montagefehler, der im eigenen Werk entstanden ist. Das Nachziehen der Mutter ist eine unkritische Nacharbeit."}, {"fall_id": "173", "text": "Sika-Fuge an der Nasszelle Tür LWS ist komplett verschmiert. Werker hat vergessen, vor dem Spritzen der Dichtmasse abzukleben.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, vor dem Spritzen der Dichtmasse abzukleben."}, "cot_begruendung": "Das Vergessen des Abklebens durch den Werker führt zu einer unsauberen Fuge, was einen Verarbeitungsfehler im eigenen Werk darstellt. Das Entfernen der Schmierer und Neuverfugen ist eine Nacharbeit."}, {"fall_id": "124", "text": "Halterung für Info-Monitor LWS wurde schief montiert, weil der Werker das Bohrloch versetzt angezeichnet hat. Zusätzliche Löcher sichtbar.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "weil der Werker das Bohrloch versetzt angezeichnet hat. Zusätzliche Löcher sichtbar."}, "cot_begruendung": "Das fehlerhafte Anzeichnen der Bohrlöcher durch den Werker ist ein Montagefehler in der eigenen Werkstatt. Die schiefe Halterung und die überflüssigen Löcher erfordern eine Nacharbeit (Bohren korrigieren, Löcher verspachteln)."}]</t>
         </is>
       </c>
     </row>
@@ -6426,7 +6426,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "58", "text": "Lack zerkratzt.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Lack zerkratzt."}, "cot_begruendung": "Der Text beschreibt lediglich das Symptom 'Lack zerkratzt', liefert jedoch keinen Kontext zur Entstehung (z. B. Transport, unachtsamer Werker, Reinigung). Zur Vermeidung von Halluzinationen muss die Abstention-Logik angewandt und 'Unbekannt' ausgegeben werden."}]</t>
+          <t>[{"fall_id": "106", "text": "Spaltmaß zwischen den Dachpaneelen im FGR RWS zu gering. Dehnungsausgleich nicht möglich. Laut 3D-Modell in Revision E ist das Paneel 5mm zu lang gezeichnet. QA sperrt den weiteren Deckenausbau.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Laut 3D-Modell in Revision E ist das Paneel 5mm zu lang gezeichnet. QA sperrt den weiteren Deckenausbau."}, "cot_begruendung": "Eine fehlerhafte Längenangabe im 3D-Modell verweist auf einen Konstruktionsfehler durch das Engineering. Die explizite Sperrung des weiteren Deckenausbaus durch die Qualitätsabteilung (QA) stuft dieses Problem als Blocker ein."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "192", "text": "Blech-Kabelkanal im Unterflurbereich WE1 ist nur 5mm von der beweglichen Achse entfernt. Gemäß EN-Richtlinien müssen hier 25mm Abstand sein. Das CAD-Modell ist hier zu knapp toleriert. EN muss die Zeichnung dringend anpassen.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Das CAD-Modell ist hier zu knapp toleriert. EN muss die Zeichnung dringend anpassen."}, "cot_begruendung": "Eine zu knappe Toleranz im CAD-Modell, die den Richtlinien widerspricht, ist ein Konstruktionsfehler des Engineerings. Da eine Kollision im laufenden Betrieb bei beweglichen Achsen katastrophale Folgen hätte, muss die Anpassung zwingend vor Streckenfreigabe erfolgen (Blocker)."}]</t>
         </is>
       </c>
     </row>
@@ -6501,7 +6501,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>[{"fall_id": "61", "text": "Schrauben an der Bugnase WE1 mit 40Nm statt 25Nm angezogen. Gewinde teilweise überdreht. Vorgabe im Arbeitsplan wurde von Schicht 1 missachtet.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "mit 40Nm statt 25Nm angezogen. Vorgabe im Arbeitsplan wurde von Schicht 1 missachtet."}, "cot_begruendung": "Das Missachten der Drehmoment-Vorgaben aus dem Arbeitsplan durch die interne Schicht ist ein prozessualer bzw. Montagefehler im Werk. Beschädigte Gewinde müssen nachgearbeitet/ersetzt werden (Nacharbeit)."}, {"fall_id": "100", "text": "Schraube M8x20 an Haltestange im FGR WE2 rundgedreht. Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat falschen Bit benutzt. Schraube muss ausgebohrt werden."}, "cot_begruendung": "Das Runddrehen einer Schraube durch Nutzung eines falschen Bits durch den Werker ist ein Montagefehler im Werk. Das Ausbohren der defekten Schraube ist zeitintensiv, aber eine klassische Nacharbeit, die den Fertigungsablauf nicht komplett stoppt."}, {"fall_id": "34", "text": "Spaltmaß an Trennwand FGR zu groß (12mm statt 5mm). Fräse 3 in der Vorfertigung war verstellt. Alle produzierten Holzwände von heute betroffen.", "zielvariablen": {"grundursache": "Fertigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Fräse 3 in der Vorfertigung war verstellt. Alle produzierten Holzwände von heute betroffen."}, "cot_begruendung": "Die Ursache liegt in einer verstellten Maschine ('Fräse 3') während der internen Teileproduktion, was auf Fertigung/Werk hindeutet. Der explizite Hinweis auf 'Alle produzierten Holzwände von heute' flaggt den Fehler eindeutig als Serie. Das Spaltmaß muss durch Nacharbeit korrigiert werden."}]</t>
+          <t>[{"fall_id": "152", "text": "Abdeckbleche für die Heizkanäle LWS aus unserer eigenen Stanzerei sind an der Kante um 10 Grad zu wenig abgekantet. Betrifft alle 40 Bleche von heute. Können so nicht montiert werden, Kante steht ab.", "zielvariablen": {"ursache": "Fertigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "aus unserer eigenen Stanzerei sind an der Kante um 10 Grad zu wenig abgekantet. Betrifft alle 40 Bleche"}, "cot_begruendung": "Ein Biegefehler aus der 'eigenen Stanzerei' ist ein interner Fertigungsfehler (Werk). Da 'alle 40 Bleche von heute' betroffen sind, liegt ein Serienfehler vor. Die Bleche müssen nachgebogen werden (Nacharbeit), stoppen aber nicht den kompletten Wagenausbau."}, {"fall_id": "61", "text": "Schrauben an der Bugnase WE1 mit 40Nm statt 25Nm angezogen. Gewinde teilweise überdreht. Vorgabe im Arbeitsplan wurde von Schicht 1 missachtet.", "zielvariablen": {"ursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "mit 40Nm statt 25Nm angezogen. Vorgabe im Arbeitsplan wurde von Schicht 1 missachtet."}, "cot_begruendung": "Das Missachten der Drehmoment-Vorgaben aus dem Arbeitsplan durch die interne Schicht ist ein prozessualer bzw. Montagefehler im Werk. Beschädigte Gewinde müssen nachgearbeitet/ersetzt werden (Nacharbeit)."}, {"fall_id": "106", "text": "Spaltmaß zwischen den Dachpaneelen im FGR RWS zu gering. Dehnungsausgleich nicht möglich. Laut 3D-Modell in Revision E ist das Paneel 5mm zu lang gezeichnet. QA sperrt den weiteren Deckenausbau.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Laut 3D-Modell in Revision E ist das Paneel 5mm zu lang gezeichnet. QA sperrt den weiteren Deckenausbau."}, "cot_begruendung": "Eine fehlerhafte Längenangabe im 3D-Modell verweist auf einen Konstruktionsfehler durch das Engineering. Die explizite Sperrung des weiteren Deckenausbaus durch die Qualitätsabteilung (QA) stuft dieses Problem als Blocker ein."}]</t>
         </is>
       </c>
     </row>
@@ -6576,7 +6576,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>[{"fall_id": "21", "text": "Spaltmaß bei Übergangstür WE2 zu groß (&gt;8mm). Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3"}, "cot_begruendung": "Wenn Scharniere physisch nicht weiter justierbar sind, liegt oft ein Toleranz- oder Konstruktionsproblem (Engineering) vor, weniger ein Montagefehler. Der explizite Hinweis auf 'Wagen 1, 2 und 3' ist ein eindeutiger Indikator für einen Serienfehler. Ein falsches Spaltmaß erfordert Nacharbeit."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "61", "text": "Schrauben an der Bugnase WE1 mit 40Nm statt 25Nm angezogen. Gewinde teilweise überdreht. Vorgabe im Arbeitsplan wurde von Schicht 1 missachtet.", "zielvariablen": {"grundursache": "Prozess", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "mit 40Nm statt 25Nm angezogen. Vorgabe im Arbeitsplan wurde von Schicht 1 missachtet."}, "cot_begruendung": "Das Missachten der Drehmoment-Vorgaben aus dem Arbeitsplan durch die interne Schicht ist ein prozessualer bzw. Montagefehler im Werk. Beschädigte Gewinde müssen nachgearbeitet/ersetzt werden (Nacharbeit)."}]</t>
+          <t>[{"fall_id": "21", "text": "Spaltmaß bei Übergangstür WE2 zu groß (&gt;8mm). Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3"}, "cot_begruendung": "Wenn Scharniere physisch nicht weiter justierbar sind, liegt oft ein Toleranz- oder Konstruktionsproblem (Engineering) vor, weniger ein Montagefehler. Der explizite Hinweis auf 'Wagen 1, 2 und 3' ist ein eindeutiger Indikator für einen Serienfehler. Ein falsches Spaltmaß erfordert Nacharbeit."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "192", "text": "Blech-Kabelkanal im Unterflurbereich WE1 ist nur 5mm von der beweglichen Achse entfernt. Gemäß EN-Richtlinien müssen hier 25mm Abstand sein. Das CAD-Modell ist hier zu knapp toleriert. EN muss die Zeichnung dringend anpassen.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Das CAD-Modell ist hier zu knapp toleriert. EN muss die Zeichnung dringend anpassen."}, "cot_begruendung": "Eine zu knappe Toleranz im CAD-Modell, die den Richtlinien widerspricht, ist ein Konstruktionsfehler des Engineerings. Da eine Kollision im laufenden Betrieb bei beweglichen Achsen katastrophale Folgen hätte, muss die Anpassung zwingend vor Streckenfreigabe erfolgen (Blocker)."}]</t>
         </is>
       </c>
     </row>
@@ -6651,7 +6651,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "46", "text": "Großer Kratzer auf Trennglas im FGR. Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen"}, "cot_begruendung": "Die Beschädigung wurde direkt durch die Reinigungskraft beim Wischen verursacht (Reinigung/Werk). Ein zerkratztes Glas in der Trennwand muss getauscht werden (Nacharbeit), stoppt aber nicht die Produktion."}]</t>
+          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "46", "text": "Großer Kratzer auf Trennglas im FGR. Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen.", "zielvariablen": {"ursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen"}, "cot_begruendung": "Die Beschädigung wurde direkt durch die Reinigungskraft beim Wischen verursacht (Reinigung/Werk). Ein zerkratztes Glas in der Trennwand muss getauscht werden (Nacharbeit), stoppt aber nicht die Produktion."}]</t>
         </is>
       </c>
     </row>
@@ -6726,7 +6726,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>[{"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}]</t>
+          <t>[{"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}]</t>
         </is>
       </c>
     </row>
@@ -6801,7 +6801,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "46", "text": "Großer Kratzer auf Trennglas im FGR. Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen"}, "cot_begruendung": "Die Beschädigung wurde direkt durch die Reinigungskraft beim Wischen verursacht (Reinigung/Werk). Ein zerkratztes Glas in der Trennwand muss getauscht werden (Nacharbeit), stoppt aber nicht die Produktion."}, {"fall_id": "87", "text": "Riss in der Bremsscheibe WE2 Achse 1. Metallurgische Prüfung zeigt Lunker im Guss. Alle Scheiben der Charge von Fa. [Platzhalter] betroffen. Keine Streckenfreigabe.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Lunker im Guss. Alle Scheiben der Charge von Fa. [Platzhalter] betroffen. Keine Streckenfreigabe."}, "cot_begruendung": "Lunker im Guss bei Lieferung durch eine externe Firma sind ein massiver Materialfehler des Lieferanten. Das Wort 'Charge' kennzeichnet es als Serienfehler. Da sicherheitsrelevante Bremsen betroffen sind und die Streckenfreigabe verweigert wird, ist dies ein absoluter Blocker."}]</t>
+          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "46", "text": "Großer Kratzer auf Trennglas im FGR. Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen.", "zielvariablen": {"ursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen"}, "cot_begruendung": "Die Beschädigung wurde direkt durch die Reinigungskraft beim Wischen verursacht (Reinigung/Werk). Ein zerkratztes Glas in der Trennwand muss getauscht werden (Nacharbeit), stoppt aber nicht die Produktion."}, {"fall_id": "173", "text": "Sika-Fuge an der Nasszelle Tür LWS ist komplett verschmiert. Werker hat vergessen, vor dem Spritzen der Dichtmasse abzukleben.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, vor dem Spritzen der Dichtmasse abzukleben."}, "cot_begruendung": "Das Vergessen des Abklebens durch den Werker führt zu einer unsauberen Fuge, was einen Verarbeitungsfehler im eigenen Werk darstellt. Das Entfernen der Schmierer und Neuverfugen ist eine Nacharbeit."}]</t>
         </is>
       </c>
     </row>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>[{"fall_id": "22", "text": "Fahrgasttür RWS öffnet nicht bei Tasterbetätigung. DCU gibt keinen Befehl raus. Ersatzteil aus Lager geholt, Tür funktioniert wieder. Defekte DCU geht an Lieferant retour.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "DCU gibt keinen Befehl raus. [...] Defekte DCU geht an Lieferant retour"}, "cot_begruendung": "Die Door Control Unit (DCU) ist intern defekt, was auf einen Materialfehler des Lieferanten schließen lässt. Da das Ersatzteil sofort aus dem Lager verfügbar war und die Produktion nicht gestoppt wurde, bleibt es bei einer Nacharbeit."}, {"fall_id": "44", "text": "Befestigung der Haltestange im FGR LWS lose. Werker hat vergessen, die Kontermutter anzubringen. Muss dringend nachgezogen werden.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, die Kontermutter anzubringen"}, "cot_begruendung": "Das explizite Vergessen der Kontermutter durch den Werker ist ein klassischer Montagefehler, der im eigenen Werk entstanden ist. Das Nachziehen der Mutter ist eine unkritische Nacharbeit."}, {"fall_id": "23", "text": "Wagennummer außen am Führerstand fehlt. Aufkleber ist nicht aufgetaucht, vermutlich auf dem Postweg verloren.", "zielvariablen": {"grundursache": "Logistik", "ursprung": "Logistik", "kritikalitaet": "Info", "serie": false, "text_snippet": "Aufkleber ist nicht aufgetaucht, vermutlich auf dem Postweg verloren"}, "cot_begruendung": "Das Fehlen von Aufklebern wegen Verlust auf dem Versandweg ist ein klassisches Logistik-Problem. Ein fehlender Aufkleber blockiert die technische Inbetriebsetzung nicht, weshalb es als 'Info' verbucht wird, bis das Ersatzteil eintrifft."}]</t>
+          <t>[{"fall_id": "22", "text": "Fahrgasttür RWS öffnet nicht bei Tasterbetätigung. DCU gibt keinen Befehl raus. Ersatzteil aus Lager geholt, Tür funktioniert wieder. Defekte DCU geht an Lieferant retour.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "DCU gibt keinen Befehl raus. [...] Defekte DCU geht an Lieferant retour"}, "cot_begruendung": "Die Door Control Unit (DCU) ist intern defekt, was auf einen Materialfehler des Lieferanten schließen lässt. Da das Ersatzteil sofort aus dem Lager verfügbar war und die Produktion nicht gestoppt wurde, bleibt es bei einer Nacharbeit."}, {"fall_id": "101", "text": "Klemmschutz an Fahrgasttür 3 LWS löst viel zu früh aus. Schließvorgang bricht bei leichtem Windstoß ab. Sensorik-Parameter in der neuen Türsoftware (V1.4) von Fa. [Platzhalter] sind zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte angefordert.", "zielvariablen": {"ursache": "Software", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Sensorik-Parameter in der neuen Türsoftware [...] zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte"}, "cot_begruendung": "Der Text beschreibt ein funktionales Problem der Fahrgasttür aufgrund zu empfindlicher Parameter in der 'neuen Türsoftware', welche von einem externen Lieferanten stammt. Da die 'gesamte Flotte' ein Update benötigt, handelt es sich um einen Serienfehler. Ein fehlerhafter Klemmschutz betrifft die Sicherheit und Zuverlässigkeit der Türen, was die Inbetriebnahme blockiert."}, {"fall_id": "44", "text": "Befestigung der Haltestange im FGR LWS lose. Werker hat vergessen, die Kontermutter anzubringen. Muss dringend nachgezogen werden.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker hat vergessen, die Kontermutter anzubringen"}, "cot_begruendung": "Das explizite Vergessen der Kontermutter durch den Werker ist ein klassischer Montagefehler, der im eigenen Werk entstanden ist. Das Nachziehen der Mutter ist eine unkritische Nacharbeit."}]</t>
         </is>
       </c>
     </row>
@@ -6951,7 +6951,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>[{"fall_id": "79", "text": "Sitzbezüge im gesamten Wagen reißen an der Naht ein. Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge müssen getauscht werden.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge"}, "cot_begruendung": "Die mangelhafte Stoffqualität eines externen Lieferanten ist ein Materialfehler. Die Bemerkungen 'gesamter Wagen' und 'neuen Serie' verweisen auf einen Serienfehler. Das Austauschen der Bezüge ist Nacharbeit, aber kein Blocker für Inbetriebsetzungen."}, {"fall_id": "73", "text": "Falsche Schrauben (M6 statt M8) für die Sitzbefestigung im gesamten FGR geliefert. Betrifft die Charge von Zulieferer [Platzhalter]. Keine Sitze können montiert werden.", "zielvariablen": {"grundursache": "Logistik", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Betrifft die Charge von Zulieferer [Platzhalter]. Keine Sitze können montiert werden."}, "cot_begruendung": "Eine Falschlieferung von Schrauben durch den Zulieferer ist ein Logistik-/Lieferantenproblem. Das Wort 'Charge' kennzeichnet das Problem als Serienfehler. Da die Sitzmontage komplett blockiert ist, liegt ein Blocker vor."}, {"fall_id": "8", "text": "Frontmaske hat matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend. Muss poliert/nachlackiert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "matte Stellen nach der Lackierung. Klarlack teilweise nicht deckend"}, "cot_begruendung": "Fehler beim Auftragen des Lacks ('Klarlack teilweise nicht deckend') weisen auf einen Verarbeitungs- bzw. Prozessfehler direkt in der Werksfertigung hin. Dies erfordert eine optische Nacharbeit, stellt aber keine funktionale Blockade dar."}]</t>
+          <t>[{"fall_id": "148", "text": "Sitzgestell wackelt.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Sitzgestell wackelt."}, "cot_begruendung": "Nur das Symptom 'wackelt' ist gegeben. Ob der Werker Schrauben vergessen hat, die Bohrungen falsch gesetzt sind oder das Gestell vom Lieferanten verzogen ist, ist nicht ersichtlich. Causal Faithfulness verlangt hier die Abstention (Unbekannt)."}, {"fall_id": "126", "text": "Alle C-Schienen zur Befestigung der Sitze aus unserer internen Fräserei sind um 5mm zu schmal gefräst worden. Maß in der Maschine war falsch eingestellt. Keine Sitze im Wagen 3 montierbar.", "zielvariablen": {"ursache": "Fertigung", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "aus unserer internen Fräserei sind um 5mm zu schmal gefräst worden. Maß in der Maschine war falsch eingestellt."}, "cot_begruendung": "Falsch gefräste Bauteile aus der 'internen Fräserei' aufgrund einer falsch eingestellten Maschine sind ein Fertigungsfehler im Werk. Da 'Alle C-Schienen' betroffen sind, ist es ein Serienproblem. Dass keine Sitze verbaut werden können, zieht einen Produktionsstopp nach sich (Blocker)."}, {"fall_id": "79", "text": "Sitzbezüge im gesamten Wagen reißen an der Naht ein. Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge müssen getauscht werden.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge"}, "cot_begruendung": "Die mangelhafte Stoffqualität eines externen Lieferanten ist ein Materialfehler. Die Bemerkungen 'gesamter Wagen' und 'neuen Serie' verweisen auf einen Serienfehler. Das Austauschen der Bezüge ist Nacharbeit, aber kein Blocker für Inbetriebsetzungen."}]</t>
         </is>
       </c>
     </row>
@@ -7026,7 +7026,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>[{"fall_id": "21", "text": "Spaltmaß bei Übergangstür WE2 zu groß (&gt;8mm). Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3"}, "cot_begruendung": "Wenn Scharniere physisch nicht weiter justierbar sind, liegt oft ein Toleranz- oder Konstruktionsproblem (Engineering) vor, weniger ein Montagefehler. Der explizite Hinweis auf 'Wagen 1, 2 und 3' ist ein eindeutiger Indikator für einen Serienfehler. Ein falsches Spaltmaß erfordert Nacharbeit."}, {"fall_id": "79", "text": "Sitzbezüge im gesamten Wagen reißen an der Naht ein. Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge müssen getauscht werden.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge"}, "cot_begruendung": "Die mangelhafte Stoffqualität eines externen Lieferanten ist ein Materialfehler. Die Bemerkungen 'gesamter Wagen' und 'neuen Serie' verweisen auf einen Serienfehler. Das Austauschen der Bezüge ist Nacharbeit, aber kein Blocker für Inbetriebsetzungen."}, {"fall_id": "23", "text": "Wagennummer außen am Führerstand fehlt. Aufkleber ist nicht aufgetaucht, vermutlich auf dem Postweg verloren.", "zielvariablen": {"grundursache": "Logistik", "ursprung": "Logistik", "kritikalitaet": "Info", "serie": false, "text_snippet": "Aufkleber ist nicht aufgetaucht, vermutlich auf dem Postweg verloren"}, "cot_begruendung": "Das Fehlen von Aufklebern wegen Verlust auf dem Versandweg ist ein klassisches Logistik-Problem. Ein fehlender Aufkleber blockiert die technische Inbetriebsetzung nicht, weshalb es als 'Info' verbucht wird, bis das Ersatzteil eintrifft."}]</t>
+          <t>[{"fall_id": "141", "text": "Erdungsband am Hochspannungsschrank WE1 nicht verschraubt, hängt lose herab. Werker hat es vergessen anzuschließen. Lebensgefahr beim Einschalten der Fahrleitungsspannung!", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker hat es vergessen anzuschließen. Lebensgefahr beim Einschalten"}, "cot_begruendung": "Das Vergessen des Erdungsbandes durch den Werker ist ein klassischer Montagefehler im eigenen Werk. Da eine lose Erdung an einem Hochspannungsschrank absolute Lebensgefahr bedeutet und die IBS verhindert, ist es ein kritischer Blocker."}, {"fall_id": "101", "text": "Klemmschutz an Fahrgasttür 3 LWS löst viel zu früh aus. Schließvorgang bricht bei leichtem Windstoß ab. Sensorik-Parameter in der neuen Türsoftware (V1.4) von Fa. [Platzhalter] sind zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte angefordert.", "zielvariablen": {"ursache": "Software", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Sensorik-Parameter in der neuen Türsoftware [...] zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte"}, "cot_begruendung": "Der Text beschreibt ein funktionales Problem der Fahrgasttür aufgrund zu empfindlicher Parameter in der 'neuen Türsoftware', welche von einem externen Lieferanten stammt. Da die 'gesamte Flotte' ein Update benötigt, handelt es sich um einen Serienfehler. Ein fehlerhafter Klemmschutz betrifft die Sicherheit und Zuverlässigkeit der Türen, was die Inbetriebnahme blockiert."}, {"fall_id": "21", "text": "Spaltmaß bei Übergangstür WE2 zu groß (&gt;8mm). Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3"}, "cot_begruendung": "Wenn Scharniere physisch nicht weiter justierbar sind, liegt oft ein Toleranz- oder Konstruktionsproblem (Engineering) vor, weniger ein Montagefehler. Der explizite Hinweis auf 'Wagen 1, 2 und 3' ist ein eindeutiger Indikator für einen Serienfehler. Ein falsches Spaltmaß erfordert Nacharbeit."}]</t>
         </is>
       </c>
     </row>
@@ -7101,7 +7101,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>[{"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "75", "text": "Großer Spiegel in der Nasszelle komplett zersplittert. Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang.", "zielvariablen": {"grundursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang."}, "cot_begruendung": "Der durchstoßene Karton im Wareneingang durch einen Gabelstapler ist ein eindeutiger Transportschaden (Logistik). Ein kaputter Spiegel muss bestellt und nachgearbeitet werden, hält den Zugbau aber nicht auf."}]</t>
+          <t>[{"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "75", "text": "Großer Spiegel in der Nasszelle komplett zersplittert. Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang.", "zielvariablen": {"ursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang."}, "cot_begruendung": "Der durchstoßene Karton im Wareneingang durch einen Gabelstapler ist ein eindeutiger Transportschaden (Logistik). Ein kaputter Spiegel muss bestellt und nachgearbeitet werden, hält den Zugbau aber nicht auf."}]</t>
         </is>
       </c>
     </row>
@@ -7176,7 +7176,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>[{"fall_id": "21", "text": "Spaltmaß bei Übergangstür WE2 zu groß (&gt;8mm). Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3"}, "cot_begruendung": "Wenn Scharniere physisch nicht weiter justierbar sind, liegt oft ein Toleranz- oder Konstruktionsproblem (Engineering) vor, weniger ein Montagefehler. Der explizite Hinweis auf 'Wagen 1, 2 und 3' ist ein eindeutiger Indikator für einen Serienfehler. Ein falsches Spaltmaß erfordert Nacharbeit."}, {"fall_id": "87", "text": "Riss in der Bremsscheibe WE2 Achse 1. Metallurgische Prüfung zeigt Lunker im Guss. Alle Scheiben der Charge von Fa. [Platzhalter] betroffen. Keine Streckenfreigabe.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Lunker im Guss. Alle Scheiben der Charge von Fa. [Platzhalter] betroffen. Keine Streckenfreigabe."}, "cot_begruendung": "Lunker im Guss bei Lieferung durch eine externe Firma sind ein massiver Materialfehler des Lieferanten. Das Wort 'Charge' kennzeichnet es als Serienfehler. Da sicherheitsrelevante Bremsen betroffen sind und die Streckenfreigabe verweigert wird, ist dies ein absoluter Blocker."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}]</t>
+          <t>[{"fall_id": "21", "text": "Spaltmaß bei Übergangstür WE2 zu groß (&gt;8mm). Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3"}, "cot_begruendung": "Wenn Scharniere physisch nicht weiter justierbar sind, liegt oft ein Toleranz- oder Konstruktionsproblem (Engineering) vor, weniger ein Montagefehler. Der explizite Hinweis auf 'Wagen 1, 2 und 3' ist ein eindeutiger Indikator für einen Serienfehler. Ein falsches Spaltmaß erfordert Nacharbeit."}, {"fall_id": "87", "text": "Riss in der Bremsscheibe WE2 Achse 1. Metallurgische Prüfung zeigt Lunker im Guss. Alle Scheiben der Charge von Fa. [Platzhalter] betroffen. Keine Streckenfreigabe.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Lunker im Guss. Alle Scheiben der Charge von Fa. [Platzhalter] betroffen. Keine Streckenfreigabe."}, "cot_begruendung": "Lunker im Guss bei Lieferung durch eine externe Firma sind ein massiver Materialfehler des Lieferanten. Das Wort 'Charge' kennzeichnet es als Serienfehler. Da sicherheitsrelevante Bremsen betroffen sind und die Streckenfreigabe verweigert wird, ist dies ein absoluter Blocker."}, {"fall_id": "194", "text": "Massive Klarlacknasen am unteren Rand der Bugmaske WE2. Werker in der Lackierkabine hat die Spritzpistole zu nah gehalten und zu viel Lack aufgetragen. Muss komplett abgeschliffen und neu lackiert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Werker in der Lackierkabine hat die Spritzpistole zu nah gehalten und zu viel Lack aufgetragen."}, "cot_begruendung": "Falscher Umgang mit der Lackierpistole durch den Werker ist ein handwerklicher Verarbeitungsfehler im eigenen Werk. Abschleifen und Neulackieren ist zwar ärgerlich, aber eine reguläre Nacharbeit."}]</t>
         </is>
       </c>
     </row>
@@ -7251,7 +7251,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>[{"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}]</t>
+          <t>[{"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}]</t>
         </is>
       </c>
     </row>
@@ -7326,7 +7326,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>[{"fall_id": "79", "text": "Sitzbezüge im gesamten Wagen reißen an der Naht ein. Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge müssen getauscht werden.", "zielvariablen": {"grundursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge"}, "cot_begruendung": "Die mangelhafte Stoffqualität eines externen Lieferanten ist ein Materialfehler. Die Bemerkungen 'gesamter Wagen' und 'neuen Serie' verweisen auf einen Serienfehler. Das Austauschen der Bezüge ist Nacharbeit, aber kein Blocker für Inbetriebsetzungen."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "73", "text": "Falsche Schrauben (M6 statt M8) für die Sitzbefestigung im gesamten FGR geliefert. Betrifft die Charge von Zulieferer [Platzhalter]. Keine Sitze können montiert werden.", "zielvariablen": {"grundursache": "Logistik", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Betrifft die Charge von Zulieferer [Platzhalter]. Keine Sitze können montiert werden."}, "cot_begruendung": "Eine Falschlieferung von Schrauben durch den Zulieferer ist ein Logistik-/Lieferantenproblem. Das Wort 'Charge' kennzeichnet das Problem als Serienfehler. Da die Sitzmontage komplett blockiert ist, liegt ein Blocker vor."}]</t>
+          <t>[{"fall_id": "79", "text": "Sitzbezüge im gesamten Wagen reißen an der Naht ein. Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge müssen getauscht werden.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Stoffqualität der neuen Serie von Fa. [Platzhalter] ist mangelhaft. Alle Bezüge"}, "cot_begruendung": "Die mangelhafte Stoffqualität eines externen Lieferanten ist ein Materialfehler. Die Bemerkungen 'gesamter Wagen' und 'neuen Serie' verweisen auf einen Serienfehler. Das Austauschen der Bezüge ist Nacharbeit, aber kein Blocker für Inbetriebsetzungen."}, {"fall_id": "199", "text": "Deutliche Kugelschreiber-Striche auf dem neuen Ledersitz der 1. Klasse. Projektleiter hat bei der Kundenbegehung ohne Unterlage auf dem Sitz seine Notizen geschrieben und dabei durchgedrückt.", "zielvariablen": {"ursache": "Handhabung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Projektleiter hat bei der Kundenbegehung ohne Unterlage auf dem Sitz seine Notizen geschrieben"}, "cot_begruendung": "Der Schaden wurde durch unvorsichtige Handhabung von internem Personal (Projektleiter) verursacht. Dies fällt in die Kategorie Handhabung im Werk/Unternehmen. Der verschmutzte oder beschädigte Bezug muss gereinigt bzw. ausgetauscht werden (Nacharbeit)."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
         </is>
       </c>
     </row>
@@ -7401,7 +7401,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "58", "text": "Lack zerkratzt.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Lack zerkratzt."}, "cot_begruendung": "Der Text beschreibt lediglich das Symptom 'Lack zerkratzt', liefert jedoch keinen Kontext zur Entstehung (z. B. Transport, unachtsamer Werker, Reinigung). Zur Vermeidung von Halluzinationen muss die Abstention-Logik angewandt und 'Unbekannt' ausgegeben werden."}]</t>
+          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "58", "text": "Lack zerkratzt.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Lack zerkratzt."}, "cot_begruendung": "Der Text beschreibt lediglich das Symptom 'Lack zerkratzt', liefert jedoch keinen Kontext zur Entstehung (z. B. Transport, unachtsamer Werker, Reinigung). Zur Vermeidung von Halluzinationen muss die Abstention-Logik angewandt und 'Unbekannt' ausgegeben werden."}]</t>
         </is>
       </c>
     </row>
@@ -7476,7 +7476,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>[{"fall_id": "75", "text": "Großer Spiegel in der Nasszelle komplett zersplittert. Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang.", "zielvariablen": {"grundursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang."}, "cot_begruendung": "Der durchstoßene Karton im Wareneingang durch einen Gabelstapler ist ein eindeutiger Transportschaden (Logistik). Ein kaputter Spiegel muss bestellt und nachgearbeitet werden, hält den Zugbau aber nicht auf."}, {"fall_id": "46", "text": "Großer Kratzer auf Trennglas im FGR. Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen"}, "cot_begruendung": "Die Beschädigung wurde direkt durch die Reinigungskraft beim Wischen verursacht (Reinigung/Werk). Ein zerkratztes Glas in der Trennwand muss getauscht werden (Nacharbeit), stoppt aber nicht die Produktion."}, {"fall_id": "63", "text": "Kurzschluss im Taster für WC-Spülung WE2. Reinigungstrupp hat mit Hochdruckreiniger direkt in den Taster gesprüht, Wasser im Gehäuse.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Reinigungstrupp hat mit Hochdruckreiniger direkt in den Taster gesprüht"}, "cot_begruendung": "Die Zerstörung des Tasters durch unsachgemäßen Einsatz eines Hochdruckreinigers ist eindeutig der Reinigung im Werk (Verursacher) zuzuschreiben. Ein defekter Spülungstaster muss getauscht werden (Nacharbeit)."}]</t>
+          <t>[{"fall_id": "104", "text": "Wischwasserbehälter WE1 undicht. Schweißnaht am Kunststoffgehäuse hat Haarrisse. Offenbar Produktionsfehler vom Hersteller. Tropft auf die darunterliegende Elektrik. Sofortiger Tausch nötig.", "zielvariablen": {"ursache": "Material", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Schweißnaht am Kunststoffgehäuse hat Haarrisse. Offenbar Produktionsfehler vom Hersteller."}, "cot_begruendung": "Ein undichter Behälter aufgrund von Haarrissen in der Schweißnaht ab Werk ist ein Materialfehler, der vom Hersteller (Lieferant) verursacht wurde. Da das Wasser auf die Elektrik tropft und ein sofortiger Tausch gefordert wird, liegt eine hohe Kritikalität (Blocker) vor."}, {"fall_id": "162", "text": "Graue Flecken auf dem neuen Fußbodenbelag im FGR. Reinigungskraft hat den Spezialreiniger nicht richtig verdünnt, wodurch Rückstände beim Trocknen entstanden sind. Einmal feucht nachwischen behebt das Problem.", "zielvariablen": {"ursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Reinigungskraft hat den Spezialreiniger nicht richtig verdünnt"}, "cot_begruendung": "Falsche Dosierung des Reinigungsmittels durch die Reinigungskraft ist ein klassischer Fehler der internen Reinigung (Werk). Da sich der Mangel durch simples Nachwischen beheben lässt, wird er als 'Info' oder sehr leichte Nacharbeit deklariert."}, {"fall_id": "75", "text": "Großer Spiegel in der Nasszelle komplett zersplittert. Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang.", "zielvariablen": {"ursache": "Transport", "ursprung": "Logistik", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Karton war durch Gabelstaplergabel durchstoßen worden bei Entladung im Wareneingang."}, "cot_begruendung": "Der durchstoßene Karton im Wareneingang durch einen Gabelstapler ist ein eindeutiger Transportschaden (Logistik). Ein kaputter Spiegel muss bestellt und nachgearbeitet werden, hält den Zugbau aber nicht auf."}]</t>
         </is>
       </c>
     </row>
@@ -7551,7 +7551,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>[{"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}]</t>
+          <t>[{"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}, {"fall_id": "101", "text": "Klemmschutz an Fahrgasttür 3 LWS löst viel zu früh aus. Schließvorgang bricht bei leichtem Windstoß ab. Sensorik-Parameter in der neuen Türsoftware (V1.4) von Fa. [Platzhalter] sind zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte angefordert.", "zielvariablen": {"ursache": "Software", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Sensorik-Parameter in der neuen Türsoftware [...] zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte"}, "cot_begruendung": "Der Text beschreibt ein funktionales Problem der Fahrgasttür aufgrund zu empfindlicher Parameter in der 'neuen Türsoftware', welche von einem externen Lieferanten stammt. Da die 'gesamte Flotte' ein Update benötigt, handelt es sich um einen Serienfehler. Ein fehlerhafter Klemmschutz betrifft die Sicherheit und Zuverlässigkeit der Türen, was die Inbetriebnahme blockiert."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}]</t>
         </is>
       </c>
     </row>
@@ -7626,7 +7626,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>[{"fall_id": "21", "text": "Spaltmaß bei Übergangstür WE2 zu groß (&gt;8mm). Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3"}, "cot_begruendung": "Wenn Scharniere physisch nicht weiter justierbar sind, liegt oft ein Toleranz- oder Konstruktionsproblem (Engineering) vor, weniger ein Montagefehler. Der explizite Hinweis auf 'Wagen 1, 2 und 3' ist ein eindeutiger Indikator für einen Serienfehler. Ein falsches Spaltmaß erfordert Nacharbeit."}, {"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}, {"fall_id": "55", "text": "Schleifspuren im Lack an Seitenwand LWS sichtbar. Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Exzenter-Schleifer in der Lackierkabine wurde mit falscher Körnung bestückt."}, "cot_begruendung": "Die falsche Bestückung des Schleifers in der internen Lackierkabine ist ein prozessualer Verarbeitungsfehler im Werk. Optische Mängel wie Schleifspuren erfordern in der Regel nur eine Politur/Nacharbeit und werden daher als Info oder Nacharbeit gekennzeichnet."}]</t>
+          <t>[{"fall_id": "21", "text": "Spaltmaß bei Übergangstür WE2 zu groß (&gt;8mm). Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Scharniere lassen sich nicht weiter justieren. Wiederholt sich bei Wagen 1, 2 und 3"}, "cot_begruendung": "Wenn Scharniere physisch nicht weiter justierbar sind, liegt oft ein Toleranz- oder Konstruktionsproblem (Engineering) vor, weniger ein Montagefehler. Der explizite Hinweis auf 'Wagen 1, 2 und 3' ist ein eindeutiger Indikator für einen Serienfehler. Ein falsches Spaltmaß erfordert Nacharbeit."}, {"fall_id": "101", "text": "Klemmschutz an Fahrgasttür 3 LWS löst viel zu früh aus. Schließvorgang bricht bei leichtem Windstoß ab. Sensorik-Parameter in der neuen Türsoftware (V1.4) von Fa. [Platzhalter] sind zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte angefordert.", "zielvariablen": {"ursache": "Software", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": true, "text_snippet": "Sensorik-Parameter in der neuen Türsoftware [...] zu empfindlich eingestellt. Update auf V1.5 für gesamte Flotte"}, "cot_begruendung": "Der Text beschreibt ein funktionales Problem der Fahrgasttür aufgrund zu empfindlicher Parameter in der 'neuen Türsoftware', welche von einem externen Lieferanten stammt. Da die 'gesamte Flotte' ein Update benötigt, handelt es sich um einen Serienfehler. Ein fehlerhafter Klemmschutz betrifft die Sicherheit und Zuverlässigkeit der Türen, was die Inbetriebnahme blockiert."}, {"fall_id": "9", "text": "Schiebetritt fährt nicht vollständig aus. Kollidiert mit Türrahmen LWS. Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft.", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "Bei allen Türen auf der linken Seite. Einstellung KKDU durch Werker fehlerhaft."}, "cot_begruendung": "Die fehlerhafte Einstellung ('Einstellung KKDU durch Werker fehlerhaft') ist eindeutig auf die Montage im Werk zurückzuführen. Der Hinweis 'Bei allen Türen auf der linken Seite' flaggt den Fehler als Serienthema auf diesem Wagen. Die Einstellung muss korrigiert werden (Nacharbeit)."}]</t>
         </is>
       </c>
     </row>
@@ -7701,7 +7701,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}]</t>
+          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}]</t>
         </is>
       </c>
     </row>
@@ -7776,7 +7776,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>[{"fall_id": "58", "text": "Lack zerkratzt.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Lack zerkratzt."}, "cot_begruendung": "Der Text beschreibt lediglich das Symptom 'Lack zerkratzt', liefert jedoch keinen Kontext zur Entstehung (z. B. Transport, unachtsamer Werker, Reinigung). Zur Vermeidung von Halluzinationen muss die Abstention-Logik angewandt und 'Unbekannt' ausgegeben werden."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
+          <t>[{"fall_id": "58", "text": "Lack zerkratzt.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Lack zerkratzt."}, "cot_begruendung": "Der Text beschreibt lediglich das Symptom 'Lack zerkratzt', liefert jedoch keinen Kontext zur Entstehung (z. B. Transport, unachtsamer Werker, Reinigung). Zur Vermeidung von Halluzinationen muss die Abstention-Logik angewandt und 'Unbekannt' ausgegeben werden."}, {"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
         </is>
       </c>
     </row>
@@ -7851,7 +7851,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>[{"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "62", "text": "Kabelkanal unterflur kollidiert mit der Druckluftleitung für die Bremsanlage. Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich.", "zielvariablen": {"grundursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Zeichnungsrevision B vom Engineering weist hier eine Überlappung der Bauteile auf. Rohrverlegung aktuell unmöglich."}, "cot_begruendung": "Eine Überlappung im 3D-Modell/Zeichnung ist ein Konstruktionsfehler aus dem Engineering. Da die Druckluftleitung für die Bremsen essenziell ist und die 'Rohrverlegung aktuell unmöglich' ist, handelt es sich um einen harten Blocker."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
+          <t>[{"fall_id": "172", "text": "Kabelbinder (schwarz, 300mm) fehlen komplett am Arbeitsplatz für die Unterflurverkabelung. Dispo hat im System den Meldebestand nicht richtig gepflegt, Lager ist leer. Kommen erst am Nachmittag.", "zielvariablen": {"ursache": "Software", "ursprung": "Logistik", "kritikalitaet": "Info", "serie": false, "text_snippet": "Dispo hat im System den Meldebestand nicht richtig gepflegt, Lager ist leer."}, "cot_begruendung": "Das Fehlen von C-Teilen aufgrund einer fehlerhaften Systempflege im ERP/Dispo-System ist ein softwareseitiges bzw. administratives Problem der internen Logistik. Kabelbinder sind temporär ersetzbar oder leicht nachzurüsten, weshalb der Ausbau meist nicht komplett steht (Info)."}, {"fall_id": "47", "text": "Deckenklappe über Gang lässt sich nicht schließen, Spaltmaß ca. 15mm. Kollision mit neuem Kabelstrang der Brandmeldeanlage, Zeichnungstoleranz hier viel zu eng.", "zielvariablen": {"ursache": "Konstruktion", "ursprung": "Engineering", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Zeichnungstoleranz hier viel zu eng."}, "cot_begruendung": "Die zu enge 'Zeichnungstoleranz' ist die Grundursache für die Kollision und fällt in die Verantwortung der Konstruktion (Engineering). Die Klappe muss nachgearbeitet/angepasst werden, was die generelle Fertigung aber nicht blockiert."}, {"fall_id": "141", "text": "Erdungsband am Hochspannungsschrank WE1 nicht verschraubt, hängt lose herab. Werker hat es vergessen anzuschließen. Lebensgefahr beim Einschalten der Fahrleitungsspannung!", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker hat es vergessen anzuschließen. Lebensgefahr beim Einschalten"}, "cot_begruendung": "Das Vergessen des Erdungsbandes durch den Werker ist ein klassischer Montagefehler im eigenen Werk. Da eine lose Erdung an einem Hochspannungsschrank absolute Lebensgefahr bedeutet und die IBS verhindert, ist es ein kritischer Blocker."}]</t>
         </is>
       </c>
     </row>
@@ -7926,7 +7926,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>[{"fall_id": "96", "text": "Kabel für Zugsicherungssystem PZB fehlen. Lieferant hat Lieferengpass für die Spezialstecker. Ohne PZB keine dynamische IBS möglich.", "zielvariablen": {"grundursache": "Logistik", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Lieferant hat Lieferengpass für die Spezialstecker. Ohne PZB keine dynamische IBS möglich."}, "cot_begruendung": "Ein Lieferengpass beim externen Zulieferer ist ein logistisches Problem (Lieferant). Da fehlende Zugsicherungskabel die fahrdynamische IBS unmöglich machen, liegt ein kritischer Blocker vor."}, {"fall_id": "70", "text": "Anschlusskabel für Notbremsschalter im FGR zu kurz geschnitten. Werker hat den Kabelstrang nicht wie vorgeschrieben in Schleife gelegt, sondern direkt gezogen. Neuverkabelung der halben Seite LWS nötig.", "zielvariablen": {"grundursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker hat den Kabelstrang nicht wie vorgeschrieben in Schleife gelegt, sondern direkt gezogen. Neuverkabelung der halben Seite LWS nötig."}, "cot_begruendung": "Der Werker hat den Kabelstrang falsch verlegt (nicht in Schleife), was einen Montagefehler im Werk darstellt. Da sicherheitsrelevante Notbremsschalter betroffen sind und die halbe Seite neu verkabelt werden muss, ist dies ein massiver Verzug und somit ein Blocker."}, {"fall_id": "26", "text": "Hauptkabelstrang HKS-3 unterflur am Drehgestell WE2 durchtrennt. Staplerfahrer hat beim Abladen der Palette reingestochen. Kabelbaum muss komplett neu.", "zielvariablen": {"grundursache": "Handhabung", "ursprung": "Logistik", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Staplerfahrer hat beim Abladen der Palette reingestochen"}, "cot_begruendung": "Der Text beschreibt eindeutig eine mechanische Beschädigung durch einen Staplerfahrer beim Abladen. Dies ist ein Handhabungsfehler, der der Logistik zuzuordnen ist. Da der Hauptkabelstrang komplett neu muss, kann das Fahrzeug elektrisch nicht in Betrieb genommen werden (Blocker)."}]</t>
+          <t>[{"fall_id": "172", "text": "Kabelbinder (schwarz, 300mm) fehlen komplett am Arbeitsplatz für die Unterflurverkabelung. Dispo hat im System den Meldebestand nicht richtig gepflegt, Lager ist leer. Kommen erst am Nachmittag.", "zielvariablen": {"ursache": "Software", "ursprung": "Logistik", "kritikalitaet": "Info", "serie": false, "text_snippet": "Dispo hat im System den Meldebestand nicht richtig gepflegt, Lager ist leer."}, "cot_begruendung": "Das Fehlen von C-Teilen aufgrund einer fehlerhaften Systempflege im ERP/Dispo-System ist ein softwareseitiges bzw. administratives Problem der internen Logistik. Kabelbinder sind temporär ersetzbar oder leicht nachzurüsten, weshalb der Ausbau meist nicht komplett steht (Info)."}, {"fall_id": "141", "text": "Erdungsband am Hochspannungsschrank WE1 nicht verschraubt, hängt lose herab. Werker hat es vergessen anzuschließen. Lebensgefahr beim Einschalten der Fahrleitungsspannung!", "zielvariablen": {"ursache": "Montage", "ursprung": "Werk", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Werker hat es vergessen anzuschließen. Lebensgefahr beim Einschalten"}, "cot_begruendung": "Das Vergessen des Erdungsbandes durch den Werker ist ein klassischer Montagefehler im eigenen Werk. Da eine lose Erdung an einem Hochspannungsschrank absolute Lebensgefahr bedeutet und die IBS verhindert, ist es ein kritischer Blocker."}, {"fall_id": "96", "text": "Kabel für Zugsicherungssystem PZB fehlen. Lieferant hat Lieferengpass für die Spezialstecker. Ohne PZB keine dynamische IBS möglich.", "zielvariablen": {"ursache": "Logistik", "ursprung": "Lieferant", "kritikalitaet": "Blocker", "serie": false, "text_snippet": "Lieferant hat Lieferengpass für die Spezialstecker. Ohne PZB keine dynamische IBS möglich."}, "cot_begruendung": "Ein Lieferengpass beim externen Zulieferer ist ein logistisches Problem (Lieferant). Da fehlende Zugsicherungskabel die fahrdynamische IBS unmöglich machen, liegt ein kritischer Blocker vor."}]</t>
         </is>
       </c>
     </row>
@@ -8001,7 +8001,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"grundursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"grundursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}, {"fall_id": "46", "text": "Großer Kratzer auf Trennglas im FGR. Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen.", "zielvariablen": {"grundursache": "Reinigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Reinigungskraft ist beim Bodenwischen mit dem Stiel des Mopps dagegengeschlagen"}, "cot_begruendung": "Die Beschädigung wurde direkt durch die Reinigungskraft beim Wischen verursacht (Reinigung/Werk). Ein zerkratztes Glas in der Trennwand muss getauscht werden (Nacharbeit), stoppt aber nicht die Produktion."}]</t>
+          <t>[{"fall_id": "7", "text": "Bei Testfahrt starkes Klappern im Deckenbereich über Nasszelle hörbar. Keine losen Teile auf den ersten Blick sichtbar. Bitte genauer prüfen.", "zielvariablen": {"ursache": "Unbekannt", "ursprung": "Unbekannt", "kritikalitaet": "Nacharbeit", "serie": false, "text_snippet": "Keine losen Teile auf den ersten Blick sichtbar."}, "cot_begruendung": "Die Informationsdichte reicht nicht aus, um eine Grundursache oder einen Ursprung abzuleiten, da nur das Symptom ('Klappern') beschrieben wird. Gemäß der Abstention-Regel verweigert das Modell hier die Ursachen-Klassifikation (Unbekannt), um Halluzinationen zu vermeiden. Eine Fehlersuche/Nacharbeit ist erforderlich."}, {"fall_id": "152", "text": "Abdeckbleche für die Heizkanäle LWS aus unserer eigenen Stanzerei sind an der Kante um 10 Grad zu wenig abgekantet. Betrifft alle 40 Bleche von heute. Können so nicht montiert werden, Kante steht ab.", "zielvariablen": {"ursache": "Fertigung", "ursprung": "Werk", "kritikalitaet": "Nacharbeit", "serie": true, "text_snippet": "aus unserer eigenen Stanzerei sind an der Kante um 10 Grad zu wenig abgekantet. Betrifft alle 40 Bleche"}, "cot_begruendung": "Ein Biegefehler aus der 'eigenen Stanzerei' ist ein interner Fertigungsfehler (Werk). Da 'alle 40 Bleche von heute' betroffen sind, liegt ein Serienfehler vor. Die Bleche müssen nachgebogen werden (Nacharbeit), stoppen aber nicht den kompletten Wagenausbau."}, {"fall_id": "97", "text": "Lacknase an der Bugmaske unten rechts. Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden.", "zielvariablen": {"ursache": "Verarbeitung", "ursprung": "Werk", "kritikalitaet": "Info", "serie": false, "text_snippet": "Zuviel Klarlack beim Lackieren im Werk aufgetragen. Muss auspoliert werden."}, "cot_begruendung": "Ein Fehler beim manuellen Lackauftrag im eigenen Werk ist ein Verarbeitungs- und Prozessfehler. Eine Lacknase ist ein reines Optikthema, das sich durch Auspolieren beheben lässt (Info/Nacharbeit)."}]</t>
         </is>
       </c>
     </row>

</xml_diff>